<commit_message>
suite des premiers modèles : 26-05-25
</commit_message>
<xml_diff>
--- a/Resultats_modeles_coleo_2024.xlsx
+++ b/Resultats_modeles_coleo_2024.xlsx
@@ -24,32 +24,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="68">
   <si>
     <t>ab.colsx</t>
   </si>
   <si>
-    <t>***</t>
-  </si>
-  <si>
-    <t>AC_UC</t>
-  </si>
-  <si>
-    <t>AC_LC</t>
-  </si>
-  <si>
-    <t>AC_BC</t>
-  </si>
-  <si>
-    <t>UC_LC</t>
-  </si>
-  <si>
-    <t>UC_BC</t>
-  </si>
-  <si>
-    <t>BC_LC</t>
-  </si>
-  <si>
     <t>toutes métriques fonistiques + toutes métriques d'habitats</t>
   </si>
   <si>
@@ -65,13 +44,376 @@
     <t>Y</t>
   </si>
   <si>
-    <t>P-value retenue</t>
-  </si>
-  <si>
-    <t>Résultat du modèle</t>
-  </si>
-  <si>
     <t>Ligne du code</t>
+  </si>
+  <si>
+    <t>1er modèle description</t>
+  </si>
+  <si>
+    <t>1er modèle P-value</t>
+  </si>
+  <si>
+    <t>2ème modèle description</t>
+  </si>
+  <si>
+    <t>2ème modèle P-value</t>
+  </si>
+  <si>
+    <t>ab.colsx ~ strate + (1 | LOCA / placette) + offset(log(prop.trap.season))</t>
+  </si>
+  <si>
+    <t>ab.colsx ~ 1 + (1 | LOCA / placette) + offset(log(prop.trap.season))</t>
+  </si>
+  <si>
+    <t>infra : 2.22e-16 ***</t>
+  </si>
+  <si>
+    <t>infra inf : 0.03114087 *</t>
+  </si>
+  <si>
+    <t>infra supp : 1.9902e-08 ***</t>
+  </si>
+  <si>
+    <t>supra : 0.00074195 ***</t>
+  </si>
+  <si>
+    <t>AICc 1er modèle</t>
+  </si>
+  <si>
+    <t>AICc 2ème modèle</t>
+  </si>
+  <si>
+    <t>2.22e-16 ***</t>
+  </si>
+  <si>
+    <t>3.7801e-06 ***</t>
+  </si>
+  <si>
+    <t>Dharma</t>
+  </si>
+  <si>
+    <t>Pas de soucis avec les présupposés du modèle</t>
+  </si>
+  <si>
+    <t>AC_UC (0,05 / 6 = 0,008)</t>
+  </si>
+  <si>
+    <t>&lt; 0.001 ***</t>
+  </si>
+  <si>
+    <t>0.0040433 **</t>
+  </si>
+  <si>
+    <t>0.0031270 **</t>
+  </si>
+  <si>
+    <t>N.S</t>
+  </si>
+  <si>
+    <t>Conclusion</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">On retrouve un effet de stratification verticale pour l'abondance cumulée totale des coléoptères saproxyliques, avec une différence d'abondance entre la strate </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>supra &amp; infra</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, ainsi qu'entre</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> infra.supp &amp; infra.inf, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">et </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>infra.supp &amp; infra</t>
+    </r>
+  </si>
+  <si>
+    <t>sr.colsx</t>
+  </si>
+  <si>
+    <t>Gaussian</t>
+  </si>
+  <si>
+    <t>sr.colsx ~ strate + (1 | LOCA / placette) + exp(pos+0|ID) + offset(log(prop.trap.season))</t>
+  </si>
+  <si>
+    <t>infra inf : 0.41284</t>
+  </si>
+  <si>
+    <t>infra supp : 3.4678e-05 ***</t>
+  </si>
+  <si>
+    <t>supra :0.17427</t>
+  </si>
+  <si>
+    <t>sr.colsx ~ 1 + (1 | LOCA / placette) + offset(log(prop.trap.season))</t>
+  </si>
+  <si>
+    <t>Modèle 1</t>
+  </si>
+  <si>
+    <t>Choix modèle mieux ajusté (delta &gt; 2)</t>
+  </si>
+  <si>
+    <t>0.0049384 **</t>
+  </si>
+  <si>
+    <t>0.0048236 **</t>
+  </si>
+  <si>
+    <t>N.S (0.0277350)</t>
+  </si>
+  <si>
+    <t>AC_LC (0,05 / 6 = 0,008)</t>
+  </si>
+  <si>
+    <t>AC_BC (0,05 / 6 = 0,008)</t>
+  </si>
+  <si>
+    <t>UC_LC (0,05 / 6 = 0,008)</t>
+  </si>
+  <si>
+    <t>UC_BC (0,05 / 6 = 0,008)</t>
+  </si>
+  <si>
+    <t>BC_LC (0,05 / 6 = 0,008)</t>
+  </si>
+  <si>
+    <t>ab.colsxrar</t>
+  </si>
+  <si>
+    <t>ab.colsxrar ~ strate + (1 | LOCA / placette) + offset(log(prop.trap.season))</t>
+  </si>
+  <si>
+    <t>infra : 0.00083824 ***</t>
+  </si>
+  <si>
+    <t xml:space="preserve">infra inf : 0.00123878 ** </t>
+  </si>
+  <si>
+    <t>infra supp : &lt; 2.22e-16 ***</t>
+  </si>
+  <si>
+    <t>supra : 0.00041702 ***</t>
+  </si>
+  <si>
+    <t>620.6581</t>
+  </si>
+  <si>
+    <t>620.6582</t>
+  </si>
+  <si>
+    <t>620.6583</t>
+  </si>
+  <si>
+    <t>620.6584</t>
+  </si>
+  <si>
+    <t>660.7834</t>
+  </si>
+  <si>
+    <t>660.7835</t>
+  </si>
+  <si>
+    <t>660.7836</t>
+  </si>
+  <si>
+    <t>660.7837</t>
+  </si>
+  <si>
+    <t>ab.colsxrar ~ 1 + (1 | LOCA / placette) + offset(log(prop.trap.season))</t>
+  </si>
+  <si>
+    <t>&lt; 2.22e-16 ***</t>
+  </si>
+  <si>
+    <t>3.2334e-10 ***</t>
+  </si>
+  <si>
+    <t>0.0068681 **</t>
+  </si>
+  <si>
+    <t>0.0023164 **</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">On retrouve un effet de stratification verticale pour La richesse spécifique cumulée totale des coléoptères saproxyliques, avec une différence de diversité spécifique entre la strate </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>infra.supp &amp; infra</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, et </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>infra.supp &amp; infra.inf</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">On retrouve un effet de stratification verticale pour l'abondance cumulée totale des coléoptères saproxyliques, avec une différence d'abondance entre la strate </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>infra &amp; infra.inf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>infra.supp &amp; infra</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>infra.supp &amp; infra.inf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, la strate </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">supra &amp; infra </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">ainsi que </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>supra et infra.supp</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -121,7 +463,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -130,6 +472,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -410,70 +767,773 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:U13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.6640625" style="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="33.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="6.77734375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="72.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.33203125" customWidth="1"/>
+    <col min="7" max="7" width="57.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="20.33203125" customWidth="1"/>
+    <col min="10" max="10" width="33.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="33.5546875" customWidth="1"/>
+    <col min="12" max="12" width="38.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.33203125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="21.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="24.109375" style="7" customWidth="1"/>
+    <col min="20" max="20" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="K1" s="1" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="M1" t="s">
-        <v>8</v>
+        <v>21</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="S1" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="T1" s="1"/>
+      <c r="U1" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:21" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
+      <c r="B2" s="3">
+        <v>321</v>
+      </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="D2" t="s">
-        <v>1</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2">
+        <v>955.84</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2">
+        <v>976.73</v>
+      </c>
+      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" t="s">
+        <v>37</v>
+      </c>
+      <c r="L2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O2" t="s">
+        <v>25</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="R2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S2" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3">
+        <v>321</v>
+      </c>
+      <c r="C3" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F3">
+        <v>955.84</v>
+      </c>
+      <c r="G3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H3" s="5"/>
+      <c r="I3">
+        <v>976.73</v>
+      </c>
+      <c r="J3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" t="s">
+        <v>37</v>
+      </c>
+      <c r="L3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" t="s">
+        <v>27</v>
+      </c>
+      <c r="N3" t="s">
+        <v>27</v>
+      </c>
+      <c r="O3" t="s">
+        <v>25</v>
+      </c>
+      <c r="P3" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>24</v>
+      </c>
+      <c r="R3" t="s">
+        <v>27</v>
+      </c>
+      <c r="S3" s="8"/>
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="3">
+        <v>321</v>
+      </c>
+      <c r="C4" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4">
+        <v>955.84</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="5"/>
+      <c r="I4">
+        <v>976.73</v>
+      </c>
+      <c r="J4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" t="s">
+        <v>37</v>
+      </c>
+      <c r="L4" t="s">
+        <v>22</v>
+      </c>
+      <c r="M4" t="s">
+        <v>27</v>
+      </c>
+      <c r="N4" t="s">
+        <v>27</v>
+      </c>
+      <c r="O4" t="s">
+        <v>25</v>
+      </c>
+      <c r="P4" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>24</v>
+      </c>
+      <c r="R4" t="s">
+        <v>27</v>
+      </c>
+      <c r="S4" s="8"/>
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="3">
+        <v>321</v>
+      </c>
+      <c r="C5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5">
+        <v>955.84</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="5"/>
+      <c r="I5">
+        <v>976.73</v>
+      </c>
+      <c r="J5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" t="s">
+        <v>37</v>
+      </c>
+      <c r="L5" t="s">
+        <v>22</v>
+      </c>
+      <c r="M5" t="s">
+        <v>27</v>
+      </c>
+      <c r="N5" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" t="s">
+        <v>25</v>
+      </c>
+      <c r="P5" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>24</v>
+      </c>
+      <c r="R5" t="s">
+        <v>27</v>
+      </c>
+      <c r="S5" s="8"/>
+    </row>
+    <row r="6" spans="1:21" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="3">
+        <v>393</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6">
+        <v>641.5</v>
+      </c>
+      <c r="G6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I6">
+        <v>646.24</v>
+      </c>
+      <c r="J6" t="s">
+        <v>39</v>
+      </c>
+      <c r="K6" t="s">
+        <v>37</v>
+      </c>
+      <c r="L6" t="s">
+        <v>22</v>
+      </c>
+      <c r="M6" t="s">
+        <v>27</v>
+      </c>
+      <c r="N6" t="s">
+        <v>27</v>
+      </c>
+      <c r="O6" t="s">
+        <v>41</v>
+      </c>
+      <c r="P6" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>24</v>
+      </c>
+      <c r="R6" t="s">
+        <v>27</v>
+      </c>
+      <c r="S6" s="8" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="3">
+        <v>393</v>
+      </c>
+      <c r="C7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7">
+        <v>641.5</v>
+      </c>
+      <c r="G7" t="s">
+        <v>36</v>
+      </c>
+      <c r="H7" s="5"/>
+      <c r="I7">
+        <v>646.24</v>
+      </c>
+      <c r="J7" t="s">
+        <v>39</v>
+      </c>
+      <c r="K7" t="s">
+        <v>37</v>
+      </c>
+      <c r="L7" t="s">
+        <v>22</v>
+      </c>
+      <c r="M7" t="s">
+        <v>27</v>
+      </c>
+      <c r="N7" t="s">
+        <v>27</v>
+      </c>
+      <c r="O7" t="s">
+        <v>41</v>
+      </c>
+      <c r="P7" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>24</v>
+      </c>
+      <c r="R7" t="s">
+        <v>27</v>
+      </c>
+      <c r="S7" s="8"/>
+    </row>
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="3">
+        <v>393</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8">
+        <v>641.5</v>
+      </c>
+      <c r="G8" t="s">
+        <v>36</v>
+      </c>
+      <c r="H8" s="5"/>
+      <c r="I8">
+        <v>646.24</v>
+      </c>
+      <c r="J8" t="s">
+        <v>39</v>
+      </c>
+      <c r="K8" t="s">
+        <v>37</v>
+      </c>
+      <c r="L8" t="s">
+        <v>22</v>
+      </c>
+      <c r="M8" t="s">
+        <v>27</v>
+      </c>
+      <c r="N8" t="s">
+        <v>27</v>
+      </c>
+      <c r="O8" t="s">
+        <v>41</v>
+      </c>
+      <c r="P8" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>24</v>
+      </c>
+      <c r="R8" t="s">
+        <v>27</v>
+      </c>
+      <c r="S8" s="8"/>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="3">
+        <v>393</v>
+      </c>
+      <c r="C9" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" t="s">
+        <v>32</v>
+      </c>
+      <c r="E9" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9">
+        <v>641.5</v>
+      </c>
+      <c r="G9" t="s">
+        <v>36</v>
+      </c>
+      <c r="H9" s="5"/>
+      <c r="I9">
+        <v>646.24</v>
+      </c>
+      <c r="J9" t="s">
+        <v>39</v>
+      </c>
+      <c r="K9" t="s">
+        <v>37</v>
+      </c>
+      <c r="L9" t="s">
+        <v>22</v>
+      </c>
+      <c r="M9" t="s">
+        <v>27</v>
+      </c>
+      <c r="N9" t="s">
+        <v>27</v>
+      </c>
+      <c r="O9" t="s">
+        <v>41</v>
+      </c>
+      <c r="P9" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>24</v>
+      </c>
+      <c r="R9" t="s">
+        <v>27</v>
+      </c>
+      <c r="S9" s="8"/>
+    </row>
+    <row r="10" spans="1:21" ht="120" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>47</v>
+      </c>
+      <c r="B10" s="3">
+        <v>455</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" t="s">
+        <v>49</v>
+      </c>
+      <c r="F10" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" t="s">
+        <v>61</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="I10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J10" t="s">
+        <v>63</v>
+      </c>
+      <c r="K10" t="s">
+        <v>37</v>
+      </c>
+      <c r="L10" t="s">
+        <v>22</v>
+      </c>
+      <c r="M10" t="s">
+        <v>24</v>
+      </c>
+      <c r="N10" t="s">
+        <v>27</v>
+      </c>
+      <c r="O10" t="s">
+        <v>65</v>
+      </c>
+      <c r="P10" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>24</v>
+      </c>
+      <c r="R10" t="s">
+        <v>64</v>
+      </c>
+      <c r="S10" s="8" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="3">
+        <v>455</v>
+      </c>
+      <c r="C11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" t="s">
+        <v>50</v>
+      </c>
+      <c r="F11" t="s">
+        <v>54</v>
+      </c>
+      <c r="G11" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" s="5"/>
+      <c r="I11" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11" t="s">
+        <v>63</v>
+      </c>
+      <c r="K11" t="s">
+        <v>37</v>
+      </c>
+      <c r="L11" t="s">
+        <v>22</v>
+      </c>
+      <c r="M11" t="s">
+        <v>24</v>
+      </c>
+      <c r="N11" t="s">
+        <v>27</v>
+      </c>
+      <c r="O11" t="s">
+        <v>65</v>
+      </c>
+      <c r="P11" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>24</v>
+      </c>
+      <c r="R11" t="s">
+        <v>64</v>
+      </c>
+      <c r="S11" s="8"/>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="3">
+        <v>455</v>
+      </c>
+      <c r="C12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" t="s">
+        <v>48</v>
+      </c>
+      <c r="E12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" t="s">
+        <v>61</v>
+      </c>
+      <c r="H12" s="5"/>
+      <c r="I12" t="s">
+        <v>59</v>
+      </c>
+      <c r="J12" t="s">
+        <v>63</v>
+      </c>
+      <c r="K12" t="s">
+        <v>37</v>
+      </c>
+      <c r="L12" t="s">
+        <v>22</v>
+      </c>
+      <c r="M12" t="s">
+        <v>24</v>
+      </c>
+      <c r="N12" t="s">
+        <v>27</v>
+      </c>
+      <c r="O12" t="s">
+        <v>65</v>
+      </c>
+      <c r="P12" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>24</v>
+      </c>
+      <c r="R12" t="s">
+        <v>64</v>
+      </c>
+      <c r="S12" s="8"/>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>47</v>
+      </c>
+      <c r="B13" s="3">
+        <v>455</v>
+      </c>
+      <c r="C13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" t="s">
+        <v>48</v>
+      </c>
+      <c r="E13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F13" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" t="s">
+        <v>61</v>
+      </c>
+      <c r="H13" s="5"/>
+      <c r="I13" t="s">
+        <v>60</v>
+      </c>
+      <c r="J13" t="s">
+        <v>63</v>
+      </c>
+      <c r="K13" t="s">
+        <v>37</v>
+      </c>
+      <c r="L13" t="s">
+        <v>22</v>
+      </c>
+      <c r="M13" t="s">
+        <v>24</v>
+      </c>
+      <c r="N13" t="s">
+        <v>27</v>
+      </c>
+      <c r="O13" t="s">
+        <v>65</v>
+      </c>
+      <c r="P13" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>24</v>
+      </c>
+      <c r="R13" t="s">
+        <v>64</v>
+      </c>
+      <c r="S13" s="8"/>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="S2:S5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="S6:S9"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="S10:S13"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
02/06/25 : dernier modèle résolue reste pos
</commit_message>
<xml_diff>
--- a/Resultats_modeles_coleo_2024.xlsx
+++ b/Resultats_modeles_coleo_2024.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2464" uniqueCount="501">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2527" uniqueCount="514">
   <si>
     <t>ab.colsx</t>
   </si>
@@ -2939,6 +2939,121 @@
       </rPr>
       <t>intra.supp &amp; infra</t>
     </r>
+  </si>
+  <si>
+    <t>t_family (Student)</t>
+  </si>
+  <si>
+    <t>CWM_canop ~ strate + (1 | LOCA / placette) + offset(log(prop.trap.season))</t>
+  </si>
+  <si>
+    <t>CWM_canop ~ 1 + (1 | LOCA / placette) + offset(log(prop.trap.season))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">infra : &lt; 2e-16 *** </t>
+  </si>
+  <si>
+    <t>infra inf : 0.535</t>
+  </si>
+  <si>
+    <t>infra supp : 4.40e-06 ***</t>
+  </si>
+  <si>
+    <t>supra : 3.09e-06 ***</t>
+  </si>
+  <si>
+    <t>-57.22125</t>
+  </si>
+  <si>
+    <t>-32.60404</t>
+  </si>
+  <si>
+    <t>5.671e-07 ***</t>
+  </si>
+  <si>
+    <t>Pas de soucis avec les présupposés du modèle, difficulté à trouver la bonne loi</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Pour la comparaison des strates 2 à 2 en ce qui concerne le Trait moyen de préférence de canopée (= héliophilie moyenne) de l’assemblage d’espèces, des différences sont observées entre </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>supra &amp; intra.inf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>supra &amp; infra</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>intra.supp &amp; intra.inf</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, et</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> intra.supp &amp; infra</t>
+    </r>
+  </si>
+  <si>
+    <t>Test de plusieurs packages pour pallier au manque de distributions dans glmmTMB qui ne fit pas avec Dharma : lme4 (glmer, glmer.nb), gamlss. Finalement les autres packages ne fonctionnent pas, distribution qui fit trouvée dans glmmTMB : t_family</t>
   </si>
 </sst>
 </file>
@@ -3006,6 +3121,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3014,9 +3132,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3408,7 +3523,7 @@
       <c r="G2" t="s">
         <v>12</v>
       </c>
-      <c r="H2" s="7" t="s">
+      <c r="H2" s="8" t="s">
         <v>19</v>
       </c>
       <c r="I2">
@@ -3441,7 +3556,7 @@
       <c r="R2" t="s">
         <v>27</v>
       </c>
-      <c r="S2" s="8" t="s">
+      <c r="S2" s="9" t="s">
         <v>83</v>
       </c>
     </row>
@@ -3467,7 +3582,7 @@
       <c r="G3" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="7"/>
+      <c r="H3" s="8"/>
       <c r="I3">
         <v>976.73</v>
       </c>
@@ -3498,7 +3613,7 @@
       <c r="R3" t="s">
         <v>27</v>
       </c>
-      <c r="S3" s="8"/>
+      <c r="S3" s="9"/>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -3522,7 +3637,7 @@
       <c r="G4" t="s">
         <v>12</v>
       </c>
-      <c r="H4" s="7"/>
+      <c r="H4" s="8"/>
       <c r="I4">
         <v>976.73</v>
       </c>
@@ -3553,7 +3668,7 @@
       <c r="R4" t="s">
         <v>27</v>
       </c>
-      <c r="S4" s="8"/>
+      <c r="S4" s="9"/>
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -3577,7 +3692,7 @@
       <c r="G5" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="7"/>
+      <c r="H5" s="8"/>
       <c r="I5">
         <v>976.73</v>
       </c>
@@ -3608,7 +3723,7 @@
       <c r="R5" t="s">
         <v>27</v>
       </c>
-      <c r="S5" s="8"/>
+      <c r="S5" s="9"/>
     </row>
     <row r="6" spans="1:21" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -3632,7 +3747,7 @@
       <c r="G6" t="s">
         <v>35</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="8" t="s">
         <v>19</v>
       </c>
       <c r="I6">
@@ -3665,7 +3780,7 @@
       <c r="R6" t="s">
         <v>27</v>
       </c>
-      <c r="S6" s="8" t="s">
+      <c r="S6" s="9" t="s">
         <v>84</v>
       </c>
     </row>
@@ -3691,7 +3806,7 @@
       <c r="G7" t="s">
         <v>35</v>
       </c>
-      <c r="H7" s="7"/>
+      <c r="H7" s="8"/>
       <c r="I7">
         <v>646.24</v>
       </c>
@@ -3722,7 +3837,7 @@
       <c r="R7" t="s">
         <v>27</v>
       </c>
-      <c r="S7" s="8"/>
+      <c r="S7" s="9"/>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -3746,7 +3861,7 @@
       <c r="G8" t="s">
         <v>35</v>
       </c>
-      <c r="H8" s="7"/>
+      <c r="H8" s="8"/>
       <c r="I8">
         <v>646.24</v>
       </c>
@@ -3777,7 +3892,7 @@
       <c r="R8" t="s">
         <v>27</v>
       </c>
-      <c r="S8" s="8"/>
+      <c r="S8" s="9"/>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -3801,7 +3916,7 @@
       <c r="G9" t="s">
         <v>35</v>
       </c>
-      <c r="H9" s="7"/>
+      <c r="H9" s="8"/>
       <c r="I9">
         <v>646.24</v>
       </c>
@@ -3832,7 +3947,7 @@
       <c r="R9" t="s">
         <v>27</v>
       </c>
-      <c r="S9" s="8"/>
+      <c r="S9" s="9"/>
     </row>
     <row r="10" spans="1:21" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -3856,7 +3971,7 @@
       <c r="G10" t="s">
         <v>54</v>
       </c>
-      <c r="H10" s="7" t="s">
+      <c r="H10" s="8" t="s">
         <v>55</v>
       </c>
       <c r="I10" t="s">
@@ -3889,7 +4004,7 @@
       <c r="R10" t="s">
         <v>57</v>
       </c>
-      <c r="S10" s="8" t="s">
+      <c r="S10" s="9" t="s">
         <v>85</v>
       </c>
     </row>
@@ -3915,7 +4030,7 @@
       <c r="G11" t="s">
         <v>54</v>
       </c>
-      <c r="H11" s="7"/>
+      <c r="H11" s="8"/>
       <c r="I11" t="s">
         <v>53</v>
       </c>
@@ -3946,7 +4061,7 @@
       <c r="R11" t="s">
         <v>57</v>
       </c>
-      <c r="S11" s="8"/>
+      <c r="S11" s="9"/>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -3970,7 +4085,7 @@
       <c r="G12" t="s">
         <v>54</v>
       </c>
-      <c r="H12" s="7"/>
+      <c r="H12" s="8"/>
       <c r="I12" t="s">
         <v>53</v>
       </c>
@@ -4001,7 +4116,7 @@
       <c r="R12" t="s">
         <v>57</v>
       </c>
-      <c r="S12" s="8"/>
+      <c r="S12" s="9"/>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -4025,7 +4140,7 @@
       <c r="G13" t="s">
         <v>54</v>
       </c>
-      <c r="H13" s="7"/>
+      <c r="H13" s="8"/>
       <c r="I13" t="s">
         <v>53</v>
       </c>
@@ -4056,7 +4171,7 @@
       <c r="R13" t="s">
         <v>57</v>
       </c>
-      <c r="S13" s="8"/>
+      <c r="S13" s="9"/>
     </row>
     <row r="14" spans="1:21" ht="131.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -4080,7 +4195,7 @@
       <c r="G14" t="s">
         <v>70</v>
       </c>
-      <c r="H14" s="7" t="s">
+      <c r="H14" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I14" t="s">
@@ -4092,7 +4207,7 @@
       <c r="K14" t="s">
         <v>36</v>
       </c>
-      <c r="L14" s="9" t="s">
+      <c r="L14" s="10" t="s">
         <v>80</v>
       </c>
       <c r="M14" t="s">
@@ -4113,7 +4228,7 @@
       <c r="R14" t="s">
         <v>24</v>
       </c>
-      <c r="S14" s="8" t="s">
+      <c r="S14" s="9" t="s">
         <v>86</v>
       </c>
     </row>
@@ -4139,7 +4254,7 @@
       <c r="G15" t="s">
         <v>70</v>
       </c>
-      <c r="H15" s="7"/>
+      <c r="H15" s="8"/>
       <c r="I15" t="s">
         <v>76</v>
       </c>
@@ -4149,7 +4264,7 @@
       <c r="K15" t="s">
         <v>36</v>
       </c>
-      <c r="L15" s="9"/>
+      <c r="L15" s="10"/>
       <c r="M15" t="s">
         <v>24</v>
       </c>
@@ -4168,7 +4283,7 @@
       <c r="R15" t="s">
         <v>24</v>
       </c>
-      <c r="S15" s="8"/>
+      <c r="S15" s="9"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -4192,7 +4307,7 @@
       <c r="G16" t="s">
         <v>70</v>
       </c>
-      <c r="H16" s="7"/>
+      <c r="H16" s="8"/>
       <c r="I16" t="s">
         <v>76</v>
       </c>
@@ -4202,7 +4317,7 @@
       <c r="K16" t="s">
         <v>36</v>
       </c>
-      <c r="L16" s="9"/>
+      <c r="L16" s="10"/>
       <c r="M16" t="s">
         <v>24</v>
       </c>
@@ -4221,7 +4336,7 @@
       <c r="R16" t="s">
         <v>24</v>
       </c>
-      <c r="S16" s="8"/>
+      <c r="S16" s="9"/>
     </row>
     <row r="17" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
@@ -4245,7 +4360,7 @@
       <c r="G17" t="s">
         <v>70</v>
       </c>
-      <c r="H17" s="7"/>
+      <c r="H17" s="8"/>
       <c r="I17" t="s">
         <v>76</v>
       </c>
@@ -4255,7 +4370,7 @@
       <c r="K17" t="s">
         <v>36</v>
       </c>
-      <c r="L17" s="9"/>
+      <c r="L17" s="10"/>
       <c r="M17" t="s">
         <v>24</v>
       </c>
@@ -4274,7 +4389,7 @@
       <c r="R17" t="s">
         <v>24</v>
       </c>
-      <c r="S17" s="8"/>
+      <c r="S17" s="9"/>
     </row>
     <row r="18" spans="1:19" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
@@ -4298,7 +4413,7 @@
       <c r="G18" t="s">
         <v>89</v>
       </c>
-      <c r="H18" s="7" t="s">
+      <c r="H18" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I18" t="s">
@@ -4331,7 +4446,7 @@
       <c r="R18" t="s">
         <v>27</v>
       </c>
-      <c r="S18" s="8" t="s">
+      <c r="S18" s="9" t="s">
         <v>109</v>
       </c>
     </row>
@@ -4357,7 +4472,7 @@
       <c r="G19" t="s">
         <v>89</v>
       </c>
-      <c r="H19" s="7"/>
+      <c r="H19" s="8"/>
       <c r="I19" t="s">
         <v>94</v>
       </c>
@@ -4388,7 +4503,7 @@
       <c r="R19" t="s">
         <v>27</v>
       </c>
-      <c r="S19" s="8"/>
+      <c r="S19" s="9"/>
     </row>
     <row r="20" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
@@ -4412,7 +4527,7 @@
       <c r="G20" t="s">
         <v>89</v>
       </c>
-      <c r="H20" s="7"/>
+      <c r="H20" s="8"/>
       <c r="I20" t="s">
         <v>94</v>
       </c>
@@ -4443,7 +4558,7 @@
       <c r="R20" t="s">
         <v>27</v>
       </c>
-      <c r="S20" s="8"/>
+      <c r="S20" s="9"/>
     </row>
     <row r="21" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
@@ -4467,7 +4582,7 @@
       <c r="G21" t="s">
         <v>89</v>
       </c>
-      <c r="H21" s="7"/>
+      <c r="H21" s="8"/>
       <c r="I21" t="s">
         <v>94</v>
       </c>
@@ -4498,7 +4613,7 @@
       <c r="R21" t="s">
         <v>27</v>
       </c>
-      <c r="S21" s="8"/>
+      <c r="S21" s="9"/>
     </row>
     <row r="22" spans="1:19" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
@@ -4522,7 +4637,7 @@
       <c r="G22" t="s">
         <v>100</v>
       </c>
-      <c r="H22" s="7" t="s">
+      <c r="H22" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I22" t="s">
@@ -4555,7 +4670,7 @@
       <c r="R22" t="s">
         <v>27</v>
       </c>
-      <c r="S22" s="8" t="s">
+      <c r="S22" s="9" t="s">
         <v>110</v>
       </c>
     </row>
@@ -4581,7 +4696,7 @@
       <c r="G23" t="s">
         <v>100</v>
       </c>
-      <c r="H23" s="7"/>
+      <c r="H23" s="8"/>
       <c r="I23" t="s">
         <v>105</v>
       </c>
@@ -4612,7 +4727,7 @@
       <c r="R23" t="s">
         <v>27</v>
       </c>
-      <c r="S23" s="8"/>
+      <c r="S23" s="9"/>
     </row>
     <row r="24" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
@@ -4636,7 +4751,7 @@
       <c r="G24" t="s">
         <v>100</v>
       </c>
-      <c r="H24" s="7"/>
+      <c r="H24" s="8"/>
       <c r="I24" t="s">
         <v>105</v>
       </c>
@@ -4667,7 +4782,7 @@
       <c r="R24" t="s">
         <v>27</v>
       </c>
-      <c r="S24" s="8"/>
+      <c r="S24" s="9"/>
     </row>
     <row r="25" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
@@ -4691,7 +4806,7 @@
       <c r="G25" t="s">
         <v>100</v>
       </c>
-      <c r="H25" s="7"/>
+      <c r="H25" s="8"/>
       <c r="I25" t="s">
         <v>105</v>
       </c>
@@ -4722,7 +4837,7 @@
       <c r="R25" t="s">
         <v>27</v>
       </c>
-      <c r="S25" s="8"/>
+      <c r="S25" s="9"/>
     </row>
     <row r="26" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
@@ -4746,7 +4861,7 @@
       <c r="G26" t="s">
         <v>113</v>
       </c>
-      <c r="H26" s="7" t="s">
+      <c r="H26" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I26" t="s">
@@ -4779,7 +4894,7 @@
       <c r="R26" t="s">
         <v>27</v>
       </c>
-      <c r="S26" s="8" t="s">
+      <c r="S26" s="9" t="s">
         <v>122</v>
       </c>
     </row>
@@ -4805,7 +4920,7 @@
       <c r="G27" t="s">
         <v>113</v>
       </c>
-      <c r="H27" s="7"/>
+      <c r="H27" s="8"/>
       <c r="I27" t="s">
         <v>118</v>
       </c>
@@ -4836,7 +4951,7 @@
       <c r="R27" t="s">
         <v>27</v>
       </c>
-      <c r="S27" s="8"/>
+      <c r="S27" s="9"/>
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
@@ -4860,7 +4975,7 @@
       <c r="G28" t="s">
         <v>113</v>
       </c>
-      <c r="H28" s="7"/>
+      <c r="H28" s="8"/>
       <c r="I28" t="s">
         <v>118</v>
       </c>
@@ -4891,7 +5006,7 @@
       <c r="R28" t="s">
         <v>27</v>
       </c>
-      <c r="S28" s="8"/>
+      <c r="S28" s="9"/>
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
@@ -4915,7 +5030,7 @@
       <c r="G29" t="s">
         <v>113</v>
       </c>
-      <c r="H29" s="7"/>
+      <c r="H29" s="8"/>
       <c r="I29" t="s">
         <v>118</v>
       </c>
@@ -4946,7 +5061,7 @@
       <c r="R29" t="s">
         <v>27</v>
       </c>
-      <c r="S29" s="8"/>
+      <c r="S29" s="9"/>
     </row>
     <row r="30" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
@@ -4970,7 +5085,7 @@
       <c r="G30" t="s">
         <v>125</v>
       </c>
-      <c r="H30" s="7" t="s">
+      <c r="H30" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I30" t="s">
@@ -5003,7 +5118,7 @@
       <c r="R30" t="s">
         <v>134</v>
       </c>
-      <c r="S30" s="8" t="s">
+      <c r="S30" s="9" t="s">
         <v>135</v>
       </c>
     </row>
@@ -5029,7 +5144,7 @@
       <c r="G31" t="s">
         <v>125</v>
       </c>
-      <c r="H31" s="7"/>
+      <c r="H31" s="8"/>
       <c r="I31" t="s">
         <v>130</v>
       </c>
@@ -5060,7 +5175,7 @@
       <c r="R31" t="s">
         <v>134</v>
       </c>
-      <c r="S31" s="8"/>
+      <c r="S31" s="9"/>
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
@@ -5084,7 +5199,7 @@
       <c r="G32" t="s">
         <v>125</v>
       </c>
-      <c r="H32" s="7"/>
+      <c r="H32" s="8"/>
       <c r="I32" t="s">
         <v>130</v>
       </c>
@@ -5115,7 +5230,7 @@
       <c r="R32" t="s">
         <v>134</v>
       </c>
-      <c r="S32" s="8"/>
+      <c r="S32" s="9"/>
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
@@ -5139,7 +5254,7 @@
       <c r="G33" t="s">
         <v>125</v>
       </c>
-      <c r="H33" s="7"/>
+      <c r="H33" s="8"/>
       <c r="I33" t="s">
         <v>130</v>
       </c>
@@ -5170,7 +5285,7 @@
       <c r="R33" t="s">
         <v>134</v>
       </c>
-      <c r="S33" s="8"/>
+      <c r="S33" s="9"/>
     </row>
     <row r="34" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
@@ -5194,7 +5309,7 @@
       <c r="G34" t="s">
         <v>138</v>
       </c>
-      <c r="H34" s="7" t="s">
+      <c r="H34" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I34" t="s">
@@ -5227,7 +5342,7 @@
       <c r="R34" t="s">
         <v>146</v>
       </c>
-      <c r="S34" s="8" t="s">
+      <c r="S34" s="9" t="s">
         <v>147</v>
       </c>
     </row>
@@ -5253,7 +5368,7 @@
       <c r="G35" t="s">
         <v>138</v>
       </c>
-      <c r="H35" s="7"/>
+      <c r="H35" s="8"/>
       <c r="I35" t="s">
         <v>143</v>
       </c>
@@ -5284,7 +5399,7 @@
       <c r="R35" t="s">
         <v>146</v>
       </c>
-      <c r="S35" s="8"/>
+      <c r="S35" s="9"/>
     </row>
     <row r="36" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
@@ -5308,7 +5423,7 @@
       <c r="G36" t="s">
         <v>138</v>
       </c>
-      <c r="H36" s="7"/>
+      <c r="H36" s="8"/>
       <c r="I36" t="s">
         <v>143</v>
       </c>
@@ -5339,7 +5454,7 @@
       <c r="R36" t="s">
         <v>146</v>
       </c>
-      <c r="S36" s="8"/>
+      <c r="S36" s="9"/>
     </row>
     <row r="37" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
@@ -5363,7 +5478,7 @@
       <c r="G37" t="s">
         <v>138</v>
       </c>
-      <c r="H37" s="7"/>
+      <c r="H37" s="8"/>
       <c r="I37" t="s">
         <v>143</v>
       </c>
@@ -5394,7 +5509,7 @@
       <c r="R37" t="s">
         <v>146</v>
       </c>
-      <c r="S37" s="8"/>
+      <c r="S37" s="9"/>
     </row>
     <row r="38" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
@@ -5418,7 +5533,7 @@
       <c r="G38" t="s">
         <v>153</v>
       </c>
-      <c r="H38" s="7" t="s">
+      <c r="H38" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I38" t="s">
@@ -5451,7 +5566,7 @@
       <c r="R38" t="s">
         <v>27</v>
       </c>
-      <c r="S38" s="8" t="s">
+      <c r="S38" s="9" t="s">
         <v>158</v>
       </c>
     </row>
@@ -5477,7 +5592,7 @@
       <c r="G39" t="s">
         <v>153</v>
       </c>
-      <c r="H39" s="7"/>
+      <c r="H39" s="8"/>
       <c r="I39" t="s">
         <v>149</v>
       </c>
@@ -5508,7 +5623,7 @@
       <c r="R39" t="s">
         <v>27</v>
       </c>
-      <c r="S39" s="8"/>
+      <c r="S39" s="9"/>
     </row>
     <row r="40" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
@@ -5532,7 +5647,7 @@
       <c r="G40" t="s">
         <v>153</v>
       </c>
-      <c r="H40" s="7"/>
+      <c r="H40" s="8"/>
       <c r="I40" t="s">
         <v>149</v>
       </c>
@@ -5563,7 +5678,7 @@
       <c r="R40" t="s">
         <v>27</v>
       </c>
-      <c r="S40" s="8"/>
+      <c r="S40" s="9"/>
     </row>
     <row r="41" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
@@ -5587,7 +5702,7 @@
       <c r="G41" t="s">
         <v>153</v>
       </c>
-      <c r="H41" s="7"/>
+      <c r="H41" s="8"/>
       <c r="I41" t="s">
         <v>149</v>
       </c>
@@ -5618,7 +5733,7 @@
       <c r="R41" t="s">
         <v>27</v>
       </c>
-      <c r="S41" s="8"/>
+      <c r="S41" s="9"/>
     </row>
     <row r="42" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
@@ -5642,7 +5757,7 @@
       <c r="G42" t="s">
         <v>162</v>
       </c>
-      <c r="H42" s="7" t="s">
+      <c r="H42" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I42" t="s">
@@ -5675,7 +5790,7 @@
       <c r="R42" t="s">
         <v>27</v>
       </c>
-      <c r="S42" s="8" t="s">
+      <c r="S42" s="9" t="s">
         <v>172</v>
       </c>
     </row>
@@ -5701,7 +5816,7 @@
       <c r="G43" t="s">
         <v>162</v>
       </c>
-      <c r="H43" s="7"/>
+      <c r="H43" s="8"/>
       <c r="I43" t="s">
         <v>167</v>
       </c>
@@ -5732,7 +5847,7 @@
       <c r="R43" t="s">
         <v>27</v>
       </c>
-      <c r="S43" s="8"/>
+      <c r="S43" s="9"/>
     </row>
     <row r="44" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
@@ -5756,7 +5871,7 @@
       <c r="G44" t="s">
         <v>162</v>
       </c>
-      <c r="H44" s="7"/>
+      <c r="H44" s="8"/>
       <c r="I44" t="s">
         <v>167</v>
       </c>
@@ -5787,7 +5902,7 @@
       <c r="R44" t="s">
         <v>27</v>
       </c>
-      <c r="S44" s="8"/>
+      <c r="S44" s="9"/>
     </row>
     <row r="45" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
@@ -5811,7 +5926,7 @@
       <c r="G45" t="s">
         <v>162</v>
       </c>
-      <c r="H45" s="7"/>
+      <c r="H45" s="8"/>
       <c r="I45" t="s">
         <v>167</v>
       </c>
@@ -5842,7 +5957,7 @@
       <c r="R45" t="s">
         <v>27</v>
       </c>
-      <c r="S45" s="8"/>
+      <c r="S45" s="9"/>
     </row>
     <row r="46" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
@@ -5866,7 +5981,7 @@
       <c r="G46" t="s">
         <v>177</v>
       </c>
-      <c r="H46" s="7" t="s">
+      <c r="H46" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I46" t="s">
@@ -5899,7 +6014,7 @@
       <c r="R46" t="s">
         <v>27</v>
       </c>
-      <c r="S46" s="8" t="s">
+      <c r="S46" s="9" t="s">
         <v>186</v>
       </c>
     </row>
@@ -5925,7 +6040,7 @@
       <c r="G47" t="s">
         <v>177</v>
       </c>
-      <c r="H47" s="7"/>
+      <c r="H47" s="8"/>
       <c r="I47" t="s">
         <v>178</v>
       </c>
@@ -5956,7 +6071,7 @@
       <c r="R47" t="s">
         <v>27</v>
       </c>
-      <c r="S47" s="8"/>
+      <c r="S47" s="9"/>
     </row>
     <row r="48" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
@@ -5980,7 +6095,7 @@
       <c r="G48" t="s">
         <v>177</v>
       </c>
-      <c r="H48" s="7"/>
+      <c r="H48" s="8"/>
       <c r="I48" t="s">
         <v>178</v>
       </c>
@@ -6011,7 +6126,7 @@
       <c r="R48" t="s">
         <v>27</v>
       </c>
-      <c r="S48" s="8"/>
+      <c r="S48" s="9"/>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
@@ -6035,7 +6150,7 @@
       <c r="G49" t="s">
         <v>177</v>
       </c>
-      <c r="H49" s="7"/>
+      <c r="H49" s="8"/>
       <c r="I49" t="s">
         <v>178</v>
       </c>
@@ -6066,7 +6181,7 @@
       <c r="R49" t="s">
         <v>27</v>
       </c>
-      <c r="S49" s="8"/>
+      <c r="S49" s="9"/>
     </row>
     <row r="50" spans="1:19" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
@@ -6090,7 +6205,7 @@
       <c r="G50" t="s">
         <v>189</v>
       </c>
-      <c r="H50" s="7" t="s">
+      <c r="H50" s="8" t="s">
         <v>197</v>
       </c>
       <c r="I50" t="s">
@@ -6123,7 +6238,7 @@
       <c r="R50" t="s">
         <v>198</v>
       </c>
-      <c r="S50" s="8" t="s">
+      <c r="S50" s="9" t="s">
         <v>201</v>
       </c>
     </row>
@@ -6149,7 +6264,7 @@
       <c r="G51" t="s">
         <v>189</v>
       </c>
-      <c r="H51" s="7"/>
+      <c r="H51" s="8"/>
       <c r="I51" t="s">
         <v>191</v>
       </c>
@@ -6180,7 +6295,7 @@
       <c r="R51" t="s">
         <v>198</v>
       </c>
-      <c r="S51" s="8"/>
+      <c r="S51" s="9"/>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
@@ -6204,7 +6319,7 @@
       <c r="G52" t="s">
         <v>189</v>
       </c>
-      <c r="H52" s="7"/>
+      <c r="H52" s="8"/>
       <c r="I52" t="s">
         <v>191</v>
       </c>
@@ -6235,7 +6350,7 @@
       <c r="R52" t="s">
         <v>198</v>
       </c>
-      <c r="S52" s="8"/>
+      <c r="S52" s="9"/>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
@@ -6259,7 +6374,7 @@
       <c r="G53" t="s">
         <v>189</v>
       </c>
-      <c r="H53" s="7"/>
+      <c r="H53" s="8"/>
       <c r="I53" t="s">
         <v>191</v>
       </c>
@@ -6290,7 +6405,7 @@
       <c r="R53" t="s">
         <v>198</v>
       </c>
-      <c r="S53" s="8"/>
+      <c r="S53" s="9"/>
     </row>
     <row r="54" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
@@ -6314,7 +6429,7 @@
       <c r="G54" t="s">
         <v>204</v>
       </c>
-      <c r="H54" s="7" t="s">
+      <c r="H54" s="8" t="s">
         <v>211</v>
       </c>
       <c r="I54" t="s">
@@ -6347,7 +6462,7 @@
       <c r="R54" t="s">
         <v>27</v>
       </c>
-      <c r="S54" s="8" t="s">
+      <c r="S54" s="9" t="s">
         <v>213</v>
       </c>
     </row>
@@ -6373,7 +6488,7 @@
       <c r="G55" t="s">
         <v>204</v>
       </c>
-      <c r="H55" s="7"/>
+      <c r="H55" s="8"/>
       <c r="I55" t="s">
         <v>210</v>
       </c>
@@ -6404,7 +6519,7 @@
       <c r="R55" t="s">
         <v>27</v>
       </c>
-      <c r="S55" s="8"/>
+      <c r="S55" s="9"/>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
@@ -6428,7 +6543,7 @@
       <c r="G56" t="s">
         <v>204</v>
       </c>
-      <c r="H56" s="7"/>
+      <c r="H56" s="8"/>
       <c r="I56" t="s">
         <v>210</v>
       </c>
@@ -6459,7 +6574,7 @@
       <c r="R56" t="s">
         <v>27</v>
       </c>
-      <c r="S56" s="8"/>
+      <c r="S56" s="9"/>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
@@ -6483,7 +6598,7 @@
       <c r="G57" t="s">
         <v>204</v>
       </c>
-      <c r="H57" s="7"/>
+      <c r="H57" s="8"/>
       <c r="I57" t="s">
         <v>210</v>
       </c>
@@ -6514,7 +6629,7 @@
       <c r="R57" t="s">
         <v>27</v>
       </c>
-      <c r="S57" s="8"/>
+      <c r="S57" s="9"/>
     </row>
     <row r="58" spans="1:19" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
@@ -6538,7 +6653,7 @@
       <c r="G58" t="s">
         <v>217</v>
       </c>
-      <c r="H58" s="7" t="s">
+      <c r="H58" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I58" t="s">
@@ -6571,7 +6686,7 @@
       <c r="R58" t="s">
         <v>27</v>
       </c>
-      <c r="S58" s="8" t="s">
+      <c r="S58" s="9" t="s">
         <v>227</v>
       </c>
     </row>
@@ -6597,7 +6712,7 @@
       <c r="G59" t="s">
         <v>217</v>
       </c>
-      <c r="H59" s="7"/>
+      <c r="H59" s="8"/>
       <c r="I59" t="s">
         <v>223</v>
       </c>
@@ -6628,7 +6743,7 @@
       <c r="R59" t="s">
         <v>27</v>
       </c>
-      <c r="S59" s="8"/>
+      <c r="S59" s="9"/>
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
@@ -6652,7 +6767,7 @@
       <c r="G60" t="s">
         <v>217</v>
       </c>
-      <c r="H60" s="7"/>
+      <c r="H60" s="8"/>
       <c r="I60" t="s">
         <v>223</v>
       </c>
@@ -6683,7 +6798,7 @@
       <c r="R60" t="s">
         <v>27</v>
       </c>
-      <c r="S60" s="8"/>
+      <c r="S60" s="9"/>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
@@ -6707,7 +6822,7 @@
       <c r="G61" t="s">
         <v>217</v>
       </c>
-      <c r="H61" s="7"/>
+      <c r="H61" s="8"/>
       <c r="I61" t="s">
         <v>223</v>
       </c>
@@ -6738,7 +6853,7 @@
       <c r="R61" t="s">
         <v>27</v>
       </c>
-      <c r="S61" s="8"/>
+      <c r="S61" s="9"/>
     </row>
     <row r="62" spans="1:19" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
@@ -6762,7 +6877,7 @@
       <c r="G62" t="s">
         <v>230</v>
       </c>
-      <c r="H62" s="7" t="s">
+      <c r="H62" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I62" t="s">
@@ -6795,7 +6910,7 @@
       <c r="R62" t="s">
         <v>27</v>
       </c>
-      <c r="S62" s="8" t="s">
+      <c r="S62" s="9" t="s">
         <v>238</v>
       </c>
     </row>
@@ -6821,7 +6936,7 @@
       <c r="G63" t="s">
         <v>230</v>
       </c>
-      <c r="H63" s="7"/>
+      <c r="H63" s="8"/>
       <c r="I63" t="s">
         <v>235</v>
       </c>
@@ -6852,7 +6967,7 @@
       <c r="R63" t="s">
         <v>27</v>
       </c>
-      <c r="S63" s="8"/>
+      <c r="S63" s="9"/>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
@@ -6876,7 +6991,7 @@
       <c r="G64" t="s">
         <v>230</v>
       </c>
-      <c r="H64" s="7"/>
+      <c r="H64" s="8"/>
       <c r="I64" t="s">
         <v>235</v>
       </c>
@@ -6907,7 +7022,7 @@
       <c r="R64" t="s">
         <v>27</v>
       </c>
-      <c r="S64" s="8"/>
+      <c r="S64" s="9"/>
     </row>
     <row r="65" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
@@ -6931,7 +7046,7 @@
       <c r="G65" t="s">
         <v>230</v>
       </c>
-      <c r="H65" s="7"/>
+      <c r="H65" s="8"/>
       <c r="I65" t="s">
         <v>235</v>
       </c>
@@ -6962,7 +7077,7 @@
       <c r="R65" t="s">
         <v>27</v>
       </c>
-      <c r="S65" s="8"/>
+      <c r="S65" s="9"/>
     </row>
     <row r="66" spans="1:19" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
@@ -6986,7 +7101,7 @@
       <c r="G66" t="s">
         <v>241</v>
       </c>
-      <c r="H66" s="7" t="s">
+      <c r="H66" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I66" t="s">
@@ -7019,7 +7134,7 @@
       <c r="R66" t="s">
         <v>248</v>
       </c>
-      <c r="S66" s="8" t="s">
+      <c r="S66" s="9" t="s">
         <v>251</v>
       </c>
     </row>
@@ -7045,7 +7160,7 @@
       <c r="G67" t="s">
         <v>241</v>
       </c>
-      <c r="H67" s="7"/>
+      <c r="H67" s="8"/>
       <c r="I67" t="s">
         <v>246</v>
       </c>
@@ -7076,7 +7191,7 @@
       <c r="R67" t="s">
         <v>248</v>
       </c>
-      <c r="S67" s="8"/>
+      <c r="S67" s="9"/>
     </row>
     <row r="68" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
@@ -7100,7 +7215,7 @@
       <c r="G68" t="s">
         <v>241</v>
       </c>
-      <c r="H68" s="7"/>
+      <c r="H68" s="8"/>
       <c r="I68" t="s">
         <v>246</v>
       </c>
@@ -7131,7 +7246,7 @@
       <c r="R68" t="s">
         <v>248</v>
       </c>
-      <c r="S68" s="8"/>
+      <c r="S68" s="9"/>
     </row>
     <row r="69" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
@@ -7155,7 +7270,7 @@
       <c r="G69" t="s">
         <v>241</v>
       </c>
-      <c r="H69" s="7"/>
+      <c r="H69" s="8"/>
       <c r="I69" t="s">
         <v>246</v>
       </c>
@@ -7186,7 +7301,7 @@
       <c r="R69" t="s">
         <v>248</v>
       </c>
-      <c r="S69" s="8"/>
+      <c r="S69" s="9"/>
     </row>
     <row r="70" spans="1:19" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
@@ -7210,7 +7325,7 @@
       <c r="G70" t="s">
         <v>254</v>
       </c>
-      <c r="H70" s="7" t="s">
+      <c r="H70" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I70" t="s">
@@ -7243,7 +7358,7 @@
       <c r="R70" t="s">
         <v>24</v>
       </c>
-      <c r="S70" s="8" t="s">
+      <c r="S70" s="9" t="s">
         <v>263</v>
       </c>
     </row>
@@ -7269,7 +7384,7 @@
       <c r="G71" t="s">
         <v>254</v>
       </c>
-      <c r="H71" s="7"/>
+      <c r="H71" s="8"/>
       <c r="I71" t="s">
         <v>259</v>
       </c>
@@ -7300,7 +7415,7 @@
       <c r="R71" t="s">
         <v>24</v>
       </c>
-      <c r="S71" s="8"/>
+      <c r="S71" s="9"/>
     </row>
     <row r="72" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
@@ -7324,7 +7439,7 @@
       <c r="G72" t="s">
         <v>254</v>
       </c>
-      <c r="H72" s="7"/>
+      <c r="H72" s="8"/>
       <c r="I72" t="s">
         <v>259</v>
       </c>
@@ -7355,7 +7470,7 @@
       <c r="R72" t="s">
         <v>24</v>
       </c>
-      <c r="S72" s="8"/>
+      <c r="S72" s="9"/>
     </row>
     <row r="73" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
@@ -7379,7 +7494,7 @@
       <c r="G73" t="s">
         <v>254</v>
       </c>
-      <c r="H73" s="7"/>
+      <c r="H73" s="8"/>
       <c r="I73" t="s">
         <v>259</v>
       </c>
@@ -7410,7 +7525,7 @@
       <c r="R73" t="s">
         <v>24</v>
       </c>
-      <c r="S73" s="8"/>
+      <c r="S73" s="9"/>
     </row>
     <row r="74" spans="1:19" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
@@ -7434,7 +7549,7 @@
       <c r="G74" t="s">
         <v>266</v>
       </c>
-      <c r="H74" s="7" t="s">
+      <c r="H74" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I74" t="s">
@@ -7467,7 +7582,7 @@
       <c r="R74" t="s">
         <v>24</v>
       </c>
-      <c r="S74" s="8" t="s">
+      <c r="S74" s="9" t="s">
         <v>287</v>
       </c>
     </row>
@@ -7493,7 +7608,7 @@
       <c r="G75" t="s">
         <v>266</v>
       </c>
-      <c r="H75" s="7"/>
+      <c r="H75" s="8"/>
       <c r="I75" t="s">
         <v>271</v>
       </c>
@@ -7524,7 +7639,7 @@
       <c r="R75" t="s">
         <v>24</v>
       </c>
-      <c r="S75" s="8"/>
+      <c r="S75" s="9"/>
     </row>
     <row r="76" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
@@ -7548,7 +7663,7 @@
       <c r="G76" t="s">
         <v>266</v>
       </c>
-      <c r="H76" s="7"/>
+      <c r="H76" s="8"/>
       <c r="I76" t="s">
         <v>271</v>
       </c>
@@ -7579,7 +7694,7 @@
       <c r="R76" t="s">
         <v>24</v>
       </c>
-      <c r="S76" s="8"/>
+      <c r="S76" s="9"/>
     </row>
     <row r="77" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
@@ -7603,7 +7718,7 @@
       <c r="G77" t="s">
         <v>266</v>
       </c>
-      <c r="H77" s="7"/>
+      <c r="H77" s="8"/>
       <c r="I77" t="s">
         <v>271</v>
       </c>
@@ -7634,7 +7749,7 @@
       <c r="R77" t="s">
         <v>24</v>
       </c>
-      <c r="S77" s="8"/>
+      <c r="S77" s="9"/>
     </row>
     <row r="78" spans="1:19" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
@@ -7658,7 +7773,7 @@
       <c r="G78" t="s">
         <v>276</v>
       </c>
-      <c r="H78" s="7" t="s">
+      <c r="H78" s="8" t="s">
         <v>281</v>
       </c>
       <c r="I78" t="s">
@@ -7691,7 +7806,7 @@
       <c r="R78" t="s">
         <v>285</v>
       </c>
-      <c r="S78" s="8" t="s">
+      <c r="S78" s="9" t="s">
         <v>288</v>
       </c>
     </row>
@@ -7717,7 +7832,7 @@
       <c r="G79" t="s">
         <v>276</v>
       </c>
-      <c r="H79" s="7"/>
+      <c r="H79" s="8"/>
       <c r="I79" t="s">
         <v>283</v>
       </c>
@@ -7748,7 +7863,7 @@
       <c r="R79" t="s">
         <v>285</v>
       </c>
-      <c r="S79" s="8"/>
+      <c r="S79" s="9"/>
     </row>
     <row r="80" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
@@ -7772,7 +7887,7 @@
       <c r="G80" t="s">
         <v>276</v>
       </c>
-      <c r="H80" s="7"/>
+      <c r="H80" s="8"/>
       <c r="I80" t="s">
         <v>283</v>
       </c>
@@ -7803,7 +7918,7 @@
       <c r="R80" t="s">
         <v>285</v>
       </c>
-      <c r="S80" s="8"/>
+      <c r="S80" s="9"/>
     </row>
     <row r="81" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
@@ -7827,7 +7942,7 @@
       <c r="G81" t="s">
         <v>276</v>
       </c>
-      <c r="H81" s="7"/>
+      <c r="H81" s="8"/>
       <c r="I81" t="s">
         <v>283</v>
       </c>
@@ -7858,7 +7973,7 @@
       <c r="R81" t="s">
         <v>285</v>
       </c>
-      <c r="S81" s="8"/>
+      <c r="S81" s="9"/>
     </row>
     <row r="82" spans="1:20" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
@@ -7882,7 +7997,7 @@
       <c r="G82" t="s">
         <v>291</v>
       </c>
-      <c r="H82" s="7" t="s">
+      <c r="H82" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I82" t="s">
@@ -7915,7 +8030,7 @@
       <c r="R82" t="s">
         <v>27</v>
       </c>
-      <c r="S82" s="8" t="s">
+      <c r="S82" s="9" t="s">
         <v>300</v>
       </c>
     </row>
@@ -7941,7 +8056,7 @@
       <c r="G83" t="s">
         <v>291</v>
       </c>
-      <c r="H83" s="7"/>
+      <c r="H83" s="8"/>
       <c r="I83" t="s">
         <v>297</v>
       </c>
@@ -7972,7 +8087,7 @@
       <c r="R83" t="s">
         <v>27</v>
       </c>
-      <c r="S83" s="8"/>
+      <c r="S83" s="9"/>
     </row>
     <row r="84" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
@@ -7996,7 +8111,7 @@
       <c r="G84" t="s">
         <v>291</v>
       </c>
-      <c r="H84" s="7"/>
+      <c r="H84" s="8"/>
       <c r="I84" t="s">
         <v>297</v>
       </c>
@@ -8027,7 +8142,7 @@
       <c r="R84" t="s">
         <v>27</v>
       </c>
-      <c r="S84" s="8"/>
+      <c r="S84" s="9"/>
     </row>
     <row r="85" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
@@ -8051,7 +8166,7 @@
       <c r="G85" t="s">
         <v>291</v>
       </c>
-      <c r="H85" s="7"/>
+      <c r="H85" s="8"/>
       <c r="I85" t="s">
         <v>297</v>
       </c>
@@ -8082,7 +8197,7 @@
       <c r="R85" t="s">
         <v>27</v>
       </c>
-      <c r="S85" s="8"/>
+      <c r="S85" s="9"/>
     </row>
     <row r="86" spans="1:20" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
@@ -8106,7 +8221,7 @@
       <c r="G86" t="s">
         <v>303</v>
       </c>
-      <c r="H86" s="7" t="s">
+      <c r="H86" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I86" t="s">
@@ -8139,7 +8254,7 @@
       <c r="R86" t="s">
         <v>27</v>
       </c>
-      <c r="S86" s="8" t="s">
+      <c r="S86" s="9" t="s">
         <v>312</v>
       </c>
     </row>
@@ -8165,7 +8280,7 @@
       <c r="G87" t="s">
         <v>303</v>
       </c>
-      <c r="H87" s="7"/>
+      <c r="H87" s="8"/>
       <c r="I87" t="s">
         <v>308</v>
       </c>
@@ -8196,7 +8311,7 @@
       <c r="R87" t="s">
         <v>27</v>
       </c>
-      <c r="S87" s="8"/>
+      <c r="S87" s="9"/>
     </row>
     <row r="88" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
@@ -8220,7 +8335,7 @@
       <c r="G88" t="s">
         <v>303</v>
       </c>
-      <c r="H88" s="7"/>
+      <c r="H88" s="8"/>
       <c r="I88" t="s">
         <v>308</v>
       </c>
@@ -8251,7 +8366,7 @@
       <c r="R88" t="s">
         <v>27</v>
       </c>
-      <c r="S88" s="8"/>
+      <c r="S88" s="9"/>
     </row>
     <row r="89" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
@@ -8275,7 +8390,7 @@
       <c r="G89" t="s">
         <v>303</v>
       </c>
-      <c r="H89" s="7"/>
+      <c r="H89" s="8"/>
       <c r="I89" t="s">
         <v>308</v>
       </c>
@@ -8306,7 +8421,7 @@
       <c r="R89" t="s">
         <v>27</v>
       </c>
-      <c r="S89" s="8"/>
+      <c r="S89" s="9"/>
     </row>
     <row r="90" spans="1:20" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
@@ -8330,7 +8445,7 @@
       <c r="G90" t="s">
         <v>409</v>
       </c>
-      <c r="H90" s="7" t="s">
+      <c r="H90" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I90" t="s">
@@ -8342,7 +8457,7 @@
       <c r="K90" t="s">
         <v>36</v>
       </c>
-      <c r="L90" s="10" t="s">
+      <c r="L90" s="7" t="s">
         <v>412</v>
       </c>
       <c r="M90" t="s">
@@ -8363,10 +8478,10 @@
       <c r="R90" t="s">
         <v>27</v>
       </c>
-      <c r="S90" s="8" t="s">
+      <c r="S90" s="9" t="s">
         <v>415</v>
       </c>
-      <c r="T90" s="10" t="s">
+      <c r="T90" s="7" t="s">
         <v>402</v>
       </c>
     </row>
@@ -8392,7 +8507,7 @@
       <c r="G91" t="s">
         <v>409</v>
       </c>
-      <c r="H91" s="7"/>
+      <c r="H91" s="8"/>
       <c r="I91" t="s">
         <v>410</v>
       </c>
@@ -8402,7 +8517,7 @@
       <c r="K91" t="s">
         <v>36</v>
       </c>
-      <c r="L91" s="10" t="s">
+      <c r="L91" s="7" t="s">
         <v>412</v>
       </c>
       <c r="M91" t="s">
@@ -8423,7 +8538,7 @@
       <c r="R91" t="s">
         <v>27</v>
       </c>
-      <c r="S91" s="8"/>
+      <c r="S91" s="9"/>
     </row>
     <row r="92" spans="1:20" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
@@ -8447,7 +8562,7 @@
       <c r="G92" t="s">
         <v>409</v>
       </c>
-      <c r="H92" s="7"/>
+      <c r="H92" s="8"/>
       <c r="I92" t="s">
         <v>410</v>
       </c>
@@ -8457,7 +8572,7 @@
       <c r="K92" t="s">
         <v>36</v>
       </c>
-      <c r="L92" s="10" t="s">
+      <c r="L92" s="7" t="s">
         <v>412</v>
       </c>
       <c r="M92" t="s">
@@ -8478,7 +8593,7 @@
       <c r="R92" t="s">
         <v>27</v>
       </c>
-      <c r="S92" s="8"/>
+      <c r="S92" s="9"/>
     </row>
     <row r="93" spans="1:20" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
@@ -8502,7 +8617,7 @@
       <c r="G93" t="s">
         <v>409</v>
       </c>
-      <c r="H93" s="7"/>
+      <c r="H93" s="8"/>
       <c r="I93" t="s">
         <v>410</v>
       </c>
@@ -8512,7 +8627,7 @@
       <c r="K93" t="s">
         <v>36</v>
       </c>
-      <c r="L93" s="10" t="s">
+      <c r="L93" s="7" t="s">
         <v>412</v>
       </c>
       <c r="M93" t="s">
@@ -8533,7 +8648,7 @@
       <c r="R93" t="s">
         <v>27</v>
       </c>
-      <c r="S93" s="8"/>
+      <c r="S93" s="9"/>
     </row>
     <row r="94" spans="1:20" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
@@ -8557,7 +8672,7 @@
       <c r="G94" t="s">
         <v>317</v>
       </c>
-      <c r="H94" s="7" t="s">
+      <c r="H94" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I94" t="s">
@@ -8590,7 +8705,7 @@
       <c r="R94" t="s">
         <v>27</v>
       </c>
-      <c r="S94" s="8" t="s">
+      <c r="S94" s="9" t="s">
         <v>325</v>
       </c>
     </row>
@@ -8616,7 +8731,7 @@
       <c r="G95" t="s">
         <v>317</v>
       </c>
-      <c r="H95" s="7"/>
+      <c r="H95" s="8"/>
       <c r="I95" t="s">
         <v>322</v>
       </c>
@@ -8647,7 +8762,7 @@
       <c r="R95" t="s">
         <v>27</v>
       </c>
-      <c r="S95" s="8"/>
+      <c r="S95" s="9"/>
     </row>
     <row r="96" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
@@ -8671,7 +8786,7 @@
       <c r="G96" t="s">
         <v>317</v>
       </c>
-      <c r="H96" s="7"/>
+      <c r="H96" s="8"/>
       <c r="I96" t="s">
         <v>322</v>
       </c>
@@ -8702,7 +8817,7 @@
       <c r="R96" t="s">
         <v>27</v>
       </c>
-      <c r="S96" s="8"/>
+      <c r="S96" s="9"/>
     </row>
     <row r="97" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
@@ -8726,7 +8841,7 @@
       <c r="G97" t="s">
         <v>317</v>
       </c>
-      <c r="H97" s="7"/>
+      <c r="H97" s="8"/>
       <c r="I97" t="s">
         <v>322</v>
       </c>
@@ -8757,7 +8872,7 @@
       <c r="R97" t="s">
         <v>27</v>
       </c>
-      <c r="S97" s="8"/>
+      <c r="S97" s="9"/>
     </row>
     <row r="98" spans="1:19" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
@@ -8781,7 +8896,7 @@
       <c r="G98" t="s">
         <v>329</v>
       </c>
-      <c r="H98" s="7" t="s">
+      <c r="H98" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I98" t="s">
@@ -8814,7 +8929,7 @@
       <c r="R98" t="s">
         <v>27</v>
       </c>
-      <c r="S98" s="8" t="s">
+      <c r="S98" s="9" t="s">
         <v>337</v>
       </c>
     </row>
@@ -8840,7 +8955,7 @@
       <c r="G99" t="s">
         <v>329</v>
       </c>
-      <c r="H99" s="7"/>
+      <c r="H99" s="8"/>
       <c r="I99" t="s">
         <v>334</v>
       </c>
@@ -8871,7 +8986,7 @@
       <c r="R99" t="s">
         <v>27</v>
       </c>
-      <c r="S99" s="8"/>
+      <c r="S99" s="9"/>
     </row>
     <row r="100" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
@@ -8895,7 +9010,7 @@
       <c r="G100" t="s">
         <v>329</v>
       </c>
-      <c r="H100" s="7"/>
+      <c r="H100" s="8"/>
       <c r="I100" t="s">
         <v>334</v>
       </c>
@@ -8926,7 +9041,7 @@
       <c r="R100" t="s">
         <v>27</v>
       </c>
-      <c r="S100" s="8"/>
+      <c r="S100" s="9"/>
     </row>
     <row r="101" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
@@ -8950,7 +9065,7 @@
       <c r="G101" t="s">
         <v>329</v>
       </c>
-      <c r="H101" s="7"/>
+      <c r="H101" s="8"/>
       <c r="I101" t="s">
         <v>334</v>
       </c>
@@ -8981,7 +9096,7 @@
       <c r="R101" t="s">
         <v>27</v>
       </c>
-      <c r="S101" s="8"/>
+      <c r="S101" s="9"/>
     </row>
     <row r="102" spans="1:19" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
@@ -9005,7 +9120,7 @@
       <c r="G102" t="s">
         <v>340</v>
       </c>
-      <c r="H102" s="7" t="s">
+      <c r="H102" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I102" t="s">
@@ -9038,7 +9153,7 @@
       <c r="R102" t="s">
         <v>27</v>
       </c>
-      <c r="S102" s="8" t="s">
+      <c r="S102" s="9" t="s">
         <v>347</v>
       </c>
     </row>
@@ -9064,7 +9179,7 @@
       <c r="G103" t="s">
         <v>340</v>
       </c>
-      <c r="H103" s="7"/>
+      <c r="H103" s="8"/>
       <c r="I103" t="s">
         <v>345</v>
       </c>
@@ -9095,7 +9210,7 @@
       <c r="R103" t="s">
         <v>27</v>
       </c>
-      <c r="S103" s="8"/>
+      <c r="S103" s="9"/>
     </row>
     <row r="104" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
@@ -9119,7 +9234,7 @@
       <c r="G104" t="s">
         <v>340</v>
       </c>
-      <c r="H104" s="7"/>
+      <c r="H104" s="8"/>
       <c r="I104" t="s">
         <v>345</v>
       </c>
@@ -9150,7 +9265,7 @@
       <c r="R104" t="s">
         <v>27</v>
       </c>
-      <c r="S104" s="8"/>
+      <c r="S104" s="9"/>
     </row>
     <row r="105" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
@@ -9174,7 +9289,7 @@
       <c r="G105" t="s">
         <v>340</v>
       </c>
-      <c r="H105" s="7"/>
+      <c r="H105" s="8"/>
       <c r="I105" t="s">
         <v>345</v>
       </c>
@@ -9205,7 +9320,7 @@
       <c r="R105" t="s">
         <v>27</v>
       </c>
-      <c r="S105" s="8"/>
+      <c r="S105" s="9"/>
     </row>
     <row r="106" spans="1:19" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
@@ -9229,7 +9344,7 @@
       <c r="G106" t="s">
         <v>351</v>
       </c>
-      <c r="H106" s="7" t="s">
+      <c r="H106" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I106" t="s">
@@ -9262,7 +9377,7 @@
       <c r="R106" t="s">
         <v>27</v>
       </c>
-      <c r="S106" s="8" t="s">
+      <c r="S106" s="9" t="s">
         <v>359</v>
       </c>
     </row>
@@ -9288,7 +9403,7 @@
       <c r="G107" t="s">
         <v>351</v>
       </c>
-      <c r="H107" s="7"/>
+      <c r="H107" s="8"/>
       <c r="I107" t="s">
         <v>356</v>
       </c>
@@ -9319,7 +9434,7 @@
       <c r="R107" t="s">
         <v>27</v>
       </c>
-      <c r="S107" s="8"/>
+      <c r="S107" s="9"/>
     </row>
     <row r="108" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
@@ -9343,7 +9458,7 @@
       <c r="G108" t="s">
         <v>351</v>
       </c>
-      <c r="H108" s="7"/>
+      <c r="H108" s="8"/>
       <c r="I108" t="s">
         <v>356</v>
       </c>
@@ -9374,7 +9489,7 @@
       <c r="R108" t="s">
         <v>27</v>
       </c>
-      <c r="S108" s="8"/>
+      <c r="S108" s="9"/>
     </row>
     <row r="109" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
@@ -9398,7 +9513,7 @@
       <c r="G109" t="s">
         <v>351</v>
       </c>
-      <c r="H109" s="7"/>
+      <c r="H109" s="8"/>
       <c r="I109" t="s">
         <v>356</v>
       </c>
@@ -9429,7 +9544,7 @@
       <c r="R109" t="s">
         <v>27</v>
       </c>
-      <c r="S109" s="8"/>
+      <c r="S109" s="9"/>
     </row>
     <row r="110" spans="1:19" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
@@ -9453,7 +9568,7 @@
       <c r="G110" t="s">
         <v>362</v>
       </c>
-      <c r="H110" s="7" t="s">
+      <c r="H110" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I110" t="s">
@@ -9486,7 +9601,7 @@
       <c r="R110" t="s">
         <v>27</v>
       </c>
-      <c r="S110" s="8" t="s">
+      <c r="S110" s="9" t="s">
         <v>371</v>
       </c>
     </row>
@@ -9512,7 +9627,7 @@
       <c r="G111" t="s">
         <v>362</v>
       </c>
-      <c r="H111" s="7"/>
+      <c r="H111" s="8"/>
       <c r="I111" t="s">
         <v>367</v>
       </c>
@@ -9543,7 +9658,7 @@
       <c r="R111" t="s">
         <v>27</v>
       </c>
-      <c r="S111" s="8"/>
+      <c r="S111" s="9"/>
     </row>
     <row r="112" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
@@ -9567,7 +9682,7 @@
       <c r="G112" t="s">
         <v>362</v>
       </c>
-      <c r="H112" s="7"/>
+      <c r="H112" s="8"/>
       <c r="I112" t="s">
         <v>367</v>
       </c>
@@ -9598,9 +9713,9 @@
       <c r="R112" t="s">
         <v>27</v>
       </c>
-      <c r="S112" s="8"/>
-    </row>
-    <row r="113" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S112" s="9"/>
+    </row>
+    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>360</v>
       </c>
@@ -9622,7 +9737,7 @@
       <c r="G113" t="s">
         <v>362</v>
       </c>
-      <c r="H113" s="7"/>
+      <c r="H113" s="8"/>
       <c r="I113" t="s">
         <v>367</v>
       </c>
@@ -9653,9 +9768,9 @@
       <c r="R113" t="s">
         <v>27</v>
       </c>
-      <c r="S113" s="8"/>
-    </row>
-    <row r="114" spans="1:19" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S113" s="9"/>
+    </row>
+    <row r="114" spans="1:20" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>372</v>
       </c>
@@ -9677,7 +9792,7 @@
       <c r="G114" t="s">
         <v>374</v>
       </c>
-      <c r="H114" s="7" t="s">
+      <c r="H114" s="8" t="s">
         <v>380</v>
       </c>
       <c r="I114" t="s">
@@ -9710,11 +9825,11 @@
       <c r="R114" t="s">
         <v>383</v>
       </c>
-      <c r="S114" s="8" t="s">
+      <c r="S114" s="9" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="115" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>372</v>
       </c>
@@ -9736,7 +9851,7 @@
       <c r="G115" t="s">
         <v>374</v>
       </c>
-      <c r="H115" s="7"/>
+      <c r="H115" s="8"/>
       <c r="I115" t="s">
         <v>381</v>
       </c>
@@ -9767,9 +9882,9 @@
       <c r="R115" t="s">
         <v>383</v>
       </c>
-      <c r="S115" s="8"/>
-    </row>
-    <row r="116" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S115" s="9"/>
+    </row>
+    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>372</v>
       </c>
@@ -9791,7 +9906,7 @@
       <c r="G116" t="s">
         <v>374</v>
       </c>
-      <c r="H116" s="7"/>
+      <c r="H116" s="8"/>
       <c r="I116" t="s">
         <v>381</v>
       </c>
@@ -9822,9 +9937,9 @@
       <c r="R116" t="s">
         <v>383</v>
       </c>
-      <c r="S116" s="8"/>
-    </row>
-    <row r="117" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S116" s="9"/>
+    </row>
+    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>372</v>
       </c>
@@ -9846,7 +9961,7 @@
       <c r="G117" t="s">
         <v>374</v>
       </c>
-      <c r="H117" s="7"/>
+      <c r="H117" s="8"/>
       <c r="I117" t="s">
         <v>381</v>
       </c>
@@ -9877,9 +9992,9 @@
       <c r="R117" t="s">
         <v>383</v>
       </c>
-      <c r="S117" s="8"/>
-    </row>
-    <row r="118" spans="1:19" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S117" s="9"/>
+    </row>
+    <row r="118" spans="1:20" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>386</v>
       </c>
@@ -9901,7 +10016,7 @@
       <c r="G118" t="s">
         <v>389</v>
       </c>
-      <c r="H118" s="7" t="s">
+      <c r="H118" s="8" t="s">
         <v>395</v>
       </c>
       <c r="I118" t="s">
@@ -9934,11 +10049,11 @@
       <c r="R118" t="s">
         <v>398</v>
       </c>
-      <c r="S118" s="8" t="s">
+      <c r="S118" s="9" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="119" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>386</v>
       </c>
@@ -9960,7 +10075,7 @@
       <c r="G119" t="s">
         <v>389</v>
       </c>
-      <c r="H119" s="7"/>
+      <c r="H119" s="8"/>
       <c r="I119" t="s">
         <v>396</v>
       </c>
@@ -9991,9 +10106,9 @@
       <c r="R119" t="s">
         <v>398</v>
       </c>
-      <c r="S119" s="8"/>
-    </row>
-    <row r="120" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S119" s="9"/>
+    </row>
+    <row r="120" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>386</v>
       </c>
@@ -10015,7 +10130,7 @@
       <c r="G120" t="s">
         <v>389</v>
       </c>
-      <c r="H120" s="7"/>
+      <c r="H120" s="8"/>
       <c r="I120" t="s">
         <v>396</v>
       </c>
@@ -10046,9 +10161,9 @@
       <c r="R120" t="s">
         <v>398</v>
       </c>
-      <c r="S120" s="8"/>
-    </row>
-    <row r="121" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S120" s="9"/>
+    </row>
+    <row r="121" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>386</v>
       </c>
@@ -10070,7 +10185,7 @@
       <c r="G121" t="s">
         <v>389</v>
       </c>
-      <c r="H121" s="7"/>
+      <c r="H121" s="8"/>
       <c r="I121" t="s">
         <v>396</v>
       </c>
@@ -10101,9 +10216,9 @@
       <c r="R121" t="s">
         <v>398</v>
       </c>
-      <c r="S121" s="8"/>
-    </row>
-    <row r="122" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S121" s="9"/>
+    </row>
+    <row r="122" spans="1:20" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>416</v>
       </c>
@@ -10125,7 +10240,7 @@
       <c r="G122" t="s">
         <v>419</v>
       </c>
-      <c r="H122" s="7" t="s">
+      <c r="H122" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I122" t="s">
@@ -10158,11 +10273,11 @@
       <c r="R122" t="s">
         <v>27</v>
       </c>
-      <c r="S122" s="8" t="s">
+      <c r="S122" s="9" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="123" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>416</v>
       </c>
@@ -10184,7 +10299,7 @@
       <c r="G123" t="s">
         <v>419</v>
       </c>
-      <c r="H123" s="7"/>
+      <c r="H123" s="8"/>
       <c r="I123" t="s">
         <v>424</v>
       </c>
@@ -10215,9 +10330,9 @@
       <c r="R123" t="s">
         <v>27</v>
       </c>
-      <c r="S123" s="8"/>
-    </row>
-    <row r="124" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S123" s="9"/>
+    </row>
+    <row r="124" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>416</v>
       </c>
@@ -10239,7 +10354,7 @@
       <c r="G124" t="s">
         <v>419</v>
       </c>
-      <c r="H124" s="7"/>
+      <c r="H124" s="8"/>
       <c r="I124" t="s">
         <v>424</v>
       </c>
@@ -10270,9 +10385,9 @@
       <c r="R124" t="s">
         <v>27</v>
       </c>
-      <c r="S124" s="8"/>
-    </row>
-    <row r="125" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S124" s="9"/>
+    </row>
+    <row r="125" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>416</v>
       </c>
@@ -10294,7 +10409,7 @@
       <c r="G125" t="s">
         <v>419</v>
       </c>
-      <c r="H125" s="7"/>
+      <c r="H125" s="8"/>
       <c r="I125" t="s">
         <v>424</v>
       </c>
@@ -10325,29 +10440,239 @@
       <c r="R125" t="s">
         <v>27</v>
       </c>
-      <c r="S125" s="8"/>
-    </row>
-    <row r="126" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S125" s="9"/>
+    </row>
+    <row r="126" spans="1:20" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="127" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="B126" s="3">
+        <v>2151</v>
+      </c>
+      <c r="C126" t="s">
+        <v>501</v>
+      </c>
+      <c r="D126" t="s">
+        <v>502</v>
+      </c>
+      <c r="E126" t="s">
+        <v>504</v>
+      </c>
+      <c r="F126" t="s">
+        <v>508</v>
+      </c>
+      <c r="G126" t="s">
+        <v>503</v>
+      </c>
+      <c r="H126" s="8" t="s">
+        <v>296</v>
+      </c>
+      <c r="I126" t="s">
+        <v>509</v>
+      </c>
+      <c r="J126" t="s">
+        <v>510</v>
+      </c>
+      <c r="K126" t="s">
+        <v>36</v>
+      </c>
+      <c r="L126" t="s">
+        <v>511</v>
+      </c>
+      <c r="M126" t="s">
+        <v>27</v>
+      </c>
+      <c r="N126" t="s">
+        <v>324</v>
+      </c>
+      <c r="O126" t="s">
+        <v>324</v>
+      </c>
+      <c r="P126" t="s">
+        <v>324</v>
+      </c>
+      <c r="Q126" t="s">
+        <v>324</v>
+      </c>
+      <c r="R126" t="s">
+        <v>27</v>
+      </c>
+      <c r="S126" s="9" t="s">
+        <v>512</v>
+      </c>
+      <c r="T126" s="10" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="127" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="128" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="B127" s="3">
+        <v>2151</v>
+      </c>
+      <c r="C127" t="s">
+        <v>501</v>
+      </c>
+      <c r="D127" t="s">
+        <v>502</v>
+      </c>
+      <c r="E127" t="s">
+        <v>505</v>
+      </c>
+      <c r="F127" t="s">
+        <v>508</v>
+      </c>
+      <c r="G127" t="s">
+        <v>503</v>
+      </c>
+      <c r="H127" s="8"/>
+      <c r="I127" t="s">
+        <v>509</v>
+      </c>
+      <c r="J127" t="s">
+        <v>510</v>
+      </c>
+      <c r="K127" t="s">
+        <v>36</v>
+      </c>
+      <c r="L127" t="s">
+        <v>511</v>
+      </c>
+      <c r="M127" t="s">
+        <v>27</v>
+      </c>
+      <c r="N127" t="s">
+        <v>324</v>
+      </c>
+      <c r="O127" t="s">
+        <v>324</v>
+      </c>
+      <c r="P127" t="s">
+        <v>324</v>
+      </c>
+      <c r="Q127" t="s">
+        <v>324</v>
+      </c>
+      <c r="R127" t="s">
+        <v>27</v>
+      </c>
+      <c r="S127" s="9"/>
+      <c r="T127" s="10"/>
+    </row>
+    <row r="128" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="129" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="B128" s="3">
+        <v>2151</v>
+      </c>
+      <c r="C128" t="s">
+        <v>501</v>
+      </c>
+      <c r="D128" t="s">
+        <v>502</v>
+      </c>
+      <c r="E128" t="s">
+        <v>506</v>
+      </c>
+      <c r="F128" t="s">
+        <v>508</v>
+      </c>
+      <c r="G128" t="s">
+        <v>503</v>
+      </c>
+      <c r="H128" s="8"/>
+      <c r="I128" t="s">
+        <v>509</v>
+      </c>
+      <c r="J128" t="s">
+        <v>510</v>
+      </c>
+      <c r="K128" t="s">
+        <v>36</v>
+      </c>
+      <c r="L128" t="s">
+        <v>511</v>
+      </c>
+      <c r="M128" t="s">
+        <v>27</v>
+      </c>
+      <c r="N128" t="s">
+        <v>324</v>
+      </c>
+      <c r="O128" t="s">
+        <v>324</v>
+      </c>
+      <c r="P128" t="s">
+        <v>324</v>
+      </c>
+      <c r="Q128" t="s">
+        <v>324</v>
+      </c>
+      <c r="R128" t="s">
+        <v>27</v>
+      </c>
+      <c r="S128" s="9"/>
+      <c r="T128" s="10"/>
+    </row>
+    <row r="129" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>427</v>
       </c>
-    </row>
-    <row r="130" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B129" s="3">
+        <v>2151</v>
+      </c>
+      <c r="C129" t="s">
+        <v>501</v>
+      </c>
+      <c r="D129" t="s">
+        <v>502</v>
+      </c>
+      <c r="E129" t="s">
+        <v>507</v>
+      </c>
+      <c r="F129" t="s">
+        <v>508</v>
+      </c>
+      <c r="G129" t="s">
+        <v>503</v>
+      </c>
+      <c r="H129" s="8"/>
+      <c r="I129" t="s">
+        <v>509</v>
+      </c>
+      <c r="J129" t="s">
+        <v>510</v>
+      </c>
+      <c r="K129" t="s">
+        <v>36</v>
+      </c>
+      <c r="L129" t="s">
+        <v>511</v>
+      </c>
+      <c r="M129" t="s">
+        <v>27</v>
+      </c>
+      <c r="N129" t="s">
+        <v>324</v>
+      </c>
+      <c r="O129" t="s">
+        <v>324</v>
+      </c>
+      <c r="P129" t="s">
+        <v>324</v>
+      </c>
+      <c r="Q129" t="s">
+        <v>324</v>
+      </c>
+      <c r="R129" t="s">
+        <v>27</v>
+      </c>
+      <c r="S129" s="9"/>
+      <c r="T129" s="10"/>
+    </row>
+    <row r="130" spans="1:20" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>428</v>
       </c>
@@ -10369,7 +10694,7 @@
       <c r="G130" t="s">
         <v>432</v>
       </c>
-      <c r="H130" s="7" t="s">
+      <c r="H130" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I130" t="s">
@@ -10402,11 +10727,11 @@
       <c r="R130" t="s">
         <v>430</v>
       </c>
-      <c r="S130" s="8" t="s">
+      <c r="S130" s="9" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="131" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>428</v>
       </c>
@@ -10428,7 +10753,7 @@
       <c r="G131" t="s">
         <v>432</v>
       </c>
-      <c r="H131" s="7"/>
+      <c r="H131" s="8"/>
       <c r="I131" t="s">
         <v>437</v>
       </c>
@@ -10459,9 +10784,9 @@
       <c r="R131" t="s">
         <v>430</v>
       </c>
-      <c r="S131" s="8"/>
-    </row>
-    <row r="132" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S131" s="9"/>
+    </row>
+    <row r="132" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>428</v>
       </c>
@@ -10483,7 +10808,7 @@
       <c r="G132" t="s">
         <v>432</v>
       </c>
-      <c r="H132" s="7"/>
+      <c r="H132" s="8"/>
       <c r="I132" t="s">
         <v>437</v>
       </c>
@@ -10514,9 +10839,9 @@
       <c r="R132" t="s">
         <v>430</v>
       </c>
-      <c r="S132" s="8"/>
-    </row>
-    <row r="133" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S132" s="9"/>
+    </row>
+    <row r="133" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>428</v>
       </c>
@@ -10538,7 +10863,7 @@
       <c r="G133" t="s">
         <v>432</v>
       </c>
-      <c r="H133" s="7"/>
+      <c r="H133" s="8"/>
       <c r="I133" t="s">
         <v>437</v>
       </c>
@@ -10569,9 +10894,9 @@
       <c r="R133" t="s">
         <v>430</v>
       </c>
-      <c r="S133" s="8"/>
-    </row>
-    <row r="134" spans="1:19" ht="144" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S133" s="9"/>
+    </row>
+    <row r="134" spans="1:20" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>440</v>
       </c>
@@ -10593,7 +10918,7 @@
       <c r="G134" t="s">
         <v>442</v>
       </c>
-      <c r="H134" s="7" t="s">
+      <c r="H134" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I134" t="s">
@@ -10626,11 +10951,11 @@
       <c r="R134" t="s">
         <v>27</v>
       </c>
-      <c r="S134" s="8" t="s">
+      <c r="S134" s="9" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="135" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>440</v>
       </c>
@@ -10652,7 +10977,7 @@
       <c r="G135" t="s">
         <v>442</v>
       </c>
-      <c r="H135" s="7"/>
+      <c r="H135" s="8"/>
       <c r="I135" t="s">
         <v>447</v>
       </c>
@@ -10683,9 +11008,9 @@
       <c r="R135" t="s">
         <v>27</v>
       </c>
-      <c r="S135" s="8"/>
-    </row>
-    <row r="136" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S135" s="9"/>
+    </row>
+    <row r="136" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>440</v>
       </c>
@@ -10707,7 +11032,7 @@
       <c r="G136" t="s">
         <v>442</v>
       </c>
-      <c r="H136" s="7"/>
+      <c r="H136" s="8"/>
       <c r="I136" t="s">
         <v>447</v>
       </c>
@@ -10738,9 +11063,9 @@
       <c r="R136" t="s">
         <v>27</v>
       </c>
-      <c r="S136" s="8"/>
-    </row>
-    <row r="137" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S136" s="9"/>
+    </row>
+    <row r="137" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>440</v>
       </c>
@@ -10762,7 +11087,7 @@
       <c r="G137" t="s">
         <v>442</v>
       </c>
-      <c r="H137" s="7"/>
+      <c r="H137" s="8"/>
       <c r="I137" t="s">
         <v>447</v>
       </c>
@@ -10793,9 +11118,9 @@
       <c r="R137" t="s">
         <v>27</v>
       </c>
-      <c r="S137" s="8"/>
-    </row>
-    <row r="138" spans="1:19" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S137" s="9"/>
+    </row>
+    <row r="138" spans="1:20" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>451</v>
       </c>
@@ -10817,7 +11142,7 @@
       <c r="G138" t="s">
         <v>453</v>
       </c>
-      <c r="H138" s="7" t="s">
+      <c r="H138" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I138" t="s">
@@ -10850,11 +11175,11 @@
       <c r="R138" t="s">
         <v>461</v>
       </c>
-      <c r="S138" s="8" t="s">
+      <c r="S138" s="9" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="139" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>451</v>
       </c>
@@ -10876,7 +11201,7 @@
       <c r="G139" t="s">
         <v>453</v>
       </c>
-      <c r="H139" s="7"/>
+      <c r="H139" s="8"/>
       <c r="I139" t="s">
         <v>458</v>
       </c>
@@ -10907,9 +11232,9 @@
       <c r="R139" t="s">
         <v>461</v>
       </c>
-      <c r="S139" s="8"/>
-    </row>
-    <row r="140" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S139" s="9"/>
+    </row>
+    <row r="140" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>451</v>
       </c>
@@ -10931,7 +11256,7 @@
       <c r="G140" t="s">
         <v>453</v>
       </c>
-      <c r="H140" s="7"/>
+      <c r="H140" s="8"/>
       <c r="I140" t="s">
         <v>458</v>
       </c>
@@ -10962,9 +11287,9 @@
       <c r="R140" t="s">
         <v>461</v>
       </c>
-      <c r="S140" s="8"/>
-    </row>
-    <row r="141" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S140" s="9"/>
+    </row>
+    <row r="141" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>451</v>
       </c>
@@ -10986,7 +11311,7 @@
       <c r="G141" t="s">
         <v>453</v>
       </c>
-      <c r="H141" s="7"/>
+      <c r="H141" s="8"/>
       <c r="I141" t="s">
         <v>458</v>
       </c>
@@ -11017,9 +11342,9 @@
       <c r="R141" t="s">
         <v>461</v>
       </c>
-      <c r="S141" s="8"/>
-    </row>
-    <row r="142" spans="1:19" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="S141" s="9"/>
+    </row>
+    <row r="142" spans="1:20" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>463</v>
       </c>
@@ -11041,7 +11366,7 @@
       <c r="G142" t="s">
         <v>466</v>
       </c>
-      <c r="H142" s="7" t="s">
+      <c r="H142" s="8" t="s">
         <v>473</v>
       </c>
       <c r="I142" t="s">
@@ -11074,11 +11399,11 @@
       <c r="R142" t="s">
         <v>27</v>
       </c>
-      <c r="S142" s="8" t="s">
+      <c r="S142" s="9" t="s">
         <v>478</v>
       </c>
     </row>
-    <row r="143" spans="1:19" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>463</v>
       </c>
@@ -11100,7 +11425,7 @@
       <c r="G143" t="s">
         <v>466</v>
       </c>
-      <c r="H143" s="7"/>
+      <c r="H143" s="8"/>
       <c r="I143" t="s">
         <v>472</v>
       </c>
@@ -11131,9 +11456,9 @@
       <c r="R143" t="s">
         <v>27</v>
       </c>
-      <c r="S143" s="8"/>
-    </row>
-    <row r="144" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="S143" s="9"/>
+    </row>
+    <row r="144" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>463</v>
       </c>
@@ -11155,7 +11480,7 @@
       <c r="G144" t="s">
         <v>466</v>
       </c>
-      <c r="H144" s="7"/>
+      <c r="H144" s="8"/>
       <c r="I144" t="s">
         <v>472</v>
       </c>
@@ -11186,7 +11511,7 @@
       <c r="R144" t="s">
         <v>27</v>
       </c>
-      <c r="S144" s="8"/>
+      <c r="S144" s="9"/>
     </row>
     <row r="145" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
@@ -11210,7 +11535,7 @@
       <c r="G145" t="s">
         <v>466</v>
       </c>
-      <c r="H145" s="7"/>
+      <c r="H145" s="8"/>
       <c r="I145" t="s">
         <v>472</v>
       </c>
@@ -11241,7 +11566,7 @@
       <c r="R145" t="s">
         <v>27</v>
       </c>
-      <c r="S145" s="8"/>
+      <c r="S145" s="9"/>
     </row>
     <row r="146" spans="1:19" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
@@ -11265,7 +11590,7 @@
       <c r="G146" t="s">
         <v>481</v>
       </c>
-      <c r="H146" s="7" t="s">
+      <c r="H146" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I146" t="s">
@@ -11298,7 +11623,7 @@
       <c r="R146" t="s">
         <v>27</v>
       </c>
-      <c r="S146" s="8" t="s">
+      <c r="S146" s="9" t="s">
         <v>489</v>
       </c>
     </row>
@@ -11324,7 +11649,7 @@
       <c r="G147" t="s">
         <v>481</v>
       </c>
-      <c r="H147" s="7"/>
+      <c r="H147" s="8"/>
       <c r="I147" t="s">
         <v>487</v>
       </c>
@@ -11355,7 +11680,7 @@
       <c r="R147" t="s">
         <v>27</v>
       </c>
-      <c r="S147" s="8"/>
+      <c r="S147" s="9"/>
     </row>
     <row r="148" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
@@ -11379,7 +11704,7 @@
       <c r="G148" t="s">
         <v>481</v>
       </c>
-      <c r="H148" s="7"/>
+      <c r="H148" s="8"/>
       <c r="I148" t="s">
         <v>487</v>
       </c>
@@ -11410,7 +11735,7 @@
       <c r="R148" t="s">
         <v>27</v>
       </c>
-      <c r="S148" s="8"/>
+      <c r="S148" s="9"/>
     </row>
     <row r="149" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
@@ -11434,7 +11759,7 @@
       <c r="G149" t="s">
         <v>481</v>
       </c>
-      <c r="H149" s="7"/>
+      <c r="H149" s="8"/>
       <c r="I149" t="s">
         <v>487</v>
       </c>
@@ -11465,7 +11790,7 @@
       <c r="R149" t="s">
         <v>27</v>
       </c>
-      <c r="S149" s="8"/>
+      <c r="S149" s="9"/>
     </row>
     <row r="150" spans="1:19" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
@@ -11489,7 +11814,7 @@
       <c r="G150" t="s">
         <v>492</v>
       </c>
-      <c r="H150" s="7" t="s">
+      <c r="H150" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I150" t="s">
@@ -11522,7 +11847,7 @@
       <c r="R150" t="s">
         <v>27</v>
       </c>
-      <c r="S150" s="8" t="s">
+      <c r="S150" s="9" t="s">
         <v>500</v>
       </c>
     </row>
@@ -11548,7 +11873,7 @@
       <c r="G151" t="s">
         <v>492</v>
       </c>
-      <c r="H151" s="7"/>
+      <c r="H151" s="8"/>
       <c r="I151" t="s">
         <v>497</v>
       </c>
@@ -11579,7 +11904,7 @@
       <c r="R151" t="s">
         <v>27</v>
       </c>
-      <c r="S151" s="8"/>
+      <c r="S151" s="9"/>
     </row>
     <row r="152" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
@@ -11603,7 +11928,7 @@
       <c r="G152" t="s">
         <v>492</v>
       </c>
-      <c r="H152" s="7"/>
+      <c r="H152" s="8"/>
       <c r="I152" t="s">
         <v>497</v>
       </c>
@@ -11634,7 +11959,7 @@
       <c r="R152" t="s">
         <v>27</v>
       </c>
-      <c r="S152" s="8"/>
+      <c r="S152" s="9"/>
     </row>
     <row r="153" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
@@ -11658,7 +11983,7 @@
       <c r="G153" t="s">
         <v>492</v>
       </c>
-      <c r="H153" s="7"/>
+      <c r="H153" s="8"/>
       <c r="I153" t="s">
         <v>497</v>
       </c>
@@ -11689,22 +12014,60 @@
       <c r="R153" t="s">
         <v>27</v>
       </c>
-      <c r="S153" s="8"/>
+      <c r="S153" s="9"/>
     </row>
   </sheetData>
-  <mergeCells count="75">
-    <mergeCell ref="H142:H145"/>
-    <mergeCell ref="S142:S145"/>
-    <mergeCell ref="H146:H149"/>
-    <mergeCell ref="S146:S149"/>
-    <mergeCell ref="H150:H153"/>
-    <mergeCell ref="S150:S153"/>
-    <mergeCell ref="H130:H133"/>
-    <mergeCell ref="S130:S133"/>
-    <mergeCell ref="H134:H137"/>
-    <mergeCell ref="S134:S137"/>
-    <mergeCell ref="H138:H141"/>
-    <mergeCell ref="S138:S141"/>
+  <mergeCells count="78">
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="S126:S129"/>
+    <mergeCell ref="T126:T129"/>
+    <mergeCell ref="H86:H89"/>
+    <mergeCell ref="S86:S89"/>
+    <mergeCell ref="H70:H73"/>
+    <mergeCell ref="S70:S73"/>
+    <mergeCell ref="H74:H77"/>
+    <mergeCell ref="S74:S77"/>
+    <mergeCell ref="H78:H81"/>
+    <mergeCell ref="S78:S81"/>
+    <mergeCell ref="H62:H65"/>
+    <mergeCell ref="S62:S65"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="S66:S69"/>
+    <mergeCell ref="H82:H85"/>
+    <mergeCell ref="S82:S85"/>
+    <mergeCell ref="H50:H53"/>
+    <mergeCell ref="S50:S53"/>
+    <mergeCell ref="H54:H57"/>
+    <mergeCell ref="S54:S57"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="S58:S61"/>
+    <mergeCell ref="H38:H41"/>
+    <mergeCell ref="S38:S41"/>
+    <mergeCell ref="H42:H45"/>
+    <mergeCell ref="S42:S45"/>
+    <mergeCell ref="H46:H49"/>
+    <mergeCell ref="S46:S49"/>
+    <mergeCell ref="S26:S29"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="S30:S33"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="S34:S37"/>
+    <mergeCell ref="H102:H105"/>
+    <mergeCell ref="S102:S105"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="S2:S5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="S6:S9"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="S10:S13"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="L14:L17"/>
+    <mergeCell ref="S14:S17"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="S18:S21"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="S22:S25"/>
+    <mergeCell ref="H26:H29"/>
     <mergeCell ref="H118:H121"/>
     <mergeCell ref="S118:S121"/>
     <mergeCell ref="H90:H93"/>
@@ -11721,53 +12084,18 @@
     <mergeCell ref="S94:S97"/>
     <mergeCell ref="H98:H101"/>
     <mergeCell ref="S98:S101"/>
-    <mergeCell ref="H102:H105"/>
-    <mergeCell ref="S102:S105"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="S2:S5"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="S6:S9"/>
-    <mergeCell ref="H10:H13"/>
-    <mergeCell ref="S10:S13"/>
-    <mergeCell ref="H14:H17"/>
-    <mergeCell ref="L14:L17"/>
-    <mergeCell ref="S14:S17"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="S18:S21"/>
-    <mergeCell ref="H22:H25"/>
-    <mergeCell ref="S22:S25"/>
-    <mergeCell ref="H26:H29"/>
-    <mergeCell ref="S26:S29"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="S30:S33"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="S34:S37"/>
-    <mergeCell ref="H38:H41"/>
-    <mergeCell ref="S38:S41"/>
-    <mergeCell ref="H42:H45"/>
-    <mergeCell ref="S42:S45"/>
-    <mergeCell ref="H46:H49"/>
-    <mergeCell ref="S46:S49"/>
-    <mergeCell ref="H50:H53"/>
-    <mergeCell ref="S50:S53"/>
-    <mergeCell ref="H54:H57"/>
-    <mergeCell ref="S54:S57"/>
-    <mergeCell ref="H58:H61"/>
-    <mergeCell ref="S58:S61"/>
-    <mergeCell ref="H62:H65"/>
-    <mergeCell ref="S62:S65"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="S66:S69"/>
-    <mergeCell ref="H82:H85"/>
-    <mergeCell ref="S82:S85"/>
-    <mergeCell ref="H86:H89"/>
-    <mergeCell ref="S86:S89"/>
-    <mergeCell ref="H70:H73"/>
-    <mergeCell ref="S70:S73"/>
-    <mergeCell ref="H74:H77"/>
-    <mergeCell ref="S74:S77"/>
-    <mergeCell ref="H78:H81"/>
-    <mergeCell ref="S78:S81"/>
+    <mergeCell ref="H130:H133"/>
+    <mergeCell ref="S130:S133"/>
+    <mergeCell ref="H134:H137"/>
+    <mergeCell ref="S134:S137"/>
+    <mergeCell ref="H138:H141"/>
+    <mergeCell ref="S138:S141"/>
+    <mergeCell ref="H142:H145"/>
+    <mergeCell ref="S142:S145"/>
+    <mergeCell ref="H146:H149"/>
+    <mergeCell ref="S146:S149"/>
+    <mergeCell ref="H150:H153"/>
+    <mergeCell ref="S150:S153"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
03/06/25 : début de tests pour faire marcher varpart
</commit_message>
<xml_diff>
--- a/Resultats_modeles_coleo_2024.xlsx
+++ b/Resultats_modeles_coleo_2024.xlsx
@@ -12018,53 +12018,18 @@
     </row>
   </sheetData>
   <mergeCells count="78">
-    <mergeCell ref="H126:H129"/>
-    <mergeCell ref="S126:S129"/>
-    <mergeCell ref="T126:T129"/>
-    <mergeCell ref="H86:H89"/>
-    <mergeCell ref="S86:S89"/>
-    <mergeCell ref="H70:H73"/>
-    <mergeCell ref="S70:S73"/>
-    <mergeCell ref="H74:H77"/>
-    <mergeCell ref="S74:S77"/>
-    <mergeCell ref="H78:H81"/>
-    <mergeCell ref="S78:S81"/>
-    <mergeCell ref="H62:H65"/>
-    <mergeCell ref="S62:S65"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="S66:S69"/>
-    <mergeCell ref="H82:H85"/>
-    <mergeCell ref="S82:S85"/>
-    <mergeCell ref="H50:H53"/>
-    <mergeCell ref="S50:S53"/>
-    <mergeCell ref="H54:H57"/>
-    <mergeCell ref="S54:S57"/>
-    <mergeCell ref="H58:H61"/>
-    <mergeCell ref="S58:S61"/>
-    <mergeCell ref="H38:H41"/>
-    <mergeCell ref="S38:S41"/>
-    <mergeCell ref="H42:H45"/>
-    <mergeCell ref="S42:S45"/>
-    <mergeCell ref="H46:H49"/>
-    <mergeCell ref="S46:S49"/>
-    <mergeCell ref="S26:S29"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="S30:S33"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="S34:S37"/>
-    <mergeCell ref="H102:H105"/>
-    <mergeCell ref="S102:S105"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="S2:S5"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="S6:S9"/>
-    <mergeCell ref="H10:H13"/>
-    <mergeCell ref="S10:S13"/>
-    <mergeCell ref="H14:H17"/>
-    <mergeCell ref="L14:L17"/>
-    <mergeCell ref="S14:S17"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="S18:S21"/>
+    <mergeCell ref="H142:H145"/>
+    <mergeCell ref="S142:S145"/>
+    <mergeCell ref="H146:H149"/>
+    <mergeCell ref="S146:S149"/>
+    <mergeCell ref="H150:H153"/>
+    <mergeCell ref="S150:S153"/>
+    <mergeCell ref="H130:H133"/>
+    <mergeCell ref="S130:S133"/>
+    <mergeCell ref="H134:H137"/>
+    <mergeCell ref="S134:S137"/>
+    <mergeCell ref="H138:H141"/>
+    <mergeCell ref="S138:S141"/>
     <mergeCell ref="H22:H25"/>
     <mergeCell ref="S22:S25"/>
     <mergeCell ref="H26:H29"/>
@@ -12072,8 +12037,6 @@
     <mergeCell ref="S118:S121"/>
     <mergeCell ref="H90:H93"/>
     <mergeCell ref="S90:S93"/>
-    <mergeCell ref="H122:H125"/>
-    <mergeCell ref="S122:S125"/>
     <mergeCell ref="H106:H109"/>
     <mergeCell ref="S106:S109"/>
     <mergeCell ref="H110:H113"/>
@@ -12083,19 +12046,56 @@
     <mergeCell ref="H94:H97"/>
     <mergeCell ref="S94:S97"/>
     <mergeCell ref="H98:H101"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="L14:L17"/>
+    <mergeCell ref="S14:S17"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="S18:S21"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="S2:S5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="S6:S9"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="S10:S13"/>
+    <mergeCell ref="S26:S29"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="S30:S33"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="S34:S37"/>
+    <mergeCell ref="H38:H41"/>
+    <mergeCell ref="S38:S41"/>
+    <mergeCell ref="H42:H45"/>
+    <mergeCell ref="S42:S45"/>
+    <mergeCell ref="H46:H49"/>
+    <mergeCell ref="S46:S49"/>
+    <mergeCell ref="H50:H53"/>
+    <mergeCell ref="S50:S53"/>
+    <mergeCell ref="H54:H57"/>
+    <mergeCell ref="S54:S57"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="S58:S61"/>
+    <mergeCell ref="H62:H65"/>
+    <mergeCell ref="S62:S65"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="S66:S69"/>
+    <mergeCell ref="H82:H85"/>
+    <mergeCell ref="S82:S85"/>
+    <mergeCell ref="H70:H73"/>
+    <mergeCell ref="S70:S73"/>
+    <mergeCell ref="H74:H77"/>
+    <mergeCell ref="S74:S77"/>
+    <mergeCell ref="H78:H81"/>
+    <mergeCell ref="S78:S81"/>
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="S126:S129"/>
+    <mergeCell ref="T126:T129"/>
+    <mergeCell ref="H86:H89"/>
+    <mergeCell ref="S86:S89"/>
+    <mergeCell ref="H102:H105"/>
+    <mergeCell ref="S102:S105"/>
+    <mergeCell ref="H122:H125"/>
+    <mergeCell ref="S122:S125"/>
     <mergeCell ref="S98:S101"/>
-    <mergeCell ref="H130:H133"/>
-    <mergeCell ref="S130:S133"/>
-    <mergeCell ref="H134:H137"/>
-    <mergeCell ref="S134:S137"/>
-    <mergeCell ref="H138:H141"/>
-    <mergeCell ref="S138:S141"/>
-    <mergeCell ref="H142:H145"/>
-    <mergeCell ref="S142:S145"/>
-    <mergeCell ref="H146:H149"/>
-    <mergeCell ref="S146:S149"/>
-    <mergeCell ref="H150:H153"/>
-    <mergeCell ref="S150:S153"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
12-06-25 : suite nmds
</commit_message>
<xml_diff>
--- a/Resultats_modeles_coleo_2024.xlsx
+++ b/Resultats_modeles_coleo_2024.xlsx
@@ -4208,6 +4208,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4216,9 +4219,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4640,7 +4640,7 @@
       <c r="G2" t="s">
         <v>154</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I2" t="s">
@@ -4697,7 +4697,7 @@
       <c r="Z2" t="s">
         <v>173</v>
       </c>
-      <c r="AA2" s="10" t="s">
+      <c r="AA2" s="11" t="s">
         <v>45</v>
       </c>
     </row>
@@ -4723,7 +4723,7 @@
       <c r="G3" t="s">
         <v>154</v>
       </c>
-      <c r="H3" s="11"/>
+      <c r="H3" s="12"/>
       <c r="I3" t="s">
         <v>150</v>
       </c>
@@ -4778,7 +4778,7 @@
       <c r="Z3" t="s">
         <v>173</v>
       </c>
-      <c r="AA3" s="10"/>
+      <c r="AA3" s="11"/>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -4802,7 +4802,7 @@
       <c r="G4" t="s">
         <v>154</v>
       </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="12"/>
       <c r="I4" t="s">
         <v>150</v>
       </c>
@@ -4857,7 +4857,7 @@
       <c r="Z4" t="s">
         <v>173</v>
       </c>
-      <c r="AA4" s="10"/>
+      <c r="AA4" s="11"/>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -4881,7 +4881,7 @@
       <c r="G5" t="s">
         <v>154</v>
       </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="12"/>
       <c r="I5" t="s">
         <v>150</v>
       </c>
@@ -4936,7 +4936,7 @@
       <c r="Z5" t="s">
         <v>173</v>
       </c>
-      <c r="AA5" s="10"/>
+      <c r="AA5" s="11"/>
     </row>
     <row r="6" spans="1:29" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -4960,7 +4960,7 @@
       <c r="G6" t="s">
         <v>184</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I6" t="s">
@@ -5017,10 +5017,10 @@
       <c r="Z6" t="s">
         <v>182</v>
       </c>
-      <c r="AA6" s="10" t="s">
+      <c r="AA6" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="AB6" s="10" t="s">
+      <c r="AB6" s="11" t="s">
         <v>174</v>
       </c>
     </row>
@@ -5046,7 +5046,7 @@
       <c r="G7" t="s">
         <v>184</v>
       </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="12"/>
       <c r="I7" t="s">
         <v>189</v>
       </c>
@@ -5101,8 +5101,8 @@
       <c r="Z7" t="s">
         <v>182</v>
       </c>
-      <c r="AA7" s="10"/>
-      <c r="AB7" s="10"/>
+      <c r="AA7" s="11"/>
+      <c r="AB7" s="11"/>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -5126,7 +5126,7 @@
       <c r="G8" t="s">
         <v>184</v>
       </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="12"/>
       <c r="I8" t="s">
         <v>189</v>
       </c>
@@ -5181,8 +5181,8 @@
       <c r="Z8" t="s">
         <v>182</v>
       </c>
-      <c r="AA8" s="10"/>
-      <c r="AB8" s="10"/>
+      <c r="AA8" s="11"/>
+      <c r="AB8" s="11"/>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -5206,7 +5206,7 @@
       <c r="G9" t="s">
         <v>184</v>
       </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="12"/>
       <c r="I9" t="s">
         <v>189</v>
       </c>
@@ -5261,8 +5261,8 @@
       <c r="Z9" t="s">
         <v>182</v>
       </c>
-      <c r="AA9" s="10"/>
-      <c r="AB9" s="10"/>
+      <c r="AA9" s="11"/>
+      <c r="AB9" s="11"/>
     </row>
     <row r="10" spans="1:29" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -5286,7 +5286,7 @@
       <c r="G10" t="s">
         <v>194</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I10" t="s">
@@ -5343,10 +5343,10 @@
       <c r="Z10" t="s">
         <v>208</v>
       </c>
-      <c r="AA10" s="10" t="s">
+      <c r="AA10" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="AB10" s="10" t="s">
+      <c r="AB10" s="11" t="s">
         <v>209</v>
       </c>
     </row>
@@ -5372,7 +5372,7 @@
       <c r="G11" t="s">
         <v>194</v>
       </c>
-      <c r="H11" s="11"/>
+      <c r="H11" s="12"/>
       <c r="I11" t="s">
         <v>199</v>
       </c>
@@ -5427,8 +5427,8 @@
       <c r="Z11" t="s">
         <v>208</v>
       </c>
-      <c r="AA11" s="10"/>
-      <c r="AB11" s="10"/>
+      <c r="AA11" s="11"/>
+      <c r="AB11" s="11"/>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -5452,7 +5452,7 @@
       <c r="G12" t="s">
         <v>194</v>
       </c>
-      <c r="H12" s="11"/>
+      <c r="H12" s="12"/>
       <c r="I12" t="s">
         <v>199</v>
       </c>
@@ -5507,8 +5507,8 @@
       <c r="Z12" t="s">
         <v>208</v>
       </c>
-      <c r="AA12" s="10"/>
-      <c r="AB12" s="10"/>
+      <c r="AA12" s="11"/>
+      <c r="AB12" s="11"/>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -5532,7 +5532,7 @@
       <c r="G13" t="s">
         <v>194</v>
       </c>
-      <c r="H13" s="11"/>
+      <c r="H13" s="12"/>
       <c r="I13" t="s">
         <v>199</v>
       </c>
@@ -5587,8 +5587,8 @@
       <c r="Z13" t="s">
         <v>208</v>
       </c>
-      <c r="AA13" s="10"/>
-      <c r="AB13" s="10"/>
+      <c r="AA13" s="11"/>
+      <c r="AB13" s="11"/>
     </row>
     <row r="14" spans="1:29" ht="131.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -5612,7 +5612,7 @@
       <c r="G14" t="s">
         <v>211</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I14" t="s">
@@ -5624,7 +5624,7 @@
       <c r="K14" t="s">
         <v>20</v>
       </c>
-      <c r="L14" s="10" t="s">
+      <c r="L14" s="11" t="s">
         <v>44</v>
       </c>
       <c r="M14" t="s">
@@ -5669,7 +5669,7 @@
       <c r="Z14" t="s">
         <v>223</v>
       </c>
-      <c r="AA14" s="10" t="s">
+      <c r="AA14" s="11" t="s">
         <v>48</v>
       </c>
     </row>
@@ -5695,7 +5695,7 @@
       <c r="G15" t="s">
         <v>211</v>
       </c>
-      <c r="H15" s="11"/>
+      <c r="H15" s="12"/>
       <c r="I15" t="s">
         <v>213</v>
       </c>
@@ -5705,7 +5705,7 @@
       <c r="K15" t="s">
         <v>20</v>
       </c>
-      <c r="L15" s="10"/>
+      <c r="L15" s="11"/>
       <c r="M15" t="s">
         <v>15</v>
       </c>
@@ -5748,7 +5748,7 @@
       <c r="Z15" t="s">
         <v>223</v>
       </c>
-      <c r="AA15" s="10"/>
+      <c r="AA15" s="11"/>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -5772,7 +5772,7 @@
       <c r="G16" t="s">
         <v>211</v>
       </c>
-      <c r="H16" s="11"/>
+      <c r="H16" s="12"/>
       <c r="I16" t="s">
         <v>213</v>
       </c>
@@ -5782,7 +5782,7 @@
       <c r="K16" t="s">
         <v>20</v>
       </c>
-      <c r="L16" s="10"/>
+      <c r="L16" s="11"/>
       <c r="M16" t="s">
         <v>15</v>
       </c>
@@ -5825,7 +5825,7 @@
       <c r="Z16" t="s">
         <v>223</v>
       </c>
-      <c r="AA16" s="10"/>
+      <c r="AA16" s="11"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
@@ -5849,7 +5849,7 @@
       <c r="G17" t="s">
         <v>211</v>
       </c>
-      <c r="H17" s="11"/>
+      <c r="H17" s="12"/>
       <c r="I17" t="s">
         <v>213</v>
       </c>
@@ -5859,7 +5859,7 @@
       <c r="K17" t="s">
         <v>20</v>
       </c>
-      <c r="L17" s="10"/>
+      <c r="L17" s="11"/>
       <c r="M17" t="s">
         <v>15</v>
       </c>
@@ -5902,7 +5902,7 @@
       <c r="Z17" t="s">
         <v>223</v>
       </c>
-      <c r="AA17" s="10"/>
+      <c r="AA17" s="11"/>
     </row>
     <row r="18" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
@@ -5926,7 +5926,7 @@
       <c r="G18" t="s">
         <v>225</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I18" t="s">
@@ -5983,10 +5983,10 @@
       <c r="Z18" t="s">
         <v>240</v>
       </c>
-      <c r="AA18" s="10" t="s">
+      <c r="AA18" s="11" t="s">
         <v>233</v>
       </c>
-      <c r="AB18" s="10" t="s">
+      <c r="AB18" s="11" t="s">
         <v>241</v>
       </c>
     </row>
@@ -6012,7 +6012,7 @@
       <c r="G19" t="s">
         <v>225</v>
       </c>
-      <c r="H19" s="11"/>
+      <c r="H19" s="12"/>
       <c r="I19" t="s">
         <v>230</v>
       </c>
@@ -6067,8 +6067,8 @@
       <c r="Z19" t="s">
         <v>240</v>
       </c>
-      <c r="AA19" s="10"/>
-      <c r="AB19" s="10"/>
+      <c r="AA19" s="11"/>
+      <c r="AB19" s="11"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
@@ -6092,7 +6092,7 @@
       <c r="G20" t="s">
         <v>225</v>
       </c>
-      <c r="H20" s="11"/>
+      <c r="H20" s="12"/>
       <c r="I20" t="s">
         <v>230</v>
       </c>
@@ -6147,8 +6147,8 @@
       <c r="Z20" t="s">
         <v>240</v>
       </c>
-      <c r="AA20" s="10"/>
-      <c r="AB20" s="10"/>
+      <c r="AA20" s="11"/>
+      <c r="AB20" s="11"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
@@ -6172,7 +6172,7 @@
       <c r="G21" t="s">
         <v>225</v>
       </c>
-      <c r="H21" s="11"/>
+      <c r="H21" s="12"/>
       <c r="I21" t="s">
         <v>230</v>
       </c>
@@ -6227,8 +6227,8 @@
       <c r="Z21" t="s">
         <v>240</v>
       </c>
-      <c r="AA21" s="10"/>
-      <c r="AB21" s="10"/>
+      <c r="AA21" s="11"/>
+      <c r="AB21" s="11"/>
     </row>
     <row r="22" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
@@ -6252,7 +6252,7 @@
       <c r="G22" t="s">
         <v>243</v>
       </c>
-      <c r="H22" s="11" t="s">
+      <c r="H22" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I22" t="s">
@@ -6297,7 +6297,7 @@
       <c r="Z22" t="s">
         <v>258</v>
       </c>
-      <c r="AA22" s="10" t="s">
+      <c r="AA22" s="11" t="s">
         <v>52</v>
       </c>
     </row>
@@ -6323,7 +6323,7 @@
       <c r="G23" t="s">
         <v>243</v>
       </c>
-      <c r="H23" s="11"/>
+      <c r="H23" s="12"/>
       <c r="I23" t="s">
         <v>249</v>
       </c>
@@ -6366,7 +6366,7 @@
       <c r="Z23" t="s">
         <v>258</v>
       </c>
-      <c r="AA23" s="10"/>
+      <c r="AA23" s="11"/>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
@@ -6390,7 +6390,7 @@
       <c r="G24" t="s">
         <v>243</v>
       </c>
-      <c r="H24" s="11"/>
+      <c r="H24" s="12"/>
       <c r="I24" t="s">
         <v>249</v>
       </c>
@@ -6433,7 +6433,7 @@
       <c r="Z24" t="s">
         <v>258</v>
       </c>
-      <c r="AA24" s="10"/>
+      <c r="AA24" s="11"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
@@ -6457,7 +6457,7 @@
       <c r="G25" t="s">
         <v>243</v>
       </c>
-      <c r="H25" s="11"/>
+      <c r="H25" s="12"/>
       <c r="I25" t="s">
         <v>249</v>
       </c>
@@ -6500,7 +6500,7 @@
       <c r="Z25" t="s">
         <v>258</v>
       </c>
-      <c r="AA25" s="10"/>
+      <c r="AA25" s="11"/>
     </row>
     <row r="26" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
@@ -6524,7 +6524,7 @@
       <c r="G26" t="s">
         <v>261</v>
       </c>
-      <c r="H26" s="11" t="s">
+      <c r="H26" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I26" t="s">
@@ -6581,10 +6581,10 @@
       <c r="Z26" t="s">
         <v>278</v>
       </c>
-      <c r="AA26" s="10" t="s">
+      <c r="AA26" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="AB26" s="10" t="s">
+      <c r="AB26" s="11" t="s">
         <v>279</v>
       </c>
     </row>
@@ -6610,7 +6610,7 @@
       <c r="G27" t="s">
         <v>261</v>
       </c>
-      <c r="H27" s="11"/>
+      <c r="H27" s="12"/>
       <c r="I27" t="s">
         <v>266</v>
       </c>
@@ -6665,8 +6665,8 @@
       <c r="Z27" t="s">
         <v>278</v>
       </c>
-      <c r="AA27" s="10"/>
-      <c r="AB27" s="10"/>
+      <c r="AA27" s="11"/>
+      <c r="AB27" s="11"/>
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
@@ -6690,7 +6690,7 @@
       <c r="G28" t="s">
         <v>261</v>
       </c>
-      <c r="H28" s="11"/>
+      <c r="H28" s="12"/>
       <c r="I28" t="s">
         <v>266</v>
       </c>
@@ -6745,8 +6745,8 @@
       <c r="Z28" t="s">
         <v>278</v>
       </c>
-      <c r="AA28" s="10"/>
-      <c r="AB28" s="10"/>
+      <c r="AA28" s="11"/>
+      <c r="AB28" s="11"/>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
@@ -6770,7 +6770,7 @@
       <c r="G29" t="s">
         <v>261</v>
       </c>
-      <c r="H29" s="11"/>
+      <c r="H29" s="12"/>
       <c r="I29" t="s">
         <v>266</v>
       </c>
@@ -6825,8 +6825,8 @@
       <c r="Z29" t="s">
         <v>278</v>
       </c>
-      <c r="AA29" s="10"/>
-      <c r="AB29" s="10"/>
+      <c r="AA29" s="11"/>
+      <c r="AB29" s="11"/>
     </row>
     <row r="30" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
@@ -6850,7 +6850,7 @@
       <c r="G30" t="s">
         <v>282</v>
       </c>
-      <c r="H30" s="11" t="s">
+      <c r="H30" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I30" t="s">
@@ -6907,10 +6907,10 @@
       <c r="Z30" t="s">
         <v>298</v>
       </c>
-      <c r="AA30" s="10" t="s">
+      <c r="AA30" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="AB30" s="10" t="s">
+      <c r="AB30" s="11" t="s">
         <v>299</v>
       </c>
     </row>
@@ -6936,7 +6936,7 @@
       <c r="G31" t="s">
         <v>282</v>
       </c>
-      <c r="H31" s="11"/>
+      <c r="H31" s="12"/>
       <c r="I31" t="s">
         <v>287</v>
       </c>
@@ -6991,8 +6991,8 @@
       <c r="Z31" t="s">
         <v>298</v>
       </c>
-      <c r="AA31" s="10"/>
-      <c r="AB31" s="10"/>
+      <c r="AA31" s="11"/>
+      <c r="AB31" s="11"/>
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
@@ -7016,7 +7016,7 @@
       <c r="G32" t="s">
         <v>282</v>
       </c>
-      <c r="H32" s="11"/>
+      <c r="H32" s="12"/>
       <c r="I32" t="s">
         <v>287</v>
       </c>
@@ -7071,8 +7071,8 @@
       <c r="Z32" t="s">
         <v>298</v>
       </c>
-      <c r="AA32" s="10"/>
-      <c r="AB32" s="10"/>
+      <c r="AA32" s="11"/>
+      <c r="AB32" s="11"/>
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
@@ -7096,7 +7096,7 @@
       <c r="G33" t="s">
         <v>282</v>
       </c>
-      <c r="H33" s="11"/>
+      <c r="H33" s="12"/>
       <c r="I33" t="s">
         <v>287</v>
       </c>
@@ -7151,8 +7151,8 @@
       <c r="Z33" t="s">
         <v>298</v>
       </c>
-      <c r="AA33" s="10"/>
-      <c r="AB33" s="10"/>
+      <c r="AA33" s="11"/>
+      <c r="AB33" s="11"/>
     </row>
     <row r="34" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
@@ -7176,7 +7176,7 @@
       <c r="G34" t="s">
         <v>302</v>
       </c>
-      <c r="H34" s="11" t="s">
+      <c r="H34" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I34" t="s">
@@ -7221,7 +7221,7 @@
       <c r="Z34" t="s">
         <v>316</v>
       </c>
-      <c r="AA34" s="10" t="s">
+      <c r="AA34" s="11" t="s">
         <v>308</v>
       </c>
     </row>
@@ -7247,7 +7247,7 @@
       <c r="G35" t="s">
         <v>302</v>
       </c>
-      <c r="H35" s="11"/>
+      <c r="H35" s="12"/>
       <c r="I35" t="s">
         <v>306</v>
       </c>
@@ -7290,7 +7290,7 @@
       <c r="Z35" t="s">
         <v>316</v>
       </c>
-      <c r="AA35" s="10"/>
+      <c r="AA35" s="11"/>
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
@@ -7314,7 +7314,7 @@
       <c r="G36" t="s">
         <v>302</v>
       </c>
-      <c r="H36" s="11"/>
+      <c r="H36" s="12"/>
       <c r="I36" t="s">
         <v>306</v>
       </c>
@@ -7357,7 +7357,7 @@
       <c r="Z36" t="s">
         <v>316</v>
       </c>
-      <c r="AA36" s="10"/>
+      <c r="AA36" s="11"/>
     </row>
     <row r="37" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
@@ -7381,7 +7381,7 @@
       <c r="G37" t="s">
         <v>302</v>
       </c>
-      <c r="H37" s="11"/>
+      <c r="H37" s="12"/>
       <c r="I37" t="s">
         <v>306</v>
       </c>
@@ -7424,7 +7424,7 @@
       <c r="Z37" t="s">
         <v>316</v>
       </c>
-      <c r="AA37" s="10"/>
+      <c r="AA37" s="11"/>
     </row>
     <row r="38" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
@@ -7448,7 +7448,7 @@
       <c r="G38" t="s">
         <v>320</v>
       </c>
-      <c r="H38" s="11" t="s">
+      <c r="H38" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I38" t="s">
@@ -7493,7 +7493,7 @@
       <c r="Z38" t="s">
         <v>332</v>
       </c>
-      <c r="AA38" s="10" t="s">
+      <c r="AA38" s="11" t="s">
         <v>317</v>
       </c>
     </row>
@@ -7519,7 +7519,7 @@
       <c r="G39" t="s">
         <v>320</v>
       </c>
-      <c r="H39" s="11"/>
+      <c r="H39" s="12"/>
       <c r="I39" t="s">
         <v>324</v>
       </c>
@@ -7562,7 +7562,7 @@
       <c r="Z39" t="s">
         <v>332</v>
       </c>
-      <c r="AA39" s="10"/>
+      <c r="AA39" s="11"/>
     </row>
     <row r="40" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
@@ -7586,7 +7586,7 @@
       <c r="G40" t="s">
         <v>320</v>
       </c>
-      <c r="H40" s="11"/>
+      <c r="H40" s="12"/>
       <c r="I40" t="s">
         <v>324</v>
       </c>
@@ -7629,7 +7629,7 @@
       <c r="Z40" t="s">
         <v>332</v>
       </c>
-      <c r="AA40" s="10"/>
+      <c r="AA40" s="11"/>
     </row>
     <row r="41" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
@@ -7653,7 +7653,7 @@
       <c r="G41" t="s">
         <v>320</v>
       </c>
-      <c r="H41" s="11"/>
+      <c r="H41" s="12"/>
       <c r="I41" t="s">
         <v>324</v>
       </c>
@@ -7696,7 +7696,7 @@
       <c r="Z41" t="s">
         <v>332</v>
       </c>
-      <c r="AA41" s="10"/>
+      <c r="AA41" s="11"/>
     </row>
     <row r="42" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
@@ -7720,7 +7720,7 @@
       <c r="G42" t="s">
         <v>334</v>
       </c>
-      <c r="H42" s="11" t="s">
+      <c r="H42" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I42" t="s">
@@ -7765,7 +7765,7 @@
       <c r="Z42" t="s">
         <v>348</v>
       </c>
-      <c r="AA42" s="10" t="s">
+      <c r="AA42" s="11" t="s">
         <v>340</v>
       </c>
     </row>
@@ -7791,7 +7791,7 @@
       <c r="G43" t="s">
         <v>334</v>
       </c>
-      <c r="H43" s="11"/>
+      <c r="H43" s="12"/>
       <c r="I43" t="s">
         <v>338</v>
       </c>
@@ -7834,7 +7834,7 @@
       <c r="Z43" t="s">
         <v>348</v>
       </c>
-      <c r="AA43" s="10"/>
+      <c r="AA43" s="11"/>
     </row>
     <row r="44" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
@@ -7858,7 +7858,7 @@
       <c r="G44" t="s">
         <v>334</v>
       </c>
-      <c r="H44" s="11"/>
+      <c r="H44" s="12"/>
       <c r="I44" t="s">
         <v>338</v>
       </c>
@@ -7901,7 +7901,7 @@
       <c r="Z44" t="s">
         <v>348</v>
       </c>
-      <c r="AA44" s="10"/>
+      <c r="AA44" s="11"/>
     </row>
     <row r="45" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
@@ -7925,7 +7925,7 @@
       <c r="G45" t="s">
         <v>334</v>
       </c>
-      <c r="H45" s="11"/>
+      <c r="H45" s="12"/>
       <c r="I45" t="s">
         <v>338</v>
       </c>
@@ -7968,7 +7968,7 @@
       <c r="Z45" t="s">
         <v>348</v>
       </c>
-      <c r="AA45" s="10"/>
+      <c r="AA45" s="11"/>
     </row>
     <row r="46" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
@@ -7992,7 +7992,7 @@
       <c r="G46" t="s">
         <v>350</v>
       </c>
-      <c r="H46" s="11" t="s">
+      <c r="H46" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I46" t="s">
@@ -8037,7 +8037,7 @@
       <c r="Z46" t="s">
         <v>364</v>
       </c>
-      <c r="AA46" s="10" t="s">
+      <c r="AA46" s="11" t="s">
         <v>357</v>
       </c>
     </row>
@@ -8063,7 +8063,7 @@
       <c r="G47" t="s">
         <v>350</v>
       </c>
-      <c r="H47" s="11"/>
+      <c r="H47" s="12"/>
       <c r="I47" t="s">
         <v>355</v>
       </c>
@@ -8106,7 +8106,7 @@
       <c r="Z47" t="s">
         <v>364</v>
       </c>
-      <c r="AA47" s="10"/>
+      <c r="AA47" s="11"/>
     </row>
     <row r="48" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
@@ -8130,7 +8130,7 @@
       <c r="G48" t="s">
         <v>350</v>
       </c>
-      <c r="H48" s="11"/>
+      <c r="H48" s="12"/>
       <c r="I48" t="s">
         <v>355</v>
       </c>
@@ -8173,7 +8173,7 @@
       <c r="Z48" t="s">
         <v>364</v>
       </c>
-      <c r="AA48" s="10"/>
+      <c r="AA48" s="11"/>
     </row>
     <row r="49" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
@@ -8197,7 +8197,7 @@
       <c r="G49" t="s">
         <v>350</v>
       </c>
-      <c r="H49" s="11"/>
+      <c r="H49" s="12"/>
       <c r="I49" t="s">
         <v>355</v>
       </c>
@@ -8240,7 +8240,7 @@
       <c r="Z49" t="s">
         <v>364</v>
       </c>
-      <c r="AA49" s="10"/>
+      <c r="AA49" s="11"/>
     </row>
     <row r="50" spans="1:28" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
@@ -8264,7 +8264,7 @@
       <c r="G50" t="s">
         <v>366</v>
       </c>
-      <c r="H50" s="11" t="s">
+      <c r="H50" s="12" t="s">
         <v>371</v>
       </c>
       <c r="I50" t="s">
@@ -8321,7 +8321,7 @@
       <c r="Z50" t="s">
         <v>384</v>
       </c>
-      <c r="AA50" s="10" t="s">
+      <c r="AA50" s="11" t="s">
         <v>377</v>
       </c>
     </row>
@@ -8347,7 +8347,7 @@
       <c r="G51" t="s">
         <v>366</v>
       </c>
-      <c r="H51" s="11"/>
+      <c r="H51" s="12"/>
       <c r="I51" t="s">
         <v>373</v>
       </c>
@@ -8402,7 +8402,7 @@
       <c r="Z51" t="s">
         <v>384</v>
       </c>
-      <c r="AA51" s="10"/>
+      <c r="AA51" s="11"/>
     </row>
     <row r="52" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
@@ -8426,7 +8426,7 @@
       <c r="G52" t="s">
         <v>366</v>
       </c>
-      <c r="H52" s="11"/>
+      <c r="H52" s="12"/>
       <c r="I52" t="s">
         <v>373</v>
       </c>
@@ -8481,7 +8481,7 @@
       <c r="Z52" t="s">
         <v>384</v>
       </c>
-      <c r="AA52" s="10"/>
+      <c r="AA52" s="11"/>
     </row>
     <row r="53" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
@@ -8505,7 +8505,7 @@
       <c r="G53" t="s">
         <v>366</v>
       </c>
-      <c r="H53" s="11"/>
+      <c r="H53" s="12"/>
       <c r="I53" t="s">
         <v>373</v>
       </c>
@@ -8560,7 +8560,7 @@
       <c r="Z53" t="s">
         <v>384</v>
       </c>
-      <c r="AA53" s="10"/>
+      <c r="AA53" s="11"/>
     </row>
     <row r="54" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
@@ -8584,7 +8584,7 @@
       <c r="G54" t="s">
         <v>387</v>
       </c>
-      <c r="H54" s="11" t="s">
+      <c r="H54" s="12" t="s">
         <v>68</v>
       </c>
       <c r="I54" t="s">
@@ -8629,10 +8629,10 @@
       <c r="Z54" t="s">
         <v>400</v>
       </c>
-      <c r="AA54" s="10" t="s">
+      <c r="AA54" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="AB54" s="10" t="s">
+      <c r="AB54" s="11" t="s">
         <v>401</v>
       </c>
     </row>
@@ -8658,7 +8658,7 @@
       <c r="G55" t="s">
         <v>387</v>
       </c>
-      <c r="H55" s="11"/>
+      <c r="H55" s="12"/>
       <c r="I55" t="s">
         <v>394</v>
       </c>
@@ -8701,8 +8701,8 @@
       <c r="Z55" t="s">
         <v>400</v>
       </c>
-      <c r="AA55" s="10"/>
-      <c r="AB55" s="10"/>
+      <c r="AA55" s="11"/>
+      <c r="AB55" s="11"/>
     </row>
     <row r="56" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
@@ -8726,7 +8726,7 @@
       <c r="G56" t="s">
         <v>387</v>
       </c>
-      <c r="H56" s="11"/>
+      <c r="H56" s="12"/>
       <c r="I56" t="s">
         <v>394</v>
       </c>
@@ -8769,8 +8769,8 @@
       <c r="Z56" t="s">
         <v>400</v>
       </c>
-      <c r="AA56" s="10"/>
-      <c r="AB56" s="10"/>
+      <c r="AA56" s="11"/>
+      <c r="AB56" s="11"/>
     </row>
     <row r="57" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
@@ -8794,7 +8794,7 @@
       <c r="G57" t="s">
         <v>387</v>
       </c>
-      <c r="H57" s="11"/>
+      <c r="H57" s="12"/>
       <c r="I57" t="s">
         <v>394</v>
       </c>
@@ -8837,8 +8837,8 @@
       <c r="Z57" t="s">
         <v>400</v>
       </c>
-      <c r="AA57" s="10"/>
-      <c r="AB57" s="10"/>
+      <c r="AA57" s="11"/>
+      <c r="AB57" s="11"/>
     </row>
     <row r="58" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
@@ -8862,7 +8862,7 @@
       <c r="G58" t="s">
         <v>404</v>
       </c>
-      <c r="H58" s="11" t="s">
+      <c r="H58" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I58" t="s">
@@ -8919,7 +8919,7 @@
       <c r="Z58" t="s">
         <v>419</v>
       </c>
-      <c r="AA58" s="10" t="s">
+      <c r="AA58" s="11" t="s">
         <v>72</v>
       </c>
     </row>
@@ -8945,7 +8945,7 @@
       <c r="G59" t="s">
         <v>404</v>
       </c>
-      <c r="H59" s="11"/>
+      <c r="H59" s="12"/>
       <c r="I59" t="s">
         <v>409</v>
       </c>
@@ -9000,7 +9000,7 @@
       <c r="Z59" t="s">
         <v>419</v>
       </c>
-      <c r="AA59" s="10"/>
+      <c r="AA59" s="11"/>
     </row>
     <row r="60" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
@@ -9024,7 +9024,7 @@
       <c r="G60" t="s">
         <v>404</v>
       </c>
-      <c r="H60" s="11"/>
+      <c r="H60" s="12"/>
       <c r="I60" t="s">
         <v>409</v>
       </c>
@@ -9079,7 +9079,7 @@
       <c r="Z60" t="s">
         <v>419</v>
       </c>
-      <c r="AA60" s="10"/>
+      <c r="AA60" s="11"/>
     </row>
     <row r="61" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
@@ -9103,7 +9103,7 @@
       <c r="G61" t="s">
         <v>404</v>
       </c>
-      <c r="H61" s="11"/>
+      <c r="H61" s="12"/>
       <c r="I61" t="s">
         <v>409</v>
       </c>
@@ -9158,7 +9158,7 @@
       <c r="Z61" t="s">
         <v>419</v>
       </c>
-      <c r="AA61" s="10"/>
+      <c r="AA61" s="11"/>
     </row>
     <row r="62" spans="1:28" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
@@ -9182,7 +9182,7 @@
       <c r="G62" t="s">
         <v>75</v>
       </c>
-      <c r="H62" s="11" t="s">
+      <c r="H62" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I62" t="s">
@@ -9239,10 +9239,10 @@
       <c r="Z62" t="s">
         <v>428</v>
       </c>
-      <c r="AA62" s="10" t="s">
+      <c r="AA62" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="AB62" s="10" t="s">
+      <c r="AB62" s="11" t="s">
         <v>420</v>
       </c>
     </row>
@@ -9268,7 +9268,7 @@
       <c r="G63" t="s">
         <v>75</v>
       </c>
-      <c r="H63" s="11"/>
+      <c r="H63" s="12"/>
       <c r="I63" t="s">
         <v>80</v>
       </c>
@@ -9323,8 +9323,8 @@
       <c r="Z63" t="s">
         <v>428</v>
       </c>
-      <c r="AA63" s="10"/>
-      <c r="AB63" s="10"/>
+      <c r="AA63" s="11"/>
+      <c r="AB63" s="11"/>
     </row>
     <row r="64" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
@@ -9348,7 +9348,7 @@
       <c r="G64" t="s">
         <v>75</v>
       </c>
-      <c r="H64" s="11"/>
+      <c r="H64" s="12"/>
       <c r="I64" t="s">
         <v>80</v>
       </c>
@@ -9403,8 +9403,8 @@
       <c r="Z64" t="s">
         <v>428</v>
       </c>
-      <c r="AA64" s="10"/>
-      <c r="AB64" s="10"/>
+      <c r="AA64" s="11"/>
+      <c r="AB64" s="11"/>
     </row>
     <row r="65" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
@@ -9428,7 +9428,7 @@
       <c r="G65" t="s">
         <v>75</v>
       </c>
-      <c r="H65" s="11"/>
+      <c r="H65" s="12"/>
       <c r="I65" t="s">
         <v>80</v>
       </c>
@@ -9483,8 +9483,8 @@
       <c r="Z65" t="s">
         <v>428</v>
       </c>
-      <c r="AA65" s="10"/>
-      <c r="AB65" s="10"/>
+      <c r="AA65" s="11"/>
+      <c r="AB65" s="11"/>
     </row>
     <row r="66" spans="1:28" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
@@ -9508,7 +9508,7 @@
       <c r="G66" t="s">
         <v>430</v>
       </c>
-      <c r="H66" s="11" t="s">
+      <c r="H66" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I66" t="s">
@@ -9565,7 +9565,7 @@
       <c r="Z66" t="s">
         <v>444</v>
       </c>
-      <c r="AA66" s="10" t="s">
+      <c r="AA66" s="11" t="s">
         <v>436</v>
       </c>
     </row>
@@ -9591,7 +9591,7 @@
       <c r="G67" t="s">
         <v>430</v>
       </c>
-      <c r="H67" s="11"/>
+      <c r="H67" s="12"/>
       <c r="I67" t="s">
         <v>434</v>
       </c>
@@ -9646,7 +9646,7 @@
       <c r="Z67" t="s">
         <v>444</v>
       </c>
-      <c r="AA67" s="10"/>
+      <c r="AA67" s="11"/>
     </row>
     <row r="68" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
@@ -9670,7 +9670,7 @@
       <c r="G68" t="s">
         <v>430</v>
       </c>
-      <c r="H68" s="11"/>
+      <c r="H68" s="12"/>
       <c r="I68" t="s">
         <v>434</v>
       </c>
@@ -9725,7 +9725,7 @@
       <c r="Z68" t="s">
         <v>444</v>
       </c>
-      <c r="AA68" s="10"/>
+      <c r="AA68" s="11"/>
     </row>
     <row r="69" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
@@ -9749,7 +9749,7 @@
       <c r="G69" t="s">
         <v>430</v>
       </c>
-      <c r="H69" s="11"/>
+      <c r="H69" s="12"/>
       <c r="I69" t="s">
         <v>434</v>
       </c>
@@ -9804,7 +9804,7 @@
       <c r="Z69" t="s">
         <v>444</v>
       </c>
-      <c r="AA69" s="10"/>
+      <c r="AA69" s="11"/>
     </row>
     <row r="70" spans="1:28" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
@@ -9828,7 +9828,7 @@
       <c r="G70" t="s">
         <v>447</v>
       </c>
-      <c r="H70" s="11" t="s">
+      <c r="H70" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I70" t="s">
@@ -9885,7 +9885,7 @@
       <c r="Z70" t="s">
         <v>463</v>
       </c>
-      <c r="AA70" s="10" t="s">
+      <c r="AA70" s="11" t="s">
         <v>456</v>
       </c>
     </row>
@@ -9911,7 +9911,7 @@
       <c r="G71" t="s">
         <v>447</v>
       </c>
-      <c r="H71" s="11"/>
+      <c r="H71" s="12"/>
       <c r="I71" t="s">
         <v>452</v>
       </c>
@@ -9966,7 +9966,7 @@
       <c r="Z71" t="s">
         <v>463</v>
       </c>
-      <c r="AA71" s="10"/>
+      <c r="AA71" s="11"/>
     </row>
     <row r="72" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
@@ -9990,7 +9990,7 @@
       <c r="G72" t="s">
         <v>447</v>
       </c>
-      <c r="H72" s="11"/>
+      <c r="H72" s="12"/>
       <c r="I72" t="s">
         <v>452</v>
       </c>
@@ -10045,7 +10045,7 @@
       <c r="Z72" t="s">
         <v>463</v>
       </c>
-      <c r="AA72" s="10"/>
+      <c r="AA72" s="11"/>
     </row>
     <row r="73" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
@@ -10069,7 +10069,7 @@
       <c r="G73" t="s">
         <v>447</v>
       </c>
-      <c r="H73" s="11"/>
+      <c r="H73" s="12"/>
       <c r="I73" t="s">
         <v>452</v>
       </c>
@@ -10124,7 +10124,7 @@
       <c r="Z73" t="s">
         <v>463</v>
       </c>
-      <c r="AA73" s="10"/>
+      <c r="AA73" s="11"/>
     </row>
     <row r="74" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
@@ -10148,7 +10148,7 @@
       <c r="G74" t="s">
         <v>465</v>
       </c>
-      <c r="H74" s="11" t="s">
+      <c r="H74" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I74" t="s">
@@ -10193,7 +10193,7 @@
       <c r="Z74" t="s">
         <v>479</v>
       </c>
-      <c r="AA74" s="10" t="s">
+      <c r="AA74" s="11" t="s">
         <v>472</v>
       </c>
     </row>
@@ -10219,7 +10219,7 @@
       <c r="G75" t="s">
         <v>465</v>
       </c>
-      <c r="H75" s="11"/>
+      <c r="H75" s="12"/>
       <c r="I75" t="s">
         <v>470</v>
       </c>
@@ -10262,7 +10262,7 @@
       <c r="Z75" t="s">
         <v>479</v>
       </c>
-      <c r="AA75" s="10"/>
+      <c r="AA75" s="11"/>
     </row>
     <row r="76" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
@@ -10286,7 +10286,7 @@
       <c r="G76" t="s">
         <v>465</v>
       </c>
-      <c r="H76" s="11"/>
+      <c r="H76" s="12"/>
       <c r="I76" t="s">
         <v>470</v>
       </c>
@@ -10329,7 +10329,7 @@
       <c r="Z76" t="s">
         <v>479</v>
       </c>
-      <c r="AA76" s="10"/>
+      <c r="AA76" s="11"/>
     </row>
     <row r="77" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
@@ -10353,7 +10353,7 @@
       <c r="G77" t="s">
         <v>465</v>
       </c>
-      <c r="H77" s="11"/>
+      <c r="H77" s="12"/>
       <c r="I77" t="s">
         <v>470</v>
       </c>
@@ -10396,7 +10396,7 @@
       <c r="Z77" t="s">
         <v>479</v>
       </c>
-      <c r="AA77" s="10"/>
+      <c r="AA77" s="11"/>
     </row>
     <row r="78" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
@@ -10420,7 +10420,7 @@
       <c r="G78" t="s">
         <v>482</v>
       </c>
-      <c r="H78" s="11" t="s">
+      <c r="H78" s="12" t="s">
         <v>488</v>
       </c>
       <c r="I78" t="s">
@@ -10465,7 +10465,7 @@
       <c r="Z78" t="s">
         <v>498</v>
       </c>
-      <c r="AA78" s="10" t="s">
+      <c r="AA78" s="11" t="s">
         <v>480</v>
       </c>
     </row>
@@ -10491,7 +10491,7 @@
       <c r="G79" t="s">
         <v>482</v>
       </c>
-      <c r="H79" s="11"/>
+      <c r="H79" s="12"/>
       <c r="I79" t="s">
         <v>489</v>
       </c>
@@ -10534,7 +10534,7 @@
       <c r="Z79" t="s">
         <v>498</v>
       </c>
-      <c r="AA79" s="10"/>
+      <c r="AA79" s="11"/>
     </row>
     <row r="80" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
@@ -10558,7 +10558,7 @@
       <c r="G80" t="s">
         <v>482</v>
       </c>
-      <c r="H80" s="11"/>
+      <c r="H80" s="12"/>
       <c r="I80" t="s">
         <v>489</v>
       </c>
@@ -10601,7 +10601,7 @@
       <c r="Z80" t="s">
         <v>498</v>
       </c>
-      <c r="AA80" s="10"/>
+      <c r="AA80" s="11"/>
     </row>
     <row r="81" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
@@ -10625,7 +10625,7 @@
       <c r="G81" t="s">
         <v>482</v>
       </c>
-      <c r="H81" s="11"/>
+      <c r="H81" s="12"/>
       <c r="I81" t="s">
         <v>489</v>
       </c>
@@ -10668,7 +10668,7 @@
       <c r="Z81" t="s">
         <v>498</v>
       </c>
-      <c r="AA81" s="10"/>
+      <c r="AA81" s="11"/>
     </row>
     <row r="82" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
@@ -10692,7 +10692,7 @@
       <c r="G82" t="s">
         <v>500</v>
       </c>
-      <c r="H82" s="11" t="s">
+      <c r="H82" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I82" t="s">
@@ -10737,7 +10737,7 @@
       <c r="Z82" t="s">
         <v>513</v>
       </c>
-      <c r="AA82" s="10" t="s">
+      <c r="AA82" s="11" t="s">
         <v>90</v>
       </c>
     </row>
@@ -10763,7 +10763,7 @@
       <c r="G83" t="s">
         <v>500</v>
       </c>
-      <c r="H83" s="11"/>
+      <c r="H83" s="12"/>
       <c r="I83" t="s">
         <v>505</v>
       </c>
@@ -10806,7 +10806,7 @@
       <c r="Z83" t="s">
         <v>513</v>
       </c>
-      <c r="AA83" s="10"/>
+      <c r="AA83" s="11"/>
     </row>
     <row r="84" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
@@ -10830,7 +10830,7 @@
       <c r="G84" t="s">
         <v>500</v>
       </c>
-      <c r="H84" s="11"/>
+      <c r="H84" s="12"/>
       <c r="I84" t="s">
         <v>505</v>
       </c>
@@ -10873,7 +10873,7 @@
       <c r="Z84" t="s">
         <v>513</v>
       </c>
-      <c r="AA84" s="10"/>
+      <c r="AA84" s="11"/>
     </row>
     <row r="85" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
@@ -10897,7 +10897,7 @@
       <c r="G85" t="s">
         <v>500</v>
       </c>
-      <c r="H85" s="11"/>
+      <c r="H85" s="12"/>
       <c r="I85" t="s">
         <v>505</v>
       </c>
@@ -10940,7 +10940,7 @@
       <c r="Z85" t="s">
         <v>513</v>
       </c>
-      <c r="AA85" s="10"/>
+      <c r="AA85" s="11"/>
     </row>
     <row r="86" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
@@ -10964,7 +10964,7 @@
       <c r="G86" t="s">
         <v>516</v>
       </c>
-      <c r="H86" s="11" t="s">
+      <c r="H86" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I86" t="s">
@@ -11009,7 +11009,7 @@
       <c r="Z86" t="s">
         <v>528</v>
       </c>
-      <c r="AA86" s="10" t="s">
+      <c r="AA86" s="11" t="s">
         <v>92</v>
       </c>
     </row>
@@ -11035,7 +11035,7 @@
       <c r="G87" t="s">
         <v>516</v>
       </c>
-      <c r="H87" s="11"/>
+      <c r="H87" s="12"/>
       <c r="I87" t="s">
         <v>520</v>
       </c>
@@ -11078,7 +11078,7 @@
       <c r="Z87" t="s">
         <v>528</v>
       </c>
-      <c r="AA87" s="10"/>
+      <c r="AA87" s="11"/>
     </row>
     <row r="88" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
@@ -11102,7 +11102,7 @@
       <c r="G88" t="s">
         <v>516</v>
       </c>
-      <c r="H88" s="11"/>
+      <c r="H88" s="12"/>
       <c r="I88" t="s">
         <v>520</v>
       </c>
@@ -11145,7 +11145,7 @@
       <c r="Z88" t="s">
         <v>528</v>
       </c>
-      <c r="AA88" s="10"/>
+      <c r="AA88" s="11"/>
     </row>
     <row r="89" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
@@ -11169,7 +11169,7 @@
       <c r="G89" t="s">
         <v>516</v>
       </c>
-      <c r="H89" s="11"/>
+      <c r="H89" s="12"/>
       <c r="I89" t="s">
         <v>520</v>
       </c>
@@ -11212,7 +11212,7 @@
       <c r="Z89" t="s">
         <v>528</v>
       </c>
-      <c r="AA89" s="10"/>
+      <c r="AA89" s="11"/>
     </row>
     <row r="90" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
@@ -11236,7 +11236,7 @@
       <c r="G90" t="s">
         <v>532</v>
       </c>
-      <c r="H90" s="11" t="s">
+      <c r="H90" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I90" t="s">
@@ -11248,7 +11248,7 @@
       <c r="K90" t="s">
         <v>20</v>
       </c>
-      <c r="L90" s="10" t="s">
+      <c r="L90" s="11" t="s">
         <v>538</v>
       </c>
       <c r="M90" t="s">
@@ -11293,7 +11293,7 @@
       <c r="Z90" t="s">
         <v>548</v>
       </c>
-      <c r="AA90" s="10" t="s">
+      <c r="AA90" s="11" t="s">
         <v>114</v>
       </c>
       <c r="AB90" s="5"/>
@@ -11320,7 +11320,7 @@
       <c r="G91" t="s">
         <v>532</v>
       </c>
-      <c r="H91" s="11"/>
+      <c r="H91" s="12"/>
       <c r="I91" t="s">
         <v>536</v>
       </c>
@@ -11330,7 +11330,7 @@
       <c r="K91" t="s">
         <v>20</v>
       </c>
-      <c r="L91" s="10"/>
+      <c r="L91" s="11"/>
       <c r="M91" t="s">
         <v>16</v>
       </c>
@@ -11373,7 +11373,7 @@
       <c r="Z91" t="s">
         <v>548</v>
       </c>
-      <c r="AA91" s="10"/>
+      <c r="AA91" s="11"/>
       <c r="AB91" s="5"/>
     </row>
     <row r="92" spans="1:28" x14ac:dyDescent="0.3">
@@ -11398,7 +11398,7 @@
       <c r="G92" t="s">
         <v>532</v>
       </c>
-      <c r="H92" s="11"/>
+      <c r="H92" s="12"/>
       <c r="I92" t="s">
         <v>536</v>
       </c>
@@ -11408,7 +11408,7 @@
       <c r="K92" t="s">
         <v>20</v>
       </c>
-      <c r="L92" s="10"/>
+      <c r="L92" s="11"/>
       <c r="M92" t="s">
         <v>16</v>
       </c>
@@ -11451,7 +11451,7 @@
       <c r="Z92" t="s">
         <v>548</v>
       </c>
-      <c r="AA92" s="10"/>
+      <c r="AA92" s="11"/>
       <c r="AB92" s="5"/>
     </row>
     <row r="93" spans="1:28" x14ac:dyDescent="0.3">
@@ -11476,7 +11476,7 @@
       <c r="G93" t="s">
         <v>532</v>
       </c>
-      <c r="H93" s="11"/>
+      <c r="H93" s="12"/>
       <c r="I93" t="s">
         <v>536</v>
       </c>
@@ -11486,7 +11486,7 @@
       <c r="K93" t="s">
         <v>20</v>
       </c>
-      <c r="L93" s="10"/>
+      <c r="L93" s="11"/>
       <c r="M93" t="s">
         <v>16</v>
       </c>
@@ -11529,7 +11529,7 @@
       <c r="Z93" t="s">
         <v>548</v>
       </c>
-      <c r="AA93" s="10"/>
+      <c r="AA93" s="11"/>
       <c r="AB93" s="5"/>
     </row>
     <row r="94" spans="1:28" ht="144" customHeight="1" x14ac:dyDescent="0.3">
@@ -11554,7 +11554,7 @@
       <c r="G94" t="s">
         <v>554</v>
       </c>
-      <c r="H94" s="11" t="s">
+      <c r="H94" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I94" t="s">
@@ -11611,7 +11611,7 @@
       <c r="Z94" t="s">
         <v>563</v>
       </c>
-      <c r="AA94" s="10" t="s">
+      <c r="AA94" s="11" t="s">
         <v>96</v>
       </c>
     </row>
@@ -11637,7 +11637,7 @@
       <c r="G95" t="s">
         <v>554</v>
       </c>
-      <c r="H95" s="11"/>
+      <c r="H95" s="12"/>
       <c r="I95" t="s">
         <v>555</v>
       </c>
@@ -11692,7 +11692,7 @@
       <c r="Z95" t="s">
         <v>563</v>
       </c>
-      <c r="AA95" s="10"/>
+      <c r="AA95" s="11"/>
     </row>
     <row r="96" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
@@ -11716,7 +11716,7 @@
       <c r="G96" t="s">
         <v>554</v>
       </c>
-      <c r="H96" s="11"/>
+      <c r="H96" s="12"/>
       <c r="I96" t="s">
         <v>555</v>
       </c>
@@ -11771,7 +11771,7 @@
       <c r="Z96" t="s">
         <v>563</v>
       </c>
-      <c r="AA96" s="10"/>
+      <c r="AA96" s="11"/>
     </row>
     <row r="97" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
@@ -11795,7 +11795,7 @@
       <c r="G97" t="s">
         <v>554</v>
       </c>
-      <c r="H97" s="11"/>
+      <c r="H97" s="12"/>
       <c r="I97" t="s">
         <v>555</v>
       </c>
@@ -11850,7 +11850,7 @@
       <c r="Z97" t="s">
         <v>563</v>
       </c>
-      <c r="AA97" s="10"/>
+      <c r="AA97" s="11"/>
     </row>
     <row r="98" spans="1:27" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
@@ -11874,7 +11874,7 @@
       <c r="G98" t="s">
         <v>570</v>
       </c>
-      <c r="H98" s="11" t="s">
+      <c r="H98" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I98" t="s">
@@ -11931,7 +11931,7 @@
       <c r="Z98" t="s">
         <v>582</v>
       </c>
-      <c r="AA98" s="10" t="s">
+      <c r="AA98" s="11" t="s">
         <v>574</v>
       </c>
     </row>
@@ -11957,7 +11957,7 @@
       <c r="G99" t="s">
         <v>570</v>
       </c>
-      <c r="H99" s="11"/>
+      <c r="H99" s="12"/>
       <c r="I99" t="s">
         <v>571</v>
       </c>
@@ -12012,7 +12012,7 @@
       <c r="Z99" t="s">
         <v>582</v>
       </c>
-      <c r="AA99" s="10"/>
+      <c r="AA99" s="11"/>
     </row>
     <row r="100" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
@@ -12036,7 +12036,7 @@
       <c r="G100" t="s">
         <v>570</v>
       </c>
-      <c r="H100" s="11"/>
+      <c r="H100" s="12"/>
       <c r="I100" t="s">
         <v>571</v>
       </c>
@@ -12091,7 +12091,7 @@
       <c r="Z100" t="s">
         <v>582</v>
       </c>
-      <c r="AA100" s="10"/>
+      <c r="AA100" s="11"/>
     </row>
     <row r="101" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
@@ -12115,7 +12115,7 @@
       <c r="G101" t="s">
         <v>570</v>
       </c>
-      <c r="H101" s="11"/>
+      <c r="H101" s="12"/>
       <c r="I101" t="s">
         <v>571</v>
       </c>
@@ -12170,7 +12170,7 @@
       <c r="Z101" t="s">
         <v>582</v>
       </c>
-      <c r="AA101" s="10"/>
+      <c r="AA101" s="11"/>
     </row>
     <row r="102" spans="1:27" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
@@ -12194,7 +12194,7 @@
       <c r="G102" t="s">
         <v>589</v>
       </c>
-      <c r="H102" s="11" t="s">
+      <c r="H102" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I102" t="s">
@@ -12251,7 +12251,7 @@
       <c r="Z102" t="s">
         <v>598</v>
       </c>
-      <c r="AA102" s="10" t="s">
+      <c r="AA102" s="11" t="s">
         <v>100</v>
       </c>
     </row>
@@ -12277,7 +12277,7 @@
       <c r="G103" t="s">
         <v>589</v>
       </c>
-      <c r="H103" s="11"/>
+      <c r="H103" s="12"/>
       <c r="I103" t="s">
         <v>585</v>
       </c>
@@ -12332,7 +12332,7 @@
       <c r="Z103" t="s">
         <v>598</v>
       </c>
-      <c r="AA103" s="10"/>
+      <c r="AA103" s="11"/>
     </row>
     <row r="104" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
@@ -12356,7 +12356,7 @@
       <c r="G104" t="s">
         <v>589</v>
       </c>
-      <c r="H104" s="11"/>
+      <c r="H104" s="12"/>
       <c r="I104" t="s">
         <v>585</v>
       </c>
@@ -12411,7 +12411,7 @@
       <c r="Z104" t="s">
         <v>598</v>
       </c>
-      <c r="AA104" s="10"/>
+      <c r="AA104" s="11"/>
     </row>
     <row r="105" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
@@ -12435,7 +12435,7 @@
       <c r="G105" t="s">
         <v>589</v>
       </c>
-      <c r="H105" s="11"/>
+      <c r="H105" s="12"/>
       <c r="I105" t="s">
         <v>585</v>
       </c>
@@ -12490,7 +12490,7 @@
       <c r="Z105" t="s">
         <v>598</v>
       </c>
-      <c r="AA105" s="10"/>
+      <c r="AA105" s="11"/>
     </row>
     <row r="106" spans="1:27" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
@@ -12514,7 +12514,7 @@
       <c r="G106" t="s">
         <v>601</v>
       </c>
-      <c r="H106" s="11" t="s">
+      <c r="H106" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I106" t="s">
@@ -12571,7 +12571,7 @@
       <c r="Z106" t="s">
         <v>611</v>
       </c>
-      <c r="AA106" s="10" t="s">
+      <c r="AA106" s="11" t="s">
         <v>107</v>
       </c>
     </row>
@@ -12597,7 +12597,7 @@
       <c r="G107" t="s">
         <v>601</v>
       </c>
-      <c r="H107" s="11"/>
+      <c r="H107" s="12"/>
       <c r="I107" t="s">
         <v>602</v>
       </c>
@@ -12652,7 +12652,7 @@
       <c r="Z107" t="s">
         <v>611</v>
       </c>
-      <c r="AA107" s="10"/>
+      <c r="AA107" s="11"/>
     </row>
     <row r="108" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
@@ -12676,7 +12676,7 @@
       <c r="G108" t="s">
         <v>601</v>
       </c>
-      <c r="H108" s="11"/>
+      <c r="H108" s="12"/>
       <c r="I108" t="s">
         <v>602</v>
       </c>
@@ -12731,7 +12731,7 @@
       <c r="Z108" t="s">
         <v>611</v>
       </c>
-      <c r="AA108" s="10"/>
+      <c r="AA108" s="11"/>
     </row>
     <row r="109" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
@@ -12755,7 +12755,7 @@
       <c r="G109" t="s">
         <v>601</v>
       </c>
-      <c r="H109" s="11"/>
+      <c r="H109" s="12"/>
       <c r="I109" t="s">
         <v>602</v>
       </c>
@@ -12810,7 +12810,7 @@
       <c r="Z109" t="s">
         <v>611</v>
       </c>
-      <c r="AA109" s="10"/>
+      <c r="AA109" s="11"/>
     </row>
     <row r="110" spans="1:27" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
@@ -12834,7 +12834,7 @@
       <c r="G110" t="s">
         <v>614</v>
       </c>
-      <c r="H110" s="11" t="s">
+      <c r="H110" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I110" t="s">
@@ -12891,7 +12891,7 @@
       <c r="Z110" t="s">
         <v>629</v>
       </c>
-      <c r="AA110" s="10" t="s">
+      <c r="AA110" s="11" t="s">
         <v>623</v>
       </c>
     </row>
@@ -12917,7 +12917,7 @@
       <c r="G111" t="s">
         <v>614</v>
       </c>
-      <c r="H111" s="11"/>
+      <c r="H111" s="12"/>
       <c r="I111" t="s">
         <v>619</v>
       </c>
@@ -12972,7 +12972,7 @@
       <c r="Z111" t="s">
         <v>629</v>
       </c>
-      <c r="AA111" s="10"/>
+      <c r="AA111" s="11"/>
     </row>
     <row r="112" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
@@ -12996,7 +12996,7 @@
       <c r="G112" t="s">
         <v>614</v>
       </c>
-      <c r="H112" s="11"/>
+      <c r="H112" s="12"/>
       <c r="I112" t="s">
         <v>619</v>
       </c>
@@ -13051,7 +13051,7 @@
       <c r="Z112" t="s">
         <v>629</v>
       </c>
-      <c r="AA112" s="10"/>
+      <c r="AA112" s="11"/>
     </row>
     <row r="113" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
@@ -13075,7 +13075,7 @@
       <c r="G113" t="s">
         <v>614</v>
       </c>
-      <c r="H113" s="11"/>
+      <c r="H113" s="12"/>
       <c r="I113" t="s">
         <v>619</v>
       </c>
@@ -13130,7 +13130,7 @@
       <c r="Z113" t="s">
         <v>629</v>
       </c>
-      <c r="AA113" s="10"/>
+      <c r="AA113" s="11"/>
     </row>
     <row r="114" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
@@ -13154,7 +13154,7 @@
       <c r="G114" t="s">
         <v>631</v>
       </c>
-      <c r="H114" s="11" t="s">
+      <c r="H114" s="12" t="s">
         <v>637</v>
       </c>
       <c r="I114" t="s">
@@ -13199,7 +13199,7 @@
       <c r="Z114" t="s">
         <v>647</v>
       </c>
-      <c r="AA114" s="10" t="s">
+      <c r="AA114" s="11" t="s">
         <v>648</v>
       </c>
     </row>
@@ -13225,7 +13225,7 @@
       <c r="G115" t="s">
         <v>631</v>
       </c>
-      <c r="H115" s="11"/>
+      <c r="H115" s="12"/>
       <c r="I115" t="s">
         <v>638</v>
       </c>
@@ -13268,7 +13268,7 @@
       <c r="Z115" t="s">
         <v>647</v>
       </c>
-      <c r="AA115" s="10"/>
+      <c r="AA115" s="11"/>
     </row>
     <row r="116" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
@@ -13292,7 +13292,7 @@
       <c r="G116" t="s">
         <v>631</v>
       </c>
-      <c r="H116" s="11"/>
+      <c r="H116" s="12"/>
       <c r="I116" t="s">
         <v>638</v>
       </c>
@@ -13335,7 +13335,7 @@
       <c r="Z116" t="s">
         <v>647</v>
       </c>
-      <c r="AA116" s="10"/>
+      <c r="AA116" s="11"/>
     </row>
     <row r="117" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
@@ -13359,7 +13359,7 @@
       <c r="G117" t="s">
         <v>631</v>
       </c>
-      <c r="H117" s="11"/>
+      <c r="H117" s="12"/>
       <c r="I117" t="s">
         <v>638</v>
       </c>
@@ -13402,7 +13402,7 @@
       <c r="Z117" t="s">
         <v>647</v>
       </c>
-      <c r="AA117" s="10"/>
+      <c r="AA117" s="11"/>
     </row>
     <row r="118" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
@@ -13426,7 +13426,7 @@
       <c r="G118" t="s">
         <v>651</v>
       </c>
-      <c r="H118" s="11" t="s">
+      <c r="H118" s="12" t="s">
         <v>659</v>
       </c>
       <c r="I118" t="s">
@@ -13471,7 +13471,7 @@
       <c r="Z118" t="s">
         <v>664</v>
       </c>
-      <c r="AA118" s="10" t="s">
+      <c r="AA118" s="11" t="s">
         <v>111</v>
       </c>
     </row>
@@ -13497,7 +13497,7 @@
       <c r="G119" t="s">
         <v>651</v>
       </c>
-      <c r="H119" s="11"/>
+      <c r="H119" s="12"/>
       <c r="I119" t="s">
         <v>657</v>
       </c>
@@ -13540,7 +13540,7 @@
       <c r="Z119" t="s">
         <v>664</v>
       </c>
-      <c r="AA119" s="10"/>
+      <c r="AA119" s="11"/>
     </row>
     <row r="120" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
@@ -13564,7 +13564,7 @@
       <c r="G120" t="s">
         <v>651</v>
       </c>
-      <c r="H120" s="11"/>
+      <c r="H120" s="12"/>
       <c r="I120" t="s">
         <v>657</v>
       </c>
@@ -13607,7 +13607,7 @@
       <c r="Z120" t="s">
         <v>664</v>
       </c>
-      <c r="AA120" s="10"/>
+      <c r="AA120" s="11"/>
     </row>
     <row r="121" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
@@ -13631,7 +13631,7 @@
       <c r="G121" t="s">
         <v>651</v>
       </c>
-      <c r="H121" s="11"/>
+      <c r="H121" s="12"/>
       <c r="I121" t="s">
         <v>657</v>
       </c>
@@ -13674,7 +13674,7 @@
       <c r="Z121" t="s">
         <v>664</v>
       </c>
-      <c r="AA121" s="10"/>
+      <c r="AA121" s="11"/>
     </row>
     <row r="122" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
@@ -13698,7 +13698,7 @@
       <c r="G122" t="s">
         <v>668</v>
       </c>
-      <c r="H122" s="11" t="s">
+      <c r="H122" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I122" t="s">
@@ -13743,7 +13743,7 @@
       <c r="Z122" t="s">
         <v>680</v>
       </c>
-      <c r="AA122" s="10" t="s">
+      <c r="AA122" s="11" t="s">
         <v>117</v>
       </c>
     </row>
@@ -13769,7 +13769,7 @@
       <c r="G123" t="s">
         <v>668</v>
       </c>
-      <c r="H123" s="11"/>
+      <c r="H123" s="12"/>
       <c r="I123" t="s">
         <v>667</v>
       </c>
@@ -13812,7 +13812,7 @@
       <c r="Z123" t="s">
         <v>680</v>
       </c>
-      <c r="AA123" s="10"/>
+      <c r="AA123" s="11"/>
     </row>
     <row r="124" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
@@ -13836,7 +13836,7 @@
       <c r="G124" t="s">
         <v>668</v>
       </c>
-      <c r="H124" s="11"/>
+      <c r="H124" s="12"/>
       <c r="I124" t="s">
         <v>667</v>
       </c>
@@ -13879,7 +13879,7 @@
       <c r="Z124" t="s">
         <v>680</v>
       </c>
-      <c r="AA124" s="10"/>
+      <c r="AA124" s="11"/>
     </row>
     <row r="125" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
@@ -13903,7 +13903,7 @@
       <c r="G125" t="s">
         <v>668</v>
       </c>
-      <c r="H125" s="11"/>
+      <c r="H125" s="12"/>
       <c r="I125" t="s">
         <v>667</v>
       </c>
@@ -13946,7 +13946,7 @@
       <c r="Z125" t="s">
         <v>680</v>
       </c>
-      <c r="AA125" s="10"/>
+      <c r="AA125" s="11"/>
     </row>
     <row r="126" spans="1:28" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
@@ -13970,7 +13970,7 @@
       <c r="G126" t="s">
         <v>685</v>
       </c>
-      <c r="H126" s="11" t="s">
+      <c r="H126" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I126" t="s">
@@ -14027,10 +14027,10 @@
       <c r="Z126" t="s">
         <v>699</v>
       </c>
-      <c r="AA126" s="10" t="s">
+      <c r="AA126" s="11" t="s">
         <v>683</v>
       </c>
-      <c r="AB126" s="12" t="s">
+      <c r="AB126" s="13" t="s">
         <v>146</v>
       </c>
     </row>
@@ -14056,7 +14056,7 @@
       <c r="G127" t="s">
         <v>685</v>
       </c>
-      <c r="H127" s="11"/>
+      <c r="H127" s="12"/>
       <c r="I127" t="s">
         <v>690</v>
       </c>
@@ -14111,8 +14111,8 @@
       <c r="Z127" t="s">
         <v>699</v>
       </c>
-      <c r="AA127" s="10"/>
-      <c r="AB127" s="12"/>
+      <c r="AA127" s="11"/>
+      <c r="AB127" s="13"/>
     </row>
     <row r="128" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
@@ -14136,7 +14136,7 @@
       <c r="G128" t="s">
         <v>685</v>
       </c>
-      <c r="H128" s="11"/>
+      <c r="H128" s="12"/>
       <c r="I128" t="s">
         <v>690</v>
       </c>
@@ -14191,8 +14191,8 @@
       <c r="Z128" t="s">
         <v>699</v>
       </c>
-      <c r="AA128" s="10"/>
-      <c r="AB128" s="12"/>
+      <c r="AA128" s="11"/>
+      <c r="AB128" s="13"/>
     </row>
     <row r="129" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
@@ -14216,7 +14216,7 @@
       <c r="G129" t="s">
         <v>685</v>
       </c>
-      <c r="H129" s="11"/>
+      <c r="H129" s="12"/>
       <c r="I129" t="s">
         <v>690</v>
       </c>
@@ -14271,8 +14271,8 @@
       <c r="Z129" t="s">
         <v>699</v>
       </c>
-      <c r="AA129" s="10"/>
-      <c r="AB129" s="12"/>
+      <c r="AA129" s="11"/>
+      <c r="AB129" s="13"/>
     </row>
     <row r="130" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
@@ -14296,7 +14296,7 @@
       <c r="G130" t="s">
         <v>123</v>
       </c>
-      <c r="H130" s="11" t="s">
+      <c r="H130" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I130" t="s">
@@ -14353,10 +14353,10 @@
       <c r="Z130" t="s">
         <v>708</v>
       </c>
-      <c r="AA130" s="10" t="s">
+      <c r="AA130" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="AB130" s="13" t="s">
+      <c r="AB130" s="10" t="s">
         <v>700</v>
       </c>
     </row>
@@ -14382,7 +14382,7 @@
       <c r="G131" t="s">
         <v>123</v>
       </c>
-      <c r="H131" s="11"/>
+      <c r="H131" s="12"/>
       <c r="I131" t="s">
         <v>128</v>
       </c>
@@ -14437,8 +14437,8 @@
       <c r="Z131" t="s">
         <v>708</v>
       </c>
-      <c r="AA131" s="10"/>
-      <c r="AB131" s="13"/>
+      <c r="AA131" s="11"/>
+      <c r="AB131" s="10"/>
     </row>
     <row r="132" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
@@ -14462,7 +14462,7 @@
       <c r="G132" t="s">
         <v>123</v>
       </c>
-      <c r="H132" s="11"/>
+      <c r="H132" s="12"/>
       <c r="I132" t="s">
         <v>128</v>
       </c>
@@ -14517,8 +14517,8 @@
       <c r="Z132" t="s">
         <v>708</v>
       </c>
-      <c r="AA132" s="10"/>
-      <c r="AB132" s="13"/>
+      <c r="AA132" s="11"/>
+      <c r="AB132" s="10"/>
     </row>
     <row r="133" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
@@ -14542,7 +14542,7 @@
       <c r="G133" t="s">
         <v>123</v>
       </c>
-      <c r="H133" s="11"/>
+      <c r="H133" s="12"/>
       <c r="I133" t="s">
         <v>128</v>
       </c>
@@ -14597,8 +14597,8 @@
       <c r="Z133" t="s">
         <v>708</v>
       </c>
-      <c r="AA133" s="10"/>
-      <c r="AB133" s="13"/>
+      <c r="AA133" s="11"/>
+      <c r="AB133" s="10"/>
     </row>
     <row r="134" spans="1:28" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
@@ -14622,7 +14622,7 @@
       <c r="G134" t="s">
         <v>711</v>
       </c>
-      <c r="H134" s="11" t="s">
+      <c r="H134" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I134" t="s">
@@ -14679,7 +14679,7 @@
       <c r="Z134" t="s">
         <v>721</v>
       </c>
-      <c r="AA134" s="10" t="s">
+      <c r="AA134" s="11" t="s">
         <v>136</v>
       </c>
     </row>
@@ -14705,7 +14705,7 @@
       <c r="G135" t="s">
         <v>711</v>
       </c>
-      <c r="H135" s="11"/>
+      <c r="H135" s="12"/>
       <c r="I135" t="s">
         <v>713</v>
       </c>
@@ -14760,7 +14760,7 @@
       <c r="Z135" t="s">
         <v>721</v>
       </c>
-      <c r="AA135" s="10"/>
+      <c r="AA135" s="11"/>
     </row>
     <row r="136" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
@@ -14784,7 +14784,7 @@
       <c r="G136" t="s">
         <v>711</v>
       </c>
-      <c r="H136" s="11"/>
+      <c r="H136" s="12"/>
       <c r="I136" t="s">
         <v>713</v>
       </c>
@@ -14839,7 +14839,7 @@
       <c r="Z136" t="s">
         <v>721</v>
       </c>
-      <c r="AA136" s="10"/>
+      <c r="AA136" s="11"/>
     </row>
     <row r="137" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
@@ -14863,7 +14863,7 @@
       <c r="G137" t="s">
         <v>711</v>
       </c>
-      <c r="H137" s="11"/>
+      <c r="H137" s="12"/>
       <c r="I137" t="s">
         <v>713</v>
       </c>
@@ -14918,7 +14918,7 @@
       <c r="Z137" t="s">
         <v>721</v>
       </c>
-      <c r="AA137" s="10"/>
+      <c r="AA137" s="11"/>
     </row>
     <row r="138" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
@@ -14942,7 +14942,7 @@
       <c r="G138" t="s">
         <v>724</v>
       </c>
-      <c r="H138" s="11" t="s">
+      <c r="H138" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I138" t="s">
@@ -14987,7 +14987,7 @@
       <c r="Z138" t="s">
         <v>738</v>
       </c>
-      <c r="AA138" s="10" t="s">
+      <c r="AA138" s="11" t="s">
         <v>138</v>
       </c>
     </row>
@@ -15013,7 +15013,7 @@
       <c r="G139" t="s">
         <v>724</v>
       </c>
-      <c r="H139" s="11"/>
+      <c r="H139" s="12"/>
       <c r="I139" t="s">
         <v>730</v>
       </c>
@@ -15056,7 +15056,7 @@
       <c r="Z139" t="s">
         <v>738</v>
       </c>
-      <c r="AA139" s="10"/>
+      <c r="AA139" s="11"/>
     </row>
     <row r="140" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
@@ -15080,7 +15080,7 @@
       <c r="G140" t="s">
         <v>724</v>
       </c>
-      <c r="H140" s="11"/>
+      <c r="H140" s="12"/>
       <c r="I140" t="s">
         <v>730</v>
       </c>
@@ -15123,7 +15123,7 @@
       <c r="Z140" t="s">
         <v>738</v>
       </c>
-      <c r="AA140" s="10"/>
+      <c r="AA140" s="11"/>
     </row>
     <row r="141" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
@@ -15147,7 +15147,7 @@
       <c r="G141" t="s">
         <v>724</v>
       </c>
-      <c r="H141" s="11"/>
+      <c r="H141" s="12"/>
       <c r="I141" t="s">
         <v>730</v>
       </c>
@@ -15190,7 +15190,7 @@
       <c r="Z141" t="s">
         <v>738</v>
       </c>
-      <c r="AA141" s="10"/>
+      <c r="AA141" s="11"/>
     </row>
     <row r="142" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
@@ -15214,7 +15214,7 @@
       <c r="G142" t="s">
         <v>741</v>
       </c>
-      <c r="H142" s="11" t="s">
+      <c r="H142" s="12" t="s">
         <v>140</v>
       </c>
       <c r="I142" t="s">
@@ -15259,7 +15259,7 @@
       <c r="Z142" t="s">
         <v>755</v>
       </c>
-      <c r="AA142" s="10" t="s">
+      <c r="AA142" s="11" t="s">
         <v>141</v>
       </c>
     </row>
@@ -15285,7 +15285,7 @@
       <c r="G143" t="s">
         <v>741</v>
       </c>
-      <c r="H143" s="11"/>
+      <c r="H143" s="12"/>
       <c r="I143" t="s">
         <v>746</v>
       </c>
@@ -15328,7 +15328,7 @@
       <c r="Z143" t="s">
         <v>755</v>
       </c>
-      <c r="AA143" s="10"/>
+      <c r="AA143" s="11"/>
     </row>
     <row r="144" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
@@ -15352,7 +15352,7 @@
       <c r="G144" t="s">
         <v>741</v>
       </c>
-      <c r="H144" s="11"/>
+      <c r="H144" s="12"/>
       <c r="I144" t="s">
         <v>746</v>
       </c>
@@ -15395,7 +15395,7 @@
       <c r="Z144" t="s">
         <v>755</v>
       </c>
-      <c r="AA144" s="10"/>
+      <c r="AA144" s="11"/>
     </row>
     <row r="145" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
@@ -15419,7 +15419,7 @@
       <c r="G145" t="s">
         <v>741</v>
       </c>
-      <c r="H145" s="11"/>
+      <c r="H145" s="12"/>
       <c r="I145" t="s">
         <v>746</v>
       </c>
@@ -15462,7 +15462,7 @@
       <c r="Z145" t="s">
         <v>755</v>
       </c>
-      <c r="AA145" s="10"/>
+      <c r="AA145" s="11"/>
     </row>
     <row r="146" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
@@ -15486,7 +15486,7 @@
       <c r="G146" t="s">
         <v>766</v>
       </c>
-      <c r="H146" s="11" t="s">
+      <c r="H146" s="12" t="s">
         <v>767</v>
       </c>
       <c r="I146" t="s">
@@ -15531,10 +15531,10 @@
       <c r="Z146" t="s">
         <v>776</v>
       </c>
-      <c r="AA146" s="10" t="s">
+      <c r="AA146" s="11" t="s">
         <v>768</v>
       </c>
-      <c r="AB146" s="10" t="s">
+      <c r="AB146" s="11" t="s">
         <v>756</v>
       </c>
     </row>
@@ -15560,7 +15560,7 @@
       <c r="G147" t="s">
         <v>766</v>
       </c>
-      <c r="H147" s="11"/>
+      <c r="H147" s="12"/>
       <c r="I147" t="s">
         <v>764</v>
       </c>
@@ -15603,8 +15603,8 @@
       <c r="Z147" t="s">
         <v>776</v>
       </c>
-      <c r="AA147" s="10"/>
-      <c r="AB147" s="10"/>
+      <c r="AA147" s="11"/>
+      <c r="AB147" s="11"/>
     </row>
     <row r="148" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
@@ -15628,7 +15628,7 @@
       <c r="G148" t="s">
         <v>766</v>
       </c>
-      <c r="H148" s="11"/>
+      <c r="H148" s="12"/>
       <c r="I148" t="s">
         <v>764</v>
       </c>
@@ -15671,8 +15671,8 @@
       <c r="Z148" t="s">
         <v>776</v>
       </c>
-      <c r="AA148" s="10"/>
-      <c r="AB148" s="10"/>
+      <c r="AA148" s="11"/>
+      <c r="AB148" s="11"/>
     </row>
     <row r="149" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
@@ -15696,7 +15696,7 @@
       <c r="G149" t="s">
         <v>766</v>
       </c>
-      <c r="H149" s="11"/>
+      <c r="H149" s="12"/>
       <c r="I149" t="s">
         <v>764</v>
       </c>
@@ -15739,8 +15739,8 @@
       <c r="Z149" t="s">
         <v>776</v>
       </c>
-      <c r="AA149" s="10"/>
-      <c r="AB149" s="10"/>
+      <c r="AA149" s="11"/>
+      <c r="AB149" s="11"/>
     </row>
     <row r="150" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
@@ -15764,7 +15764,7 @@
       <c r="G150" t="s">
         <v>779</v>
       </c>
-      <c r="H150" s="11" t="s">
+      <c r="H150" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I150" t="s">
@@ -15821,7 +15821,7 @@
       <c r="Z150" t="s">
         <v>797</v>
       </c>
-      <c r="AA150" s="10" t="s">
+      <c r="AA150" s="11" t="s">
         <v>789</v>
       </c>
     </row>
@@ -15847,7 +15847,7 @@
       <c r="G151" t="s">
         <v>779</v>
       </c>
-      <c r="H151" s="11"/>
+      <c r="H151" s="12"/>
       <c r="I151" t="s">
         <v>784</v>
       </c>
@@ -15902,7 +15902,7 @@
       <c r="Z151" t="s">
         <v>797</v>
       </c>
-      <c r="AA151" s="10"/>
+      <c r="AA151" s="11"/>
     </row>
     <row r="152" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
@@ -15926,7 +15926,7 @@
       <c r="G152" t="s">
         <v>779</v>
       </c>
-      <c r="H152" s="11"/>
+      <c r="H152" s="12"/>
       <c r="I152" t="s">
         <v>784</v>
       </c>
@@ -15981,7 +15981,7 @@
       <c r="Z152" t="s">
         <v>797</v>
       </c>
-      <c r="AA152" s="10"/>
+      <c r="AA152" s="11"/>
     </row>
     <row r="153" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
@@ -16005,7 +16005,7 @@
       <c r="G153" t="s">
         <v>779</v>
       </c>
-      <c r="H153" s="11"/>
+      <c r="H153" s="12"/>
       <c r="I153" t="s">
         <v>784</v>
       </c>
@@ -16060,7 +16060,7 @@
       <c r="Z153" t="s">
         <v>797</v>
       </c>
-      <c r="AA153" s="10"/>
+      <c r="AA153" s="11"/>
     </row>
     <row r="154" spans="1:28" ht="187.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
@@ -16084,7 +16084,7 @@
       <c r="G154" t="s">
         <v>806</v>
       </c>
-      <c r="H154" s="11" t="s">
+      <c r="H154" s="12" t="s">
         <v>807</v>
       </c>
       <c r="I154" t="s">
@@ -16141,7 +16141,7 @@
       <c r="Z154" t="s">
         <v>816</v>
       </c>
-      <c r="AA154" s="10" t="s">
+      <c r="AA154" s="11" t="s">
         <v>817</v>
       </c>
     </row>
@@ -16167,7 +16167,7 @@
       <c r="G155" t="s">
         <v>806</v>
       </c>
-      <c r="H155" s="11"/>
+      <c r="H155" s="12"/>
       <c r="I155" t="s">
         <v>808</v>
       </c>
@@ -16222,7 +16222,7 @@
       <c r="Z155" t="s">
         <v>816</v>
       </c>
-      <c r="AA155" s="10"/>
+      <c r="AA155" s="11"/>
     </row>
     <row r="156" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
@@ -16246,7 +16246,7 @@
       <c r="G156" t="s">
         <v>806</v>
       </c>
-      <c r="H156" s="11"/>
+      <c r="H156" s="12"/>
       <c r="I156" t="s">
         <v>808</v>
       </c>
@@ -16301,7 +16301,7 @@
       <c r="Z156" t="s">
         <v>816</v>
       </c>
-      <c r="AA156" s="10"/>
+      <c r="AA156" s="11"/>
     </row>
     <row r="157" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
@@ -16325,7 +16325,7 @@
       <c r="G157" t="s">
         <v>806</v>
       </c>
-      <c r="H157" s="11"/>
+      <c r="H157" s="12"/>
       <c r="I157" t="s">
         <v>808</v>
       </c>
@@ -16380,7 +16380,7 @@
       <c r="Z157" t="s">
         <v>816</v>
       </c>
-      <c r="AA157" s="10"/>
+      <c r="AA157" s="11"/>
     </row>
     <row r="158" spans="1:28" ht="187.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
@@ -16404,7 +16404,7 @@
       <c r="G158" t="s">
         <v>821</v>
       </c>
-      <c r="H158" s="11" t="s">
+      <c r="H158" s="12" t="s">
         <v>828</v>
       </c>
       <c r="I158" t="s">
@@ -16461,7 +16461,7 @@
       <c r="Z158" t="s">
         <v>816</v>
       </c>
-      <c r="AA158" s="10" t="s">
+      <c r="AA158" s="11" t="s">
         <v>835</v>
       </c>
     </row>
@@ -16487,7 +16487,7 @@
       <c r="G159" t="s">
         <v>821</v>
       </c>
-      <c r="H159" s="11"/>
+      <c r="H159" s="12"/>
       <c r="I159" t="s">
         <v>827</v>
       </c>
@@ -16542,7 +16542,7 @@
       <c r="Z159" t="s">
         <v>816</v>
       </c>
-      <c r="AA159" s="10"/>
+      <c r="AA159" s="11"/>
     </row>
     <row r="160" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
@@ -16566,7 +16566,7 @@
       <c r="G160" t="s">
         <v>821</v>
       </c>
-      <c r="H160" s="11"/>
+      <c r="H160" s="12"/>
       <c r="I160" t="s">
         <v>827</v>
       </c>
@@ -16621,7 +16621,7 @@
       <c r="Z160" t="s">
         <v>816</v>
       </c>
-      <c r="AA160" s="10"/>
+      <c r="AA160" s="11"/>
     </row>
     <row r="161" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
@@ -16645,7 +16645,7 @@
       <c r="G161" t="s">
         <v>821</v>
       </c>
-      <c r="H161" s="11"/>
+      <c r="H161" s="12"/>
       <c r="I161" t="s">
         <v>827</v>
       </c>
@@ -16700,33 +16700,62 @@
       <c r="Z161" t="s">
         <v>816</v>
       </c>
-      <c r="AA161" s="10"/>
+      <c r="AA161" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="92">
-    <mergeCell ref="AB130:AB133"/>
-    <mergeCell ref="AB146:AB149"/>
-    <mergeCell ref="H154:H157"/>
-    <mergeCell ref="AA154:AA157"/>
-    <mergeCell ref="H158:H161"/>
-    <mergeCell ref="AA158:AA161"/>
-    <mergeCell ref="L90:L93"/>
-    <mergeCell ref="AB18:AB21"/>
-    <mergeCell ref="AB26:AB29"/>
-    <mergeCell ref="AB30:AB33"/>
-    <mergeCell ref="AB54:AB57"/>
-    <mergeCell ref="AB62:AB65"/>
-    <mergeCell ref="AA26:AA29"/>
-    <mergeCell ref="H142:H145"/>
-    <mergeCell ref="AA142:AA145"/>
-    <mergeCell ref="H146:H149"/>
-    <mergeCell ref="AA146:AA149"/>
-    <mergeCell ref="H150:H153"/>
-    <mergeCell ref="AA150:AA153"/>
-    <mergeCell ref="H130:H133"/>
-    <mergeCell ref="AA130:AA133"/>
-    <mergeCell ref="H134:H137"/>
-    <mergeCell ref="AA134:AA137"/>
+    <mergeCell ref="AB6:AB9"/>
+    <mergeCell ref="AB10:AB13"/>
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="AA126:AA129"/>
+    <mergeCell ref="AB126:AB129"/>
+    <mergeCell ref="H86:H89"/>
+    <mergeCell ref="AA86:AA89"/>
+    <mergeCell ref="H102:H105"/>
+    <mergeCell ref="AA102:AA105"/>
+    <mergeCell ref="H122:H125"/>
+    <mergeCell ref="AA122:AA125"/>
+    <mergeCell ref="AA98:AA101"/>
+    <mergeCell ref="H62:H65"/>
+    <mergeCell ref="AA62:AA65"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="AA66:AA69"/>
+    <mergeCell ref="H82:H85"/>
+    <mergeCell ref="AA82:AA85"/>
+    <mergeCell ref="H70:H73"/>
+    <mergeCell ref="AA70:AA73"/>
+    <mergeCell ref="H74:H77"/>
+    <mergeCell ref="AA74:AA77"/>
+    <mergeCell ref="H78:H81"/>
+    <mergeCell ref="AA78:AA81"/>
+    <mergeCell ref="H50:H53"/>
+    <mergeCell ref="AA50:AA53"/>
+    <mergeCell ref="H54:H57"/>
+    <mergeCell ref="AA54:AA57"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="AA58:AA61"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="AA2:AA5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="AA6:AA9"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="AA10:AA13"/>
+    <mergeCell ref="AA94:AA97"/>
+    <mergeCell ref="H98:H101"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="L14:L17"/>
+    <mergeCell ref="AA14:AA17"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="AA18:AA21"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="AA30:AA33"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="AA34:AA37"/>
+    <mergeCell ref="H38:H41"/>
+    <mergeCell ref="AA38:AA41"/>
+    <mergeCell ref="H42:H45"/>
+    <mergeCell ref="AA42:AA45"/>
+    <mergeCell ref="H46:H49"/>
     <mergeCell ref="H138:H141"/>
     <mergeCell ref="AA138:AA141"/>
     <mergeCell ref="H22:H25"/>
@@ -16743,59 +16772,30 @@
     <mergeCell ref="H114:H117"/>
     <mergeCell ref="AA114:AA117"/>
     <mergeCell ref="H94:H97"/>
-    <mergeCell ref="AA94:AA97"/>
-    <mergeCell ref="H98:H101"/>
-    <mergeCell ref="H14:H17"/>
-    <mergeCell ref="L14:L17"/>
-    <mergeCell ref="AA14:AA17"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="AA18:AA21"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="AA2:AA5"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="AA6:AA9"/>
-    <mergeCell ref="H10:H13"/>
-    <mergeCell ref="AA10:AA13"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="AA30:AA33"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="AA34:AA37"/>
-    <mergeCell ref="H38:H41"/>
-    <mergeCell ref="AA38:AA41"/>
-    <mergeCell ref="H42:H45"/>
-    <mergeCell ref="AA42:AA45"/>
-    <mergeCell ref="H46:H49"/>
+    <mergeCell ref="L90:L93"/>
+    <mergeCell ref="AB18:AB21"/>
+    <mergeCell ref="AB26:AB29"/>
+    <mergeCell ref="AB30:AB33"/>
+    <mergeCell ref="AB54:AB57"/>
+    <mergeCell ref="AB62:AB65"/>
+    <mergeCell ref="AA26:AA29"/>
     <mergeCell ref="AA46:AA49"/>
-    <mergeCell ref="H50:H53"/>
-    <mergeCell ref="AA50:AA53"/>
-    <mergeCell ref="H54:H57"/>
-    <mergeCell ref="AA54:AA57"/>
-    <mergeCell ref="H58:H61"/>
-    <mergeCell ref="AA58:AA61"/>
-    <mergeCell ref="H82:H85"/>
-    <mergeCell ref="AA82:AA85"/>
-    <mergeCell ref="H70:H73"/>
-    <mergeCell ref="AA70:AA73"/>
-    <mergeCell ref="H74:H77"/>
-    <mergeCell ref="AA74:AA77"/>
-    <mergeCell ref="H78:H81"/>
-    <mergeCell ref="AA78:AA81"/>
-    <mergeCell ref="AB6:AB9"/>
-    <mergeCell ref="AB10:AB13"/>
-    <mergeCell ref="H126:H129"/>
-    <mergeCell ref="AA126:AA129"/>
-    <mergeCell ref="AB126:AB129"/>
-    <mergeCell ref="H86:H89"/>
-    <mergeCell ref="AA86:AA89"/>
-    <mergeCell ref="H102:H105"/>
-    <mergeCell ref="AA102:AA105"/>
-    <mergeCell ref="H122:H125"/>
-    <mergeCell ref="AA122:AA125"/>
-    <mergeCell ref="AA98:AA101"/>
-    <mergeCell ref="H62:H65"/>
-    <mergeCell ref="AA62:AA65"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="AA66:AA69"/>
+    <mergeCell ref="AB130:AB133"/>
+    <mergeCell ref="AB146:AB149"/>
+    <mergeCell ref="H154:H157"/>
+    <mergeCell ref="AA154:AA157"/>
+    <mergeCell ref="H158:H161"/>
+    <mergeCell ref="AA158:AA161"/>
+    <mergeCell ref="H142:H145"/>
+    <mergeCell ref="AA142:AA145"/>
+    <mergeCell ref="H146:H149"/>
+    <mergeCell ref="AA146:AA149"/>
+    <mergeCell ref="H150:H153"/>
+    <mergeCell ref="AA150:AA153"/>
+    <mergeCell ref="H130:H133"/>
+    <mergeCell ref="AA130:AA133"/>
+    <mergeCell ref="H134:H137"/>
+    <mergeCell ref="AA134:AA137"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
16-06-25 : suite nmds et début des dendrogramme sous agnes
</commit_message>
<xml_diff>
--- a/Resultats_modeles_coleo_2024.xlsx
+++ b/Resultats_modeles_coleo_2024.xlsx
@@ -4273,6 +4273,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4281,9 +4284,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4705,7 +4705,7 @@
       <c r="G2" t="s">
         <v>154</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I2" t="s">
@@ -4762,7 +4762,7 @@
       <c r="Z2" t="s">
         <v>173</v>
       </c>
-      <c r="AA2" s="10" t="s">
+      <c r="AA2" s="11" t="s">
         <v>45</v>
       </c>
     </row>
@@ -4788,7 +4788,7 @@
       <c r="G3" t="s">
         <v>154</v>
       </c>
-      <c r="H3" s="11"/>
+      <c r="H3" s="12"/>
       <c r="I3" t="s">
         <v>150</v>
       </c>
@@ -4843,7 +4843,7 @@
       <c r="Z3" t="s">
         <v>173</v>
       </c>
-      <c r="AA3" s="10"/>
+      <c r="AA3" s="11"/>
     </row>
     <row r="4" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
@@ -4867,7 +4867,7 @@
       <c r="G4" t="s">
         <v>154</v>
       </c>
-      <c r="H4" s="11"/>
+      <c r="H4" s="12"/>
       <c r="I4" t="s">
         <v>150</v>
       </c>
@@ -4922,7 +4922,7 @@
       <c r="Z4" t="s">
         <v>173</v>
       </c>
-      <c r="AA4" s="10"/>
+      <c r="AA4" s="11"/>
     </row>
     <row r="5" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -4946,7 +4946,7 @@
       <c r="G5" t="s">
         <v>154</v>
       </c>
-      <c r="H5" s="11"/>
+      <c r="H5" s="12"/>
       <c r="I5" t="s">
         <v>150</v>
       </c>
@@ -5001,7 +5001,7 @@
       <c r="Z5" t="s">
         <v>173</v>
       </c>
-      <c r="AA5" s="10"/>
+      <c r="AA5" s="11"/>
     </row>
     <row r="6" spans="1:29" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
@@ -5025,7 +5025,7 @@
       <c r="G6" t="s">
         <v>184</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I6" t="s">
@@ -5082,10 +5082,10 @@
       <c r="Z6" t="s">
         <v>182</v>
       </c>
-      <c r="AA6" s="10" t="s">
+      <c r="AA6" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="AB6" s="10" t="s">
+      <c r="AB6" s="11" t="s">
         <v>174</v>
       </c>
     </row>
@@ -5111,7 +5111,7 @@
       <c r="G7" t="s">
         <v>184</v>
       </c>
-      <c r="H7" s="11"/>
+      <c r="H7" s="12"/>
       <c r="I7" t="s">
         <v>189</v>
       </c>
@@ -5166,8 +5166,8 @@
       <c r="Z7" t="s">
         <v>182</v>
       </c>
-      <c r="AA7" s="10"/>
-      <c r="AB7" s="10"/>
+      <c r="AA7" s="11"/>
+      <c r="AB7" s="11"/>
     </row>
     <row r="8" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -5191,7 +5191,7 @@
       <c r="G8" t="s">
         <v>184</v>
       </c>
-      <c r="H8" s="11"/>
+      <c r="H8" s="12"/>
       <c r="I8" t="s">
         <v>189</v>
       </c>
@@ -5246,8 +5246,8 @@
       <c r="Z8" t="s">
         <v>182</v>
       </c>
-      <c r="AA8" s="10"/>
-      <c r="AB8" s="10"/>
+      <c r="AA8" s="11"/>
+      <c r="AB8" s="11"/>
     </row>
     <row r="9" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
@@ -5271,7 +5271,7 @@
       <c r="G9" t="s">
         <v>184</v>
       </c>
-      <c r="H9" s="11"/>
+      <c r="H9" s="12"/>
       <c r="I9" t="s">
         <v>189</v>
       </c>
@@ -5326,8 +5326,8 @@
       <c r="Z9" t="s">
         <v>182</v>
       </c>
-      <c r="AA9" s="10"/>
-      <c r="AB9" s="10"/>
+      <c r="AA9" s="11"/>
+      <c r="AB9" s="11"/>
     </row>
     <row r="10" spans="1:29" ht="120" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
@@ -5351,7 +5351,7 @@
       <c r="G10" t="s">
         <v>194</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I10" t="s">
@@ -5408,10 +5408,10 @@
       <c r="Z10" t="s">
         <v>208</v>
       </c>
-      <c r="AA10" s="10" t="s">
+      <c r="AA10" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="AB10" s="10" t="s">
+      <c r="AB10" s="11" t="s">
         <v>209</v>
       </c>
     </row>
@@ -5437,7 +5437,7 @@
       <c r="G11" t="s">
         <v>194</v>
       </c>
-      <c r="H11" s="11"/>
+      <c r="H11" s="12"/>
       <c r="I11" t="s">
         <v>199</v>
       </c>
@@ -5492,8 +5492,8 @@
       <c r="Z11" t="s">
         <v>208</v>
       </c>
-      <c r="AA11" s="10"/>
-      <c r="AB11" s="10"/>
+      <c r="AA11" s="11"/>
+      <c r="AB11" s="11"/>
     </row>
     <row r="12" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
@@ -5517,7 +5517,7 @@
       <c r="G12" t="s">
         <v>194</v>
       </c>
-      <c r="H12" s="11"/>
+      <c r="H12" s="12"/>
       <c r="I12" t="s">
         <v>199</v>
       </c>
@@ -5572,8 +5572,8 @@
       <c r="Z12" t="s">
         <v>208</v>
       </c>
-      <c r="AA12" s="10"/>
-      <c r="AB12" s="10"/>
+      <c r="AA12" s="11"/>
+      <c r="AB12" s="11"/>
     </row>
     <row r="13" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -5597,7 +5597,7 @@
       <c r="G13" t="s">
         <v>194</v>
       </c>
-      <c r="H13" s="11"/>
+      <c r="H13" s="12"/>
       <c r="I13" t="s">
         <v>199</v>
       </c>
@@ -5652,8 +5652,8 @@
       <c r="Z13" t="s">
         <v>208</v>
       </c>
-      <c r="AA13" s="10"/>
-      <c r="AB13" s="10"/>
+      <c r="AA13" s="11"/>
+      <c r="AB13" s="11"/>
     </row>
     <row r="14" spans="1:29" ht="131.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -5677,7 +5677,7 @@
       <c r="G14" t="s">
         <v>211</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I14" t="s">
@@ -5689,7 +5689,7 @@
       <c r="K14" t="s">
         <v>20</v>
       </c>
-      <c r="L14" s="10" t="s">
+      <c r="L14" s="11" t="s">
         <v>44</v>
       </c>
       <c r="M14" t="s">
@@ -5734,7 +5734,7 @@
       <c r="Z14" t="s">
         <v>223</v>
       </c>
-      <c r="AA14" s="10" t="s">
+      <c r="AA14" s="11" t="s">
         <v>48</v>
       </c>
     </row>
@@ -5760,7 +5760,7 @@
       <c r="G15" t="s">
         <v>211</v>
       </c>
-      <c r="H15" s="11"/>
+      <c r="H15" s="12"/>
       <c r="I15" t="s">
         <v>213</v>
       </c>
@@ -5770,7 +5770,7 @@
       <c r="K15" t="s">
         <v>20</v>
       </c>
-      <c r="L15" s="10"/>
+      <c r="L15" s="11"/>
       <c r="M15" t="s">
         <v>15</v>
       </c>
@@ -5813,7 +5813,7 @@
       <c r="Z15" t="s">
         <v>223</v>
       </c>
-      <c r="AA15" s="10"/>
+      <c r="AA15" s="11"/>
     </row>
     <row r="16" spans="1:29" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -5837,7 +5837,7 @@
       <c r="G16" t="s">
         <v>211</v>
       </c>
-      <c r="H16" s="11"/>
+      <c r="H16" s="12"/>
       <c r="I16" t="s">
         <v>213</v>
       </c>
@@ -5847,7 +5847,7 @@
       <c r="K16" t="s">
         <v>20</v>
       </c>
-      <c r="L16" s="10"/>
+      <c r="L16" s="11"/>
       <c r="M16" t="s">
         <v>15</v>
       </c>
@@ -5890,7 +5890,7 @@
       <c r="Z16" t="s">
         <v>223</v>
       </c>
-      <c r="AA16" s="10"/>
+      <c r="AA16" s="11"/>
     </row>
     <row r="17" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
@@ -5914,7 +5914,7 @@
       <c r="G17" t="s">
         <v>211</v>
       </c>
-      <c r="H17" s="11"/>
+      <c r="H17" s="12"/>
       <c r="I17" t="s">
         <v>213</v>
       </c>
@@ -5924,7 +5924,7 @@
       <c r="K17" t="s">
         <v>20</v>
       </c>
-      <c r="L17" s="10"/>
+      <c r="L17" s="11"/>
       <c r="M17" t="s">
         <v>15</v>
       </c>
@@ -5967,7 +5967,7 @@
       <c r="Z17" t="s">
         <v>223</v>
       </c>
-      <c r="AA17" s="10"/>
+      <c r="AA17" s="11"/>
     </row>
     <row r="18" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
@@ -5991,7 +5991,7 @@
       <c r="G18" t="s">
         <v>225</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I18" t="s">
@@ -6048,10 +6048,10 @@
       <c r="Z18" t="s">
         <v>240</v>
       </c>
-      <c r="AA18" s="10" t="s">
+      <c r="AA18" s="11" t="s">
         <v>233</v>
       </c>
-      <c r="AB18" s="10" t="s">
+      <c r="AB18" s="11" t="s">
         <v>241</v>
       </c>
     </row>
@@ -6077,7 +6077,7 @@
       <c r="G19" t="s">
         <v>225</v>
       </c>
-      <c r="H19" s="11"/>
+      <c r="H19" s="12"/>
       <c r="I19" t="s">
         <v>230</v>
       </c>
@@ -6132,8 +6132,8 @@
       <c r="Z19" t="s">
         <v>240</v>
       </c>
-      <c r="AA19" s="10"/>
-      <c r="AB19" s="10"/>
+      <c r="AA19" s="11"/>
+      <c r="AB19" s="11"/>
     </row>
     <row r="20" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
@@ -6157,7 +6157,7 @@
       <c r="G20" t="s">
         <v>225</v>
       </c>
-      <c r="H20" s="11"/>
+      <c r="H20" s="12"/>
       <c r="I20" t="s">
         <v>230</v>
       </c>
@@ -6212,8 +6212,8 @@
       <c r="Z20" t="s">
         <v>240</v>
       </c>
-      <c r="AA20" s="10"/>
-      <c r="AB20" s="10"/>
+      <c r="AA20" s="11"/>
+      <c r="AB20" s="11"/>
     </row>
     <row r="21" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
@@ -6237,7 +6237,7 @@
       <c r="G21" t="s">
         <v>225</v>
       </c>
-      <c r="H21" s="11"/>
+      <c r="H21" s="12"/>
       <c r="I21" t="s">
         <v>230</v>
       </c>
@@ -6292,8 +6292,8 @@
       <c r="Z21" t="s">
         <v>240</v>
       </c>
-      <c r="AA21" s="10"/>
-      <c r="AB21" s="10"/>
+      <c r="AA21" s="11"/>
+      <c r="AB21" s="11"/>
     </row>
     <row r="22" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
@@ -6317,7 +6317,7 @@
       <c r="G22" t="s">
         <v>243</v>
       </c>
-      <c r="H22" s="11" t="s">
+      <c r="H22" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I22" t="s">
@@ -6362,7 +6362,7 @@
       <c r="Z22" t="s">
         <v>258</v>
       </c>
-      <c r="AA22" s="10" t="s">
+      <c r="AA22" s="11" t="s">
         <v>52</v>
       </c>
     </row>
@@ -6388,7 +6388,7 @@
       <c r="G23" t="s">
         <v>243</v>
       </c>
-      <c r="H23" s="11"/>
+      <c r="H23" s="12"/>
       <c r="I23" t="s">
         <v>249</v>
       </c>
@@ -6431,7 +6431,7 @@
       <c r="Z23" t="s">
         <v>258</v>
       </c>
-      <c r="AA23" s="10"/>
+      <c r="AA23" s="11"/>
     </row>
     <row r="24" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
@@ -6455,7 +6455,7 @@
       <c r="G24" t="s">
         <v>243</v>
       </c>
-      <c r="H24" s="11"/>
+      <c r="H24" s="12"/>
       <c r="I24" t="s">
         <v>249</v>
       </c>
@@ -6498,7 +6498,7 @@
       <c r="Z24" t="s">
         <v>258</v>
       </c>
-      <c r="AA24" s="10"/>
+      <c r="AA24" s="11"/>
     </row>
     <row r="25" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
@@ -6522,7 +6522,7 @@
       <c r="G25" t="s">
         <v>243</v>
       </c>
-      <c r="H25" s="11"/>
+      <c r="H25" s="12"/>
       <c r="I25" t="s">
         <v>249</v>
       </c>
@@ -6565,7 +6565,7 @@
       <c r="Z25" t="s">
         <v>258</v>
       </c>
-      <c r="AA25" s="10"/>
+      <c r="AA25" s="11"/>
     </row>
     <row r="26" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
@@ -6589,7 +6589,7 @@
       <c r="G26" t="s">
         <v>261</v>
       </c>
-      <c r="H26" s="11" t="s">
+      <c r="H26" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I26" t="s">
@@ -6646,10 +6646,10 @@
       <c r="Z26" t="s">
         <v>278</v>
       </c>
-      <c r="AA26" s="10" t="s">
+      <c r="AA26" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="AB26" s="10" t="s">
+      <c r="AB26" s="11" t="s">
         <v>279</v>
       </c>
     </row>
@@ -6675,7 +6675,7 @@
       <c r="G27" t="s">
         <v>261</v>
       </c>
-      <c r="H27" s="11"/>
+      <c r="H27" s="12"/>
       <c r="I27" t="s">
         <v>266</v>
       </c>
@@ -6730,8 +6730,8 @@
       <c r="Z27" t="s">
         <v>278</v>
       </c>
-      <c r="AA27" s="10"/>
-      <c r="AB27" s="10"/>
+      <c r="AA27" s="11"/>
+      <c r="AB27" s="11"/>
     </row>
     <row r="28" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
@@ -6755,7 +6755,7 @@
       <c r="G28" t="s">
         <v>261</v>
       </c>
-      <c r="H28" s="11"/>
+      <c r="H28" s="12"/>
       <c r="I28" t="s">
         <v>266</v>
       </c>
@@ -6810,8 +6810,8 @@
       <c r="Z28" t="s">
         <v>278</v>
       </c>
-      <c r="AA28" s="10"/>
-      <c r="AB28" s="10"/>
+      <c r="AA28" s="11"/>
+      <c r="AB28" s="11"/>
     </row>
     <row r="29" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
@@ -6835,7 +6835,7 @@
       <c r="G29" t="s">
         <v>261</v>
       </c>
-      <c r="H29" s="11"/>
+      <c r="H29" s="12"/>
       <c r="I29" t="s">
         <v>266</v>
       </c>
@@ -6890,8 +6890,8 @@
       <c r="Z29" t="s">
         <v>278</v>
       </c>
-      <c r="AA29" s="10"/>
-      <c r="AB29" s="10"/>
+      <c r="AA29" s="11"/>
+      <c r="AB29" s="11"/>
     </row>
     <row r="30" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
@@ -6915,7 +6915,7 @@
       <c r="G30" t="s">
         <v>282</v>
       </c>
-      <c r="H30" s="11" t="s">
+      <c r="H30" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I30" t="s">
@@ -6972,10 +6972,10 @@
       <c r="Z30" t="s">
         <v>298</v>
       </c>
-      <c r="AA30" s="10" t="s">
+      <c r="AA30" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="AB30" s="10" t="s">
+      <c r="AB30" s="11" t="s">
         <v>299</v>
       </c>
     </row>
@@ -7001,7 +7001,7 @@
       <c r="G31" t="s">
         <v>282</v>
       </c>
-      <c r="H31" s="11"/>
+      <c r="H31" s="12"/>
       <c r="I31" t="s">
         <v>287</v>
       </c>
@@ -7056,8 +7056,8 @@
       <c r="Z31" t="s">
         <v>298</v>
       </c>
-      <c r="AA31" s="10"/>
-      <c r="AB31" s="10"/>
+      <c r="AA31" s="11"/>
+      <c r="AB31" s="11"/>
     </row>
     <row r="32" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
@@ -7081,7 +7081,7 @@
       <c r="G32" t="s">
         <v>282</v>
       </c>
-      <c r="H32" s="11"/>
+      <c r="H32" s="12"/>
       <c r="I32" t="s">
         <v>287</v>
       </c>
@@ -7136,8 +7136,8 @@
       <c r="Z32" t="s">
         <v>298</v>
       </c>
-      <c r="AA32" s="10"/>
-      <c r="AB32" s="10"/>
+      <c r="AA32" s="11"/>
+      <c r="AB32" s="11"/>
     </row>
     <row r="33" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
@@ -7161,7 +7161,7 @@
       <c r="G33" t="s">
         <v>282</v>
       </c>
-      <c r="H33" s="11"/>
+      <c r="H33" s="12"/>
       <c r="I33" t="s">
         <v>287</v>
       </c>
@@ -7216,8 +7216,8 @@
       <c r="Z33" t="s">
         <v>298</v>
       </c>
-      <c r="AA33" s="10"/>
-      <c r="AB33" s="10"/>
+      <c r="AA33" s="11"/>
+      <c r="AB33" s="11"/>
     </row>
     <row r="34" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
@@ -7241,7 +7241,7 @@
       <c r="G34" t="s">
         <v>302</v>
       </c>
-      <c r="H34" s="11" t="s">
+      <c r="H34" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I34" t="s">
@@ -7286,7 +7286,7 @@
       <c r="Z34" t="s">
         <v>315</v>
       </c>
-      <c r="AA34" s="10" t="s">
+      <c r="AA34" s="11" t="s">
         <v>835</v>
       </c>
     </row>
@@ -7312,7 +7312,7 @@
       <c r="G35" t="s">
         <v>302</v>
       </c>
-      <c r="H35" s="11"/>
+      <c r="H35" s="12"/>
       <c r="I35" t="s">
         <v>306</v>
       </c>
@@ -7355,7 +7355,7 @@
       <c r="Z35" t="s">
         <v>315</v>
       </c>
-      <c r="AA35" s="10"/>
+      <c r="AA35" s="11"/>
     </row>
     <row r="36" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
@@ -7379,7 +7379,7 @@
       <c r="G36" t="s">
         <v>302</v>
       </c>
-      <c r="H36" s="11"/>
+      <c r="H36" s="12"/>
       <c r="I36" t="s">
         <v>306</v>
       </c>
@@ -7422,7 +7422,7 @@
       <c r="Z36" t="s">
         <v>315</v>
       </c>
-      <c r="AA36" s="10"/>
+      <c r="AA36" s="11"/>
     </row>
     <row r="37" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
@@ -7446,7 +7446,7 @@
       <c r="G37" t="s">
         <v>302</v>
       </c>
-      <c r="H37" s="11"/>
+      <c r="H37" s="12"/>
       <c r="I37" t="s">
         <v>306</v>
       </c>
@@ -7489,7 +7489,7 @@
       <c r="Z37" t="s">
         <v>315</v>
       </c>
-      <c r="AA37" s="10"/>
+      <c r="AA37" s="11"/>
     </row>
     <row r="38" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
@@ -7513,7 +7513,7 @@
       <c r="G38" t="s">
         <v>318</v>
       </c>
-      <c r="H38" s="11" t="s">
+      <c r="H38" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I38" t="s">
@@ -7558,7 +7558,7 @@
       <c r="Z38" t="s">
         <v>330</v>
       </c>
-      <c r="AA38" s="10" t="s">
+      <c r="AA38" s="11" t="s">
         <v>834</v>
       </c>
     </row>
@@ -7584,7 +7584,7 @@
       <c r="G39" t="s">
         <v>318</v>
       </c>
-      <c r="H39" s="11"/>
+      <c r="H39" s="12"/>
       <c r="I39" t="s">
         <v>322</v>
       </c>
@@ -7627,7 +7627,7 @@
       <c r="Z39" t="s">
         <v>330</v>
       </c>
-      <c r="AA39" s="10"/>
+      <c r="AA39" s="11"/>
     </row>
     <row r="40" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
@@ -7651,7 +7651,7 @@
       <c r="G40" t="s">
         <v>318</v>
       </c>
-      <c r="H40" s="11"/>
+      <c r="H40" s="12"/>
       <c r="I40" t="s">
         <v>322</v>
       </c>
@@ -7694,7 +7694,7 @@
       <c r="Z40" t="s">
         <v>330</v>
       </c>
-      <c r="AA40" s="10"/>
+      <c r="AA40" s="11"/>
     </row>
     <row r="41" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
@@ -7718,7 +7718,7 @@
       <c r="G41" t="s">
         <v>318</v>
       </c>
-      <c r="H41" s="11"/>
+      <c r="H41" s="12"/>
       <c r="I41" t="s">
         <v>322</v>
       </c>
@@ -7761,7 +7761,7 @@
       <c r="Z41" t="s">
         <v>330</v>
       </c>
-      <c r="AA41" s="10"/>
+      <c r="AA41" s="11"/>
     </row>
     <row r="42" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
@@ -7785,7 +7785,7 @@
       <c r="G42" t="s">
         <v>332</v>
       </c>
-      <c r="H42" s="11" t="s">
+      <c r="H42" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I42" t="s">
@@ -7830,7 +7830,7 @@
       <c r="Z42" t="s">
         <v>346</v>
       </c>
-      <c r="AA42" s="10" t="s">
+      <c r="AA42" s="11" t="s">
         <v>338</v>
       </c>
     </row>
@@ -7856,7 +7856,7 @@
       <c r="G43" t="s">
         <v>332</v>
       </c>
-      <c r="H43" s="11"/>
+      <c r="H43" s="12"/>
       <c r="I43" t="s">
         <v>336</v>
       </c>
@@ -7899,7 +7899,7 @@
       <c r="Z43" t="s">
         <v>346</v>
       </c>
-      <c r="AA43" s="10"/>
+      <c r="AA43" s="11"/>
     </row>
     <row r="44" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
@@ -7923,7 +7923,7 @@
       <c r="G44" t="s">
         <v>332</v>
       </c>
-      <c r="H44" s="11"/>
+      <c r="H44" s="12"/>
       <c r="I44" t="s">
         <v>336</v>
       </c>
@@ -7966,7 +7966,7 @@
       <c r="Z44" t="s">
         <v>346</v>
       </c>
-      <c r="AA44" s="10"/>
+      <c r="AA44" s="11"/>
     </row>
     <row r="45" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
@@ -7990,7 +7990,7 @@
       <c r="G45" t="s">
         <v>332</v>
       </c>
-      <c r="H45" s="11"/>
+      <c r="H45" s="12"/>
       <c r="I45" t="s">
         <v>336</v>
       </c>
@@ -8033,7 +8033,7 @@
       <c r="Z45" t="s">
         <v>346</v>
       </c>
-      <c r="AA45" s="10"/>
+      <c r="AA45" s="11"/>
     </row>
     <row r="46" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
@@ -8057,7 +8057,7 @@
       <c r="G46" t="s">
         <v>348</v>
       </c>
-      <c r="H46" s="11" t="s">
+      <c r="H46" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I46" t="s">
@@ -8102,7 +8102,7 @@
       <c r="Z46" t="s">
         <v>362</v>
       </c>
-      <c r="AA46" s="10" t="s">
+      <c r="AA46" s="11" t="s">
         <v>355</v>
       </c>
     </row>
@@ -8128,7 +8128,7 @@
       <c r="G47" t="s">
         <v>348</v>
       </c>
-      <c r="H47" s="11"/>
+      <c r="H47" s="12"/>
       <c r="I47" t="s">
         <v>353</v>
       </c>
@@ -8171,7 +8171,7 @@
       <c r="Z47" t="s">
         <v>362</v>
       </c>
-      <c r="AA47" s="10"/>
+      <c r="AA47" s="11"/>
     </row>
     <row r="48" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
@@ -8195,7 +8195,7 @@
       <c r="G48" t="s">
         <v>348</v>
       </c>
-      <c r="H48" s="11"/>
+      <c r="H48" s="12"/>
       <c r="I48" t="s">
         <v>353</v>
       </c>
@@ -8238,7 +8238,7 @@
       <c r="Z48" t="s">
         <v>362</v>
       </c>
-      <c r="AA48" s="10"/>
+      <c r="AA48" s="11"/>
     </row>
     <row r="49" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
@@ -8262,7 +8262,7 @@
       <c r="G49" t="s">
         <v>348</v>
       </c>
-      <c r="H49" s="11"/>
+      <c r="H49" s="12"/>
       <c r="I49" t="s">
         <v>353</v>
       </c>
@@ -8305,7 +8305,7 @@
       <c r="Z49" t="s">
         <v>362</v>
       </c>
-      <c r="AA49" s="10"/>
+      <c r="AA49" s="11"/>
     </row>
     <row r="50" spans="1:28" ht="72" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
@@ -8329,7 +8329,7 @@
       <c r="G50" t="s">
         <v>364</v>
       </c>
-      <c r="H50" s="11" t="s">
+      <c r="H50" s="12" t="s">
         <v>369</v>
       </c>
       <c r="I50" t="s">
@@ -8386,7 +8386,7 @@
       <c r="Z50" t="s">
         <v>382</v>
       </c>
-      <c r="AA50" s="10" t="s">
+      <c r="AA50" s="11" t="s">
         <v>375</v>
       </c>
     </row>
@@ -8412,7 +8412,7 @@
       <c r="G51" t="s">
         <v>364</v>
       </c>
-      <c r="H51" s="11"/>
+      <c r="H51" s="12"/>
       <c r="I51" t="s">
         <v>371</v>
       </c>
@@ -8467,7 +8467,7 @@
       <c r="Z51" t="s">
         <v>382</v>
       </c>
-      <c r="AA51" s="10"/>
+      <c r="AA51" s="11"/>
     </row>
     <row r="52" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
@@ -8491,7 +8491,7 @@
       <c r="G52" t="s">
         <v>364</v>
       </c>
-      <c r="H52" s="11"/>
+      <c r="H52" s="12"/>
       <c r="I52" t="s">
         <v>371</v>
       </c>
@@ -8546,7 +8546,7 @@
       <c r="Z52" t="s">
         <v>382</v>
       </c>
-      <c r="AA52" s="10"/>
+      <c r="AA52" s="11"/>
     </row>
     <row r="53" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
@@ -8570,7 +8570,7 @@
       <c r="G53" t="s">
         <v>364</v>
       </c>
-      <c r="H53" s="11"/>
+      <c r="H53" s="12"/>
       <c r="I53" t="s">
         <v>371</v>
       </c>
@@ -8625,7 +8625,7 @@
       <c r="Z53" t="s">
         <v>382</v>
       </c>
-      <c r="AA53" s="10"/>
+      <c r="AA53" s="11"/>
     </row>
     <row r="54" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
@@ -8649,7 +8649,7 @@
       <c r="G54" t="s">
         <v>385</v>
       </c>
-      <c r="H54" s="11" t="s">
+      <c r="H54" s="12" t="s">
         <v>68</v>
       </c>
       <c r="I54" t="s">
@@ -8694,10 +8694,10 @@
       <c r="Z54" t="s">
         <v>398</v>
       </c>
-      <c r="AA54" s="10" t="s">
+      <c r="AA54" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="AB54" s="10" t="s">
+      <c r="AB54" s="11" t="s">
         <v>399</v>
       </c>
     </row>
@@ -8723,7 +8723,7 @@
       <c r="G55" t="s">
         <v>385</v>
       </c>
-      <c r="H55" s="11"/>
+      <c r="H55" s="12"/>
       <c r="I55" t="s">
         <v>392</v>
       </c>
@@ -8766,8 +8766,8 @@
       <c r="Z55" t="s">
         <v>398</v>
       </c>
-      <c r="AA55" s="10"/>
-      <c r="AB55" s="10"/>
+      <c r="AA55" s="11"/>
+      <c r="AB55" s="11"/>
     </row>
     <row r="56" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
@@ -8791,7 +8791,7 @@
       <c r="G56" t="s">
         <v>385</v>
       </c>
-      <c r="H56" s="11"/>
+      <c r="H56" s="12"/>
       <c r="I56" t="s">
         <v>392</v>
       </c>
@@ -8834,8 +8834,8 @@
       <c r="Z56" t="s">
         <v>398</v>
       </c>
-      <c r="AA56" s="10"/>
-      <c r="AB56" s="10"/>
+      <c r="AA56" s="11"/>
+      <c r="AB56" s="11"/>
     </row>
     <row r="57" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
@@ -8859,7 +8859,7 @@
       <c r="G57" t="s">
         <v>385</v>
       </c>
-      <c r="H57" s="11"/>
+      <c r="H57" s="12"/>
       <c r="I57" t="s">
         <v>392</v>
       </c>
@@ -8902,8 +8902,8 @@
       <c r="Z57" t="s">
         <v>398</v>
       </c>
-      <c r="AA57" s="10"/>
-      <c r="AB57" s="10"/>
+      <c r="AA57" s="11"/>
+      <c r="AB57" s="11"/>
     </row>
     <row r="58" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
@@ -8927,7 +8927,7 @@
       <c r="G58" t="s">
         <v>402</v>
       </c>
-      <c r="H58" s="11" t="s">
+      <c r="H58" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I58" t="s">
@@ -8984,7 +8984,7 @@
       <c r="Z58" t="s">
         <v>417</v>
       </c>
-      <c r="AA58" s="10" t="s">
+      <c r="AA58" s="11" t="s">
         <v>72</v>
       </c>
     </row>
@@ -9010,7 +9010,7 @@
       <c r="G59" t="s">
         <v>402</v>
       </c>
-      <c r="H59" s="11"/>
+      <c r="H59" s="12"/>
       <c r="I59" t="s">
         <v>407</v>
       </c>
@@ -9065,7 +9065,7 @@
       <c r="Z59" t="s">
         <v>417</v>
       </c>
-      <c r="AA59" s="10"/>
+      <c r="AA59" s="11"/>
     </row>
     <row r="60" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
@@ -9089,7 +9089,7 @@
       <c r="G60" t="s">
         <v>402</v>
       </c>
-      <c r="H60" s="11"/>
+      <c r="H60" s="12"/>
       <c r="I60" t="s">
         <v>407</v>
       </c>
@@ -9144,7 +9144,7 @@
       <c r="Z60" t="s">
         <v>417</v>
       </c>
-      <c r="AA60" s="10"/>
+      <c r="AA60" s="11"/>
     </row>
     <row r="61" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
@@ -9168,7 +9168,7 @@
       <c r="G61" t="s">
         <v>402</v>
       </c>
-      <c r="H61" s="11"/>
+      <c r="H61" s="12"/>
       <c r="I61" t="s">
         <v>407</v>
       </c>
@@ -9223,7 +9223,7 @@
       <c r="Z61" t="s">
         <v>417</v>
       </c>
-      <c r="AA61" s="10"/>
+      <c r="AA61" s="11"/>
     </row>
     <row r="62" spans="1:28" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
@@ -9247,7 +9247,7 @@
       <c r="G62" t="s">
         <v>75</v>
       </c>
-      <c r="H62" s="11" t="s">
+      <c r="H62" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I62" t="s">
@@ -9304,10 +9304,10 @@
       <c r="Z62" t="s">
         <v>426</v>
       </c>
-      <c r="AA62" s="10" t="s">
+      <c r="AA62" s="11" t="s">
         <v>83</v>
       </c>
-      <c r="AB62" s="10" t="s">
+      <c r="AB62" s="11" t="s">
         <v>418</v>
       </c>
     </row>
@@ -9333,7 +9333,7 @@
       <c r="G63" t="s">
         <v>75</v>
       </c>
-      <c r="H63" s="11"/>
+      <c r="H63" s="12"/>
       <c r="I63" t="s">
         <v>80</v>
       </c>
@@ -9388,8 +9388,8 @@
       <c r="Z63" t="s">
         <v>426</v>
       </c>
-      <c r="AA63" s="10"/>
-      <c r="AB63" s="10"/>
+      <c r="AA63" s="11"/>
+      <c r="AB63" s="11"/>
     </row>
     <row r="64" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
@@ -9413,7 +9413,7 @@
       <c r="G64" t="s">
         <v>75</v>
       </c>
-      <c r="H64" s="11"/>
+      <c r="H64" s="12"/>
       <c r="I64" t="s">
         <v>80</v>
       </c>
@@ -9468,8 +9468,8 @@
       <c r="Z64" t="s">
         <v>426</v>
       </c>
-      <c r="AA64" s="10"/>
-      <c r="AB64" s="10"/>
+      <c r="AA64" s="11"/>
+      <c r="AB64" s="11"/>
     </row>
     <row r="65" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
@@ -9493,7 +9493,7 @@
       <c r="G65" t="s">
         <v>75</v>
       </c>
-      <c r="H65" s="11"/>
+      <c r="H65" s="12"/>
       <c r="I65" t="s">
         <v>80</v>
       </c>
@@ -9548,8 +9548,8 @@
       <c r="Z65" t="s">
         <v>426</v>
       </c>
-      <c r="AA65" s="10"/>
-      <c r="AB65" s="10"/>
+      <c r="AA65" s="11"/>
+      <c r="AB65" s="11"/>
     </row>
     <row r="66" spans="1:28" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
@@ -9573,7 +9573,7 @@
       <c r="G66" t="s">
         <v>428</v>
       </c>
-      <c r="H66" s="11" t="s">
+      <c r="H66" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I66" t="s">
@@ -9630,7 +9630,7 @@
       <c r="Z66" t="s">
         <v>442</v>
       </c>
-      <c r="AA66" s="10" t="s">
+      <c r="AA66" s="11" t="s">
         <v>434</v>
       </c>
     </row>
@@ -9656,7 +9656,7 @@
       <c r="G67" t="s">
         <v>428</v>
       </c>
-      <c r="H67" s="11"/>
+      <c r="H67" s="12"/>
       <c r="I67" t="s">
         <v>432</v>
       </c>
@@ -9711,7 +9711,7 @@
       <c r="Z67" t="s">
         <v>442</v>
       </c>
-      <c r="AA67" s="10"/>
+      <c r="AA67" s="11"/>
     </row>
     <row r="68" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
@@ -9735,7 +9735,7 @@
       <c r="G68" t="s">
         <v>428</v>
       </c>
-      <c r="H68" s="11"/>
+      <c r="H68" s="12"/>
       <c r="I68" t="s">
         <v>432</v>
       </c>
@@ -9790,7 +9790,7 @@
       <c r="Z68" t="s">
         <v>442</v>
       </c>
-      <c r="AA68" s="10"/>
+      <c r="AA68" s="11"/>
     </row>
     <row r="69" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
@@ -9814,7 +9814,7 @@
       <c r="G69" t="s">
         <v>428</v>
       </c>
-      <c r="H69" s="11"/>
+      <c r="H69" s="12"/>
       <c r="I69" t="s">
         <v>432</v>
       </c>
@@ -9869,7 +9869,7 @@
       <c r="Z69" t="s">
         <v>442</v>
       </c>
-      <c r="AA69" s="10"/>
+      <c r="AA69" s="11"/>
     </row>
     <row r="70" spans="1:28" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
@@ -9893,7 +9893,7 @@
       <c r="G70" t="s">
         <v>445</v>
       </c>
-      <c r="H70" s="11" t="s">
+      <c r="H70" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I70" t="s">
@@ -9950,7 +9950,7 @@
       <c r="Z70" t="s">
         <v>461</v>
       </c>
-      <c r="AA70" s="10" t="s">
+      <c r="AA70" s="11" t="s">
         <v>454</v>
       </c>
     </row>
@@ -9976,7 +9976,7 @@
       <c r="G71" t="s">
         <v>445</v>
       </c>
-      <c r="H71" s="11"/>
+      <c r="H71" s="12"/>
       <c r="I71" t="s">
         <v>450</v>
       </c>
@@ -10031,7 +10031,7 @@
       <c r="Z71" t="s">
         <v>461</v>
       </c>
-      <c r="AA71" s="10"/>
+      <c r="AA71" s="11"/>
     </row>
     <row r="72" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
@@ -10055,7 +10055,7 @@
       <c r="G72" t="s">
         <v>445</v>
       </c>
-      <c r="H72" s="11"/>
+      <c r="H72" s="12"/>
       <c r="I72" t="s">
         <v>450</v>
       </c>
@@ -10110,7 +10110,7 @@
       <c r="Z72" t="s">
         <v>461</v>
       </c>
-      <c r="AA72" s="10"/>
+      <c r="AA72" s="11"/>
     </row>
     <row r="73" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
@@ -10134,7 +10134,7 @@
       <c r="G73" t="s">
         <v>445</v>
       </c>
-      <c r="H73" s="11"/>
+      <c r="H73" s="12"/>
       <c r="I73" t="s">
         <v>450</v>
       </c>
@@ -10189,7 +10189,7 @@
       <c r="Z73" t="s">
         <v>461</v>
       </c>
-      <c r="AA73" s="10"/>
+      <c r="AA73" s="11"/>
     </row>
     <row r="74" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
@@ -10213,7 +10213,7 @@
       <c r="G74" t="s">
         <v>463</v>
       </c>
-      <c r="H74" s="11" t="s">
+      <c r="H74" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I74" t="s">
@@ -10258,7 +10258,7 @@
       <c r="Z74" t="s">
         <v>477</v>
       </c>
-      <c r="AA74" s="10" t="s">
+      <c r="AA74" s="11" t="s">
         <v>470</v>
       </c>
     </row>
@@ -10284,7 +10284,7 @@
       <c r="G75" t="s">
         <v>463</v>
       </c>
-      <c r="H75" s="11"/>
+      <c r="H75" s="12"/>
       <c r="I75" t="s">
         <v>468</v>
       </c>
@@ -10327,7 +10327,7 @@
       <c r="Z75" t="s">
         <v>477</v>
       </c>
-      <c r="AA75" s="10"/>
+      <c r="AA75" s="11"/>
     </row>
     <row r="76" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
@@ -10351,7 +10351,7 @@
       <c r="G76" t="s">
         <v>463</v>
       </c>
-      <c r="H76" s="11"/>
+      <c r="H76" s="12"/>
       <c r="I76" t="s">
         <v>468</v>
       </c>
@@ -10394,7 +10394,7 @@
       <c r="Z76" t="s">
         <v>477</v>
       </c>
-      <c r="AA76" s="10"/>
+      <c r="AA76" s="11"/>
     </row>
     <row r="77" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
@@ -10418,7 +10418,7 @@
       <c r="G77" t="s">
         <v>463</v>
       </c>
-      <c r="H77" s="11"/>
+      <c r="H77" s="12"/>
       <c r="I77" t="s">
         <v>468</v>
       </c>
@@ -10461,7 +10461,7 @@
       <c r="Z77" t="s">
         <v>477</v>
       </c>
-      <c r="AA77" s="10"/>
+      <c r="AA77" s="11"/>
     </row>
     <row r="78" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
@@ -10485,7 +10485,7 @@
       <c r="G78" t="s">
         <v>480</v>
       </c>
-      <c r="H78" s="11" t="s">
+      <c r="H78" s="12" t="s">
         <v>486</v>
       </c>
       <c r="I78" t="s">
@@ -10530,7 +10530,7 @@
       <c r="Z78" t="s">
         <v>496</v>
       </c>
-      <c r="AA78" s="10" t="s">
+      <c r="AA78" s="11" t="s">
         <v>478</v>
       </c>
     </row>
@@ -10556,7 +10556,7 @@
       <c r="G79" t="s">
         <v>480</v>
       </c>
-      <c r="H79" s="11"/>
+      <c r="H79" s="12"/>
       <c r="I79" t="s">
         <v>487</v>
       </c>
@@ -10599,7 +10599,7 @@
       <c r="Z79" t="s">
         <v>496</v>
       </c>
-      <c r="AA79" s="10"/>
+      <c r="AA79" s="11"/>
     </row>
     <row r="80" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
@@ -10623,7 +10623,7 @@
       <c r="G80" t="s">
         <v>480</v>
       </c>
-      <c r="H80" s="11"/>
+      <c r="H80" s="12"/>
       <c r="I80" t="s">
         <v>487</v>
       </c>
@@ -10666,7 +10666,7 @@
       <c r="Z80" t="s">
         <v>496</v>
       </c>
-      <c r="AA80" s="10"/>
+      <c r="AA80" s="11"/>
     </row>
     <row r="81" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
@@ -10690,7 +10690,7 @@
       <c r="G81" t="s">
         <v>480</v>
       </c>
-      <c r="H81" s="11"/>
+      <c r="H81" s="12"/>
       <c r="I81" t="s">
         <v>487</v>
       </c>
@@ -10733,7 +10733,7 @@
       <c r="Z81" t="s">
         <v>496</v>
       </c>
-      <c r="AA81" s="10"/>
+      <c r="AA81" s="11"/>
     </row>
     <row r="82" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
@@ -10757,7 +10757,7 @@
       <c r="G82" t="s">
         <v>498</v>
       </c>
-      <c r="H82" s="11" t="s">
+      <c r="H82" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I82" t="s">
@@ -10802,7 +10802,7 @@
       <c r="Z82" t="s">
         <v>511</v>
       </c>
-      <c r="AA82" s="10" t="s">
+      <c r="AA82" s="11" t="s">
         <v>90</v>
       </c>
     </row>
@@ -10828,7 +10828,7 @@
       <c r="G83" t="s">
         <v>498</v>
       </c>
-      <c r="H83" s="11"/>
+      <c r="H83" s="12"/>
       <c r="I83" t="s">
         <v>503</v>
       </c>
@@ -10871,7 +10871,7 @@
       <c r="Z83" t="s">
         <v>511</v>
       </c>
-      <c r="AA83" s="10"/>
+      <c r="AA83" s="11"/>
     </row>
     <row r="84" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
@@ -10895,7 +10895,7 @@
       <c r="G84" t="s">
         <v>498</v>
       </c>
-      <c r="H84" s="11"/>
+      <c r="H84" s="12"/>
       <c r="I84" t="s">
         <v>503</v>
       </c>
@@ -10938,7 +10938,7 @@
       <c r="Z84" t="s">
         <v>511</v>
       </c>
-      <c r="AA84" s="10"/>
+      <c r="AA84" s="11"/>
     </row>
     <row r="85" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
@@ -10962,7 +10962,7 @@
       <c r="G85" t="s">
         <v>498</v>
       </c>
-      <c r="H85" s="11"/>
+      <c r="H85" s="12"/>
       <c r="I85" t="s">
         <v>503</v>
       </c>
@@ -11005,7 +11005,7 @@
       <c r="Z85" t="s">
         <v>511</v>
       </c>
-      <c r="AA85" s="10"/>
+      <c r="AA85" s="11"/>
     </row>
     <row r="86" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
@@ -11029,7 +11029,7 @@
       <c r="G86" t="s">
         <v>514</v>
       </c>
-      <c r="H86" s="11" t="s">
+      <c r="H86" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I86" t="s">
@@ -11074,7 +11074,7 @@
       <c r="Z86" t="s">
         <v>526</v>
       </c>
-      <c r="AA86" s="10" t="s">
+      <c r="AA86" s="11" t="s">
         <v>92</v>
       </c>
     </row>
@@ -11100,7 +11100,7 @@
       <c r="G87" t="s">
         <v>514</v>
       </c>
-      <c r="H87" s="11"/>
+      <c r="H87" s="12"/>
       <c r="I87" t="s">
         <v>518</v>
       </c>
@@ -11143,7 +11143,7 @@
       <c r="Z87" t="s">
         <v>526</v>
       </c>
-      <c r="AA87" s="10"/>
+      <c r="AA87" s="11"/>
     </row>
     <row r="88" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
@@ -11167,7 +11167,7 @@
       <c r="G88" t="s">
         <v>514</v>
       </c>
-      <c r="H88" s="11"/>
+      <c r="H88" s="12"/>
       <c r="I88" t="s">
         <v>518</v>
       </c>
@@ -11210,7 +11210,7 @@
       <c r="Z88" t="s">
         <v>526</v>
       </c>
-      <c r="AA88" s="10"/>
+      <c r="AA88" s="11"/>
     </row>
     <row r="89" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
@@ -11234,7 +11234,7 @@
       <c r="G89" t="s">
         <v>514</v>
       </c>
-      <c r="H89" s="11"/>
+      <c r="H89" s="12"/>
       <c r="I89" t="s">
         <v>518</v>
       </c>
@@ -11277,7 +11277,7 @@
       <c r="Z89" t="s">
         <v>526</v>
       </c>
-      <c r="AA89" s="10"/>
+      <c r="AA89" s="11"/>
     </row>
     <row r="90" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
@@ -11301,7 +11301,7 @@
       <c r="G90" t="s">
         <v>530</v>
       </c>
-      <c r="H90" s="11" t="s">
+      <c r="H90" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I90" t="s">
@@ -11313,7 +11313,7 @@
       <c r="K90" t="s">
         <v>20</v>
       </c>
-      <c r="L90" s="10" t="s">
+      <c r="L90" s="11" t="s">
         <v>536</v>
       </c>
       <c r="M90" t="s">
@@ -11358,7 +11358,7 @@
       <c r="Z90" t="s">
         <v>546</v>
       </c>
-      <c r="AA90" s="10" t="s">
+      <c r="AA90" s="11" t="s">
         <v>114</v>
       </c>
       <c r="AB90" s="5"/>
@@ -11385,7 +11385,7 @@
       <c r="G91" t="s">
         <v>530</v>
       </c>
-      <c r="H91" s="11"/>
+      <c r="H91" s="12"/>
       <c r="I91" t="s">
         <v>534</v>
       </c>
@@ -11395,7 +11395,7 @@
       <c r="K91" t="s">
         <v>20</v>
       </c>
-      <c r="L91" s="10"/>
+      <c r="L91" s="11"/>
       <c r="M91" t="s">
         <v>16</v>
       </c>
@@ -11438,7 +11438,7 @@
       <c r="Z91" t="s">
         <v>546</v>
       </c>
-      <c r="AA91" s="10"/>
+      <c r="AA91" s="11"/>
       <c r="AB91" s="5"/>
     </row>
     <row r="92" spans="1:28" x14ac:dyDescent="0.3">
@@ -11463,7 +11463,7 @@
       <c r="G92" t="s">
         <v>530</v>
       </c>
-      <c r="H92" s="11"/>
+      <c r="H92" s="12"/>
       <c r="I92" t="s">
         <v>534</v>
       </c>
@@ -11473,7 +11473,7 @@
       <c r="K92" t="s">
         <v>20</v>
       </c>
-      <c r="L92" s="10"/>
+      <c r="L92" s="11"/>
       <c r="M92" t="s">
         <v>16</v>
       </c>
@@ -11516,7 +11516,7 @@
       <c r="Z92" t="s">
         <v>546</v>
       </c>
-      <c r="AA92" s="10"/>
+      <c r="AA92" s="11"/>
       <c r="AB92" s="5"/>
     </row>
     <row r="93" spans="1:28" x14ac:dyDescent="0.3">
@@ -11541,7 +11541,7 @@
       <c r="G93" t="s">
         <v>530</v>
       </c>
-      <c r="H93" s="11"/>
+      <c r="H93" s="12"/>
       <c r="I93" t="s">
         <v>534</v>
       </c>
@@ -11551,7 +11551,7 @@
       <c r="K93" t="s">
         <v>20</v>
       </c>
-      <c r="L93" s="10"/>
+      <c r="L93" s="11"/>
       <c r="M93" t="s">
         <v>16</v>
       </c>
@@ -11594,7 +11594,7 @@
       <c r="Z93" t="s">
         <v>546</v>
       </c>
-      <c r="AA93" s="10"/>
+      <c r="AA93" s="11"/>
       <c r="AB93" s="5"/>
     </row>
     <row r="94" spans="1:28" ht="144" customHeight="1" x14ac:dyDescent="0.3">
@@ -11619,7 +11619,7 @@
       <c r="G94" t="s">
         <v>552</v>
       </c>
-      <c r="H94" s="11" t="s">
+      <c r="H94" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I94" t="s">
@@ -11676,7 +11676,7 @@
       <c r="Z94" t="s">
         <v>561</v>
       </c>
-      <c r="AA94" s="10" t="s">
+      <c r="AA94" s="11" t="s">
         <v>96</v>
       </c>
     </row>
@@ -11702,7 +11702,7 @@
       <c r="G95" t="s">
         <v>552</v>
       </c>
-      <c r="H95" s="11"/>
+      <c r="H95" s="12"/>
       <c r="I95" t="s">
         <v>553</v>
       </c>
@@ -11757,7 +11757,7 @@
       <c r="Z95" t="s">
         <v>561</v>
       </c>
-      <c r="AA95" s="10"/>
+      <c r="AA95" s="11"/>
     </row>
     <row r="96" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
@@ -11781,7 +11781,7 @@
       <c r="G96" t="s">
         <v>552</v>
       </c>
-      <c r="H96" s="11"/>
+      <c r="H96" s="12"/>
       <c r="I96" t="s">
         <v>553</v>
       </c>
@@ -11836,7 +11836,7 @@
       <c r="Z96" t="s">
         <v>561</v>
       </c>
-      <c r="AA96" s="10"/>
+      <c r="AA96" s="11"/>
     </row>
     <row r="97" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
@@ -11860,7 +11860,7 @@
       <c r="G97" t="s">
         <v>552</v>
       </c>
-      <c r="H97" s="11"/>
+      <c r="H97" s="12"/>
       <c r="I97" t="s">
         <v>553</v>
       </c>
@@ -11915,7 +11915,7 @@
       <c r="Z97" t="s">
         <v>561</v>
       </c>
-      <c r="AA97" s="10"/>
+      <c r="AA97" s="11"/>
     </row>
     <row r="98" spans="1:27" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
@@ -11939,7 +11939,7 @@
       <c r="G98" t="s">
         <v>568</v>
       </c>
-      <c r="H98" s="11" t="s">
+      <c r="H98" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I98" t="s">
@@ -11996,7 +11996,7 @@
       <c r="Z98" t="s">
         <v>580</v>
       </c>
-      <c r="AA98" s="10" t="s">
+      <c r="AA98" s="11" t="s">
         <v>572</v>
       </c>
     </row>
@@ -12022,7 +12022,7 @@
       <c r="G99" t="s">
         <v>568</v>
       </c>
-      <c r="H99" s="11"/>
+      <c r="H99" s="12"/>
       <c r="I99" t="s">
         <v>569</v>
       </c>
@@ -12077,7 +12077,7 @@
       <c r="Z99" t="s">
         <v>580</v>
       </c>
-      <c r="AA99" s="10"/>
+      <c r="AA99" s="11"/>
     </row>
     <row r="100" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
@@ -12101,7 +12101,7 @@
       <c r="G100" t="s">
         <v>568</v>
       </c>
-      <c r="H100" s="11"/>
+      <c r="H100" s="12"/>
       <c r="I100" t="s">
         <v>569</v>
       </c>
@@ -12156,7 +12156,7 @@
       <c r="Z100" t="s">
         <v>580</v>
       </c>
-      <c r="AA100" s="10"/>
+      <c r="AA100" s="11"/>
     </row>
     <row r="101" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
@@ -12180,7 +12180,7 @@
       <c r="G101" t="s">
         <v>568</v>
       </c>
-      <c r="H101" s="11"/>
+      <c r="H101" s="12"/>
       <c r="I101" t="s">
         <v>569</v>
       </c>
@@ -12235,7 +12235,7 @@
       <c r="Z101" t="s">
         <v>580</v>
       </c>
-      <c r="AA101" s="10"/>
+      <c r="AA101" s="11"/>
     </row>
     <row r="102" spans="1:27" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
@@ -12259,7 +12259,7 @@
       <c r="G102" t="s">
         <v>587</v>
       </c>
-      <c r="H102" s="11" t="s">
+      <c r="H102" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I102" t="s">
@@ -12316,7 +12316,7 @@
       <c r="Z102" t="s">
         <v>596</v>
       </c>
-      <c r="AA102" s="10" t="s">
+      <c r="AA102" s="11" t="s">
         <v>100</v>
       </c>
     </row>
@@ -12342,7 +12342,7 @@
       <c r="G103" t="s">
         <v>587</v>
       </c>
-      <c r="H103" s="11"/>
+      <c r="H103" s="12"/>
       <c r="I103" t="s">
         <v>583</v>
       </c>
@@ -12397,7 +12397,7 @@
       <c r="Z103" t="s">
         <v>596</v>
       </c>
-      <c r="AA103" s="10"/>
+      <c r="AA103" s="11"/>
     </row>
     <row r="104" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
@@ -12421,7 +12421,7 @@
       <c r="G104" t="s">
         <v>587</v>
       </c>
-      <c r="H104" s="11"/>
+      <c r="H104" s="12"/>
       <c r="I104" t="s">
         <v>583</v>
       </c>
@@ -12476,7 +12476,7 @@
       <c r="Z104" t="s">
         <v>596</v>
       </c>
-      <c r="AA104" s="10"/>
+      <c r="AA104" s="11"/>
     </row>
     <row r="105" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
@@ -12500,7 +12500,7 @@
       <c r="G105" t="s">
         <v>587</v>
       </c>
-      <c r="H105" s="11"/>
+      <c r="H105" s="12"/>
       <c r="I105" t="s">
         <v>583</v>
       </c>
@@ -12555,7 +12555,7 @@
       <c r="Z105" t="s">
         <v>596</v>
       </c>
-      <c r="AA105" s="10"/>
+      <c r="AA105" s="11"/>
     </row>
     <row r="106" spans="1:27" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
@@ -12579,7 +12579,7 @@
       <c r="G106" t="s">
         <v>599</v>
       </c>
-      <c r="H106" s="11" t="s">
+      <c r="H106" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I106" t="s">
@@ -12636,7 +12636,7 @@
       <c r="Z106" t="s">
         <v>609</v>
       </c>
-      <c r="AA106" s="10" t="s">
+      <c r="AA106" s="11" t="s">
         <v>107</v>
       </c>
     </row>
@@ -12662,7 +12662,7 @@
       <c r="G107" t="s">
         <v>599</v>
       </c>
-      <c r="H107" s="11"/>
+      <c r="H107" s="12"/>
       <c r="I107" t="s">
         <v>600</v>
       </c>
@@ -12717,7 +12717,7 @@
       <c r="Z107" t="s">
         <v>609</v>
       </c>
-      <c r="AA107" s="10"/>
+      <c r="AA107" s="11"/>
     </row>
     <row r="108" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
@@ -12741,7 +12741,7 @@
       <c r="G108" t="s">
         <v>599</v>
       </c>
-      <c r="H108" s="11"/>
+      <c r="H108" s="12"/>
       <c r="I108" t="s">
         <v>600</v>
       </c>
@@ -12796,7 +12796,7 @@
       <c r="Z108" t="s">
         <v>609</v>
       </c>
-      <c r="AA108" s="10"/>
+      <c r="AA108" s="11"/>
     </row>
     <row r="109" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
@@ -12820,7 +12820,7 @@
       <c r="G109" t="s">
         <v>599</v>
       </c>
-      <c r="H109" s="11"/>
+      <c r="H109" s="12"/>
       <c r="I109" t="s">
         <v>600</v>
       </c>
@@ -12875,7 +12875,7 @@
       <c r="Z109" t="s">
         <v>609</v>
       </c>
-      <c r="AA109" s="10"/>
+      <c r="AA109" s="11"/>
     </row>
     <row r="110" spans="1:27" ht="129.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
@@ -12899,7 +12899,7 @@
       <c r="G110" t="s">
         <v>612</v>
       </c>
-      <c r="H110" s="11" t="s">
+      <c r="H110" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I110" t="s">
@@ -12956,7 +12956,7 @@
       <c r="Z110" t="s">
         <v>626</v>
       </c>
-      <c r="AA110" s="10" t="s">
+      <c r="AA110" s="11" t="s">
         <v>833</v>
       </c>
     </row>
@@ -12982,7 +12982,7 @@
       <c r="G111" t="s">
         <v>612</v>
       </c>
-      <c r="H111" s="11"/>
+      <c r="H111" s="12"/>
       <c r="I111" t="s">
         <v>617</v>
       </c>
@@ -13037,7 +13037,7 @@
       <c r="Z111" t="s">
         <v>626</v>
       </c>
-      <c r="AA111" s="10"/>
+      <c r="AA111" s="11"/>
     </row>
     <row r="112" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
@@ -13061,7 +13061,7 @@
       <c r="G112" t="s">
         <v>612</v>
       </c>
-      <c r="H112" s="11"/>
+      <c r="H112" s="12"/>
       <c r="I112" t="s">
         <v>617</v>
       </c>
@@ -13116,7 +13116,7 @@
       <c r="Z112" t="s">
         <v>626</v>
       </c>
-      <c r="AA112" s="10"/>
+      <c r="AA112" s="11"/>
     </row>
     <row r="113" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
@@ -13140,7 +13140,7 @@
       <c r="G113" t="s">
         <v>612</v>
       </c>
-      <c r="H113" s="11"/>
+      <c r="H113" s="12"/>
       <c r="I113" t="s">
         <v>617</v>
       </c>
@@ -13195,7 +13195,7 @@
       <c r="Z113" t="s">
         <v>626</v>
       </c>
-      <c r="AA113" s="10"/>
+      <c r="AA113" s="11"/>
     </row>
     <row r="114" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
@@ -13219,7 +13219,7 @@
       <c r="G114" t="s">
         <v>628</v>
       </c>
-      <c r="H114" s="11" t="s">
+      <c r="H114" s="12" t="s">
         <v>634</v>
       </c>
       <c r="I114" t="s">
@@ -13264,7 +13264,7 @@
       <c r="Z114" t="s">
         <v>644</v>
       </c>
-      <c r="AA114" s="10" t="s">
+      <c r="AA114" s="11" t="s">
         <v>645</v>
       </c>
     </row>
@@ -13290,7 +13290,7 @@
       <c r="G115" t="s">
         <v>628</v>
       </c>
-      <c r="H115" s="11"/>
+      <c r="H115" s="12"/>
       <c r="I115" t="s">
         <v>635</v>
       </c>
@@ -13333,7 +13333,7 @@
       <c r="Z115" t="s">
         <v>644</v>
       </c>
-      <c r="AA115" s="10"/>
+      <c r="AA115" s="11"/>
     </row>
     <row r="116" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
@@ -13357,7 +13357,7 @@
       <c r="G116" t="s">
         <v>628</v>
       </c>
-      <c r="H116" s="11"/>
+      <c r="H116" s="12"/>
       <c r="I116" t="s">
         <v>635</v>
       </c>
@@ -13400,7 +13400,7 @@
       <c r="Z116" t="s">
         <v>644</v>
       </c>
-      <c r="AA116" s="10"/>
+      <c r="AA116" s="11"/>
     </row>
     <row r="117" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
@@ -13424,7 +13424,7 @@
       <c r="G117" t="s">
         <v>628</v>
       </c>
-      <c r="H117" s="11"/>
+      <c r="H117" s="12"/>
       <c r="I117" t="s">
         <v>635</v>
       </c>
@@ -13467,7 +13467,7 @@
       <c r="Z117" t="s">
         <v>644</v>
       </c>
-      <c r="AA117" s="10"/>
+      <c r="AA117" s="11"/>
     </row>
     <row r="118" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
@@ -13491,7 +13491,7 @@
       <c r="G118" t="s">
         <v>648</v>
       </c>
-      <c r="H118" s="11" t="s">
+      <c r="H118" s="12" t="s">
         <v>656</v>
       </c>
       <c r="I118" t="s">
@@ -13536,7 +13536,7 @@
       <c r="Z118" t="s">
         <v>661</v>
       </c>
-      <c r="AA118" s="10" t="s">
+      <c r="AA118" s="11" t="s">
         <v>111</v>
       </c>
     </row>
@@ -13562,7 +13562,7 @@
       <c r="G119" t="s">
         <v>648</v>
       </c>
-      <c r="H119" s="11"/>
+      <c r="H119" s="12"/>
       <c r="I119" t="s">
         <v>654</v>
       </c>
@@ -13605,7 +13605,7 @@
       <c r="Z119" t="s">
         <v>661</v>
       </c>
-      <c r="AA119" s="10"/>
+      <c r="AA119" s="11"/>
     </row>
     <row r="120" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
@@ -13629,7 +13629,7 @@
       <c r="G120" t="s">
         <v>648</v>
       </c>
-      <c r="H120" s="11"/>
+      <c r="H120" s="12"/>
       <c r="I120" t="s">
         <v>654</v>
       </c>
@@ -13672,7 +13672,7 @@
       <c r="Z120" t="s">
         <v>661</v>
       </c>
-      <c r="AA120" s="10"/>
+      <c r="AA120" s="11"/>
     </row>
     <row r="121" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
@@ -13696,7 +13696,7 @@
       <c r="G121" t="s">
         <v>648</v>
       </c>
-      <c r="H121" s="11"/>
+      <c r="H121" s="12"/>
       <c r="I121" t="s">
         <v>654</v>
       </c>
@@ -13739,7 +13739,7 @@
       <c r="Z121" t="s">
         <v>661</v>
       </c>
-      <c r="AA121" s="10"/>
+      <c r="AA121" s="11"/>
     </row>
     <row r="122" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
@@ -13763,7 +13763,7 @@
       <c r="G122" t="s">
         <v>665</v>
       </c>
-      <c r="H122" s="11" t="s">
+      <c r="H122" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I122" t="s">
@@ -13808,7 +13808,7 @@
       <c r="Z122" t="s">
         <v>677</v>
       </c>
-      <c r="AA122" s="10" t="s">
+      <c r="AA122" s="11" t="s">
         <v>117</v>
       </c>
     </row>
@@ -13834,7 +13834,7 @@
       <c r="G123" t="s">
         <v>665</v>
       </c>
-      <c r="H123" s="11"/>
+      <c r="H123" s="12"/>
       <c r="I123" t="s">
         <v>664</v>
       </c>
@@ -13877,7 +13877,7 @@
       <c r="Z123" t="s">
         <v>677</v>
       </c>
-      <c r="AA123" s="10"/>
+      <c r="AA123" s="11"/>
     </row>
     <row r="124" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
@@ -13901,7 +13901,7 @@
       <c r="G124" t="s">
         <v>665</v>
       </c>
-      <c r="H124" s="11"/>
+      <c r="H124" s="12"/>
       <c r="I124" t="s">
         <v>664</v>
       </c>
@@ -13944,7 +13944,7 @@
       <c r="Z124" t="s">
         <v>677</v>
       </c>
-      <c r="AA124" s="10"/>
+      <c r="AA124" s="11"/>
     </row>
     <row r="125" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
@@ -13968,7 +13968,7 @@
       <c r="G125" t="s">
         <v>665</v>
       </c>
-      <c r="H125" s="11"/>
+      <c r="H125" s="12"/>
       <c r="I125" t="s">
         <v>664</v>
       </c>
@@ -14011,7 +14011,7 @@
       <c r="Z125" t="s">
         <v>677</v>
       </c>
-      <c r="AA125" s="10"/>
+      <c r="AA125" s="11"/>
     </row>
     <row r="126" spans="1:28" ht="158.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
@@ -14035,7 +14035,7 @@
       <c r="G126" t="s">
         <v>682</v>
       </c>
-      <c r="H126" s="11" t="s">
+      <c r="H126" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I126" t="s">
@@ -14092,10 +14092,10 @@
       <c r="Z126" t="s">
         <v>696</v>
       </c>
-      <c r="AA126" s="10" t="s">
+      <c r="AA126" s="11" t="s">
         <v>680</v>
       </c>
-      <c r="AB126" s="12" t="s">
+      <c r="AB126" s="13" t="s">
         <v>146</v>
       </c>
     </row>
@@ -14121,7 +14121,7 @@
       <c r="G127" t="s">
         <v>682</v>
       </c>
-      <c r="H127" s="11"/>
+      <c r="H127" s="12"/>
       <c r="I127" t="s">
         <v>687</v>
       </c>
@@ -14176,8 +14176,8 @@
       <c r="Z127" t="s">
         <v>696</v>
       </c>
-      <c r="AA127" s="10"/>
-      <c r="AB127" s="12"/>
+      <c r="AA127" s="11"/>
+      <c r="AB127" s="13"/>
     </row>
     <row r="128" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
@@ -14201,7 +14201,7 @@
       <c r="G128" t="s">
         <v>682</v>
       </c>
-      <c r="H128" s="11"/>
+      <c r="H128" s="12"/>
       <c r="I128" t="s">
         <v>687</v>
       </c>
@@ -14256,8 +14256,8 @@
       <c r="Z128" t="s">
         <v>696</v>
       </c>
-      <c r="AA128" s="10"/>
-      <c r="AB128" s="12"/>
+      <c r="AA128" s="11"/>
+      <c r="AB128" s="13"/>
     </row>
     <row r="129" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
@@ -14281,7 +14281,7 @@
       <c r="G129" t="s">
         <v>682</v>
       </c>
-      <c r="H129" s="11"/>
+      <c r="H129" s="12"/>
       <c r="I129" t="s">
         <v>687</v>
       </c>
@@ -14336,8 +14336,8 @@
       <c r="Z129" t="s">
         <v>696</v>
       </c>
-      <c r="AA129" s="10"/>
-      <c r="AB129" s="12"/>
+      <c r="AA129" s="11"/>
+      <c r="AB129" s="13"/>
     </row>
     <row r="130" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
@@ -14361,7 +14361,7 @@
       <c r="G130" t="s">
         <v>123</v>
       </c>
-      <c r="H130" s="11" t="s">
+      <c r="H130" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I130" t="s">
@@ -14418,10 +14418,10 @@
       <c r="Z130" t="s">
         <v>705</v>
       </c>
-      <c r="AA130" s="10" t="s">
+      <c r="AA130" s="11" t="s">
         <v>130</v>
       </c>
-      <c r="AB130" s="13" t="s">
+      <c r="AB130" s="10" t="s">
         <v>697</v>
       </c>
     </row>
@@ -14447,7 +14447,7 @@
       <c r="G131" t="s">
         <v>123</v>
       </c>
-      <c r="H131" s="11"/>
+      <c r="H131" s="12"/>
       <c r="I131" t="s">
         <v>128</v>
       </c>
@@ -14502,8 +14502,8 @@
       <c r="Z131" t="s">
         <v>705</v>
       </c>
-      <c r="AA131" s="10"/>
-      <c r="AB131" s="13"/>
+      <c r="AA131" s="11"/>
+      <c r="AB131" s="10"/>
     </row>
     <row r="132" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
@@ -14527,7 +14527,7 @@
       <c r="G132" t="s">
         <v>123</v>
       </c>
-      <c r="H132" s="11"/>
+      <c r="H132" s="12"/>
       <c r="I132" t="s">
         <v>128</v>
       </c>
@@ -14582,8 +14582,8 @@
       <c r="Z132" t="s">
         <v>705</v>
       </c>
-      <c r="AA132" s="10"/>
-      <c r="AB132" s="13"/>
+      <c r="AA132" s="11"/>
+      <c r="AB132" s="10"/>
     </row>
     <row r="133" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
@@ -14607,7 +14607,7 @@
       <c r="G133" t="s">
         <v>123</v>
       </c>
-      <c r="H133" s="11"/>
+      <c r="H133" s="12"/>
       <c r="I133" t="s">
         <v>128</v>
       </c>
@@ -14662,8 +14662,8 @@
       <c r="Z133" t="s">
         <v>705</v>
       </c>
-      <c r="AA133" s="10"/>
-      <c r="AB133" s="13"/>
+      <c r="AA133" s="11"/>
+      <c r="AB133" s="10"/>
     </row>
     <row r="134" spans="1:28" ht="144" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
@@ -14687,7 +14687,7 @@
       <c r="G134" t="s">
         <v>708</v>
       </c>
-      <c r="H134" s="11" t="s">
+      <c r="H134" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I134" t="s">
@@ -14744,7 +14744,7 @@
       <c r="Z134" t="s">
         <v>718</v>
       </c>
-      <c r="AA134" s="10" t="s">
+      <c r="AA134" s="11" t="s">
         <v>136</v>
       </c>
     </row>
@@ -14770,7 +14770,7 @@
       <c r="G135" t="s">
         <v>708</v>
       </c>
-      <c r="H135" s="11"/>
+      <c r="H135" s="12"/>
       <c r="I135" t="s">
         <v>710</v>
       </c>
@@ -14825,7 +14825,7 @@
       <c r="Z135" t="s">
         <v>718</v>
       </c>
-      <c r="AA135" s="10"/>
+      <c r="AA135" s="11"/>
     </row>
     <row r="136" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
@@ -14849,7 +14849,7 @@
       <c r="G136" t="s">
         <v>708</v>
       </c>
-      <c r="H136" s="11"/>
+      <c r="H136" s="12"/>
       <c r="I136" t="s">
         <v>710</v>
       </c>
@@ -14904,7 +14904,7 @@
       <c r="Z136" t="s">
         <v>718</v>
       </c>
-      <c r="AA136" s="10"/>
+      <c r="AA136" s="11"/>
     </row>
     <row r="137" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
@@ -14928,7 +14928,7 @@
       <c r="G137" t="s">
         <v>708</v>
       </c>
-      <c r="H137" s="11"/>
+      <c r="H137" s="12"/>
       <c r="I137" t="s">
         <v>710</v>
       </c>
@@ -14983,7 +14983,7 @@
       <c r="Z137" t="s">
         <v>718</v>
       </c>
-      <c r="AA137" s="10"/>
+      <c r="AA137" s="11"/>
     </row>
     <row r="138" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
@@ -15007,7 +15007,7 @@
       <c r="G138" t="s">
         <v>721</v>
       </c>
-      <c r="H138" s="11" t="s">
+      <c r="H138" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I138" t="s">
@@ -15052,7 +15052,7 @@
       <c r="Z138" t="s">
         <v>735</v>
       </c>
-      <c r="AA138" s="10" t="s">
+      <c r="AA138" s="11" t="s">
         <v>138</v>
       </c>
     </row>
@@ -15078,7 +15078,7 @@
       <c r="G139" t="s">
         <v>721</v>
       </c>
-      <c r="H139" s="11"/>
+      <c r="H139" s="12"/>
       <c r="I139" t="s">
         <v>727</v>
       </c>
@@ -15121,7 +15121,7 @@
       <c r="Z139" t="s">
         <v>735</v>
       </c>
-      <c r="AA139" s="10"/>
+      <c r="AA139" s="11"/>
     </row>
     <row r="140" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
@@ -15145,7 +15145,7 @@
       <c r="G140" t="s">
         <v>721</v>
       </c>
-      <c r="H140" s="11"/>
+      <c r="H140" s="12"/>
       <c r="I140" t="s">
         <v>727</v>
       </c>
@@ -15188,7 +15188,7 @@
       <c r="Z140" t="s">
         <v>735</v>
       </c>
-      <c r="AA140" s="10"/>
+      <c r="AA140" s="11"/>
     </row>
     <row r="141" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
@@ -15212,7 +15212,7 @@
       <c r="G141" t="s">
         <v>721</v>
       </c>
-      <c r="H141" s="11"/>
+      <c r="H141" s="12"/>
       <c r="I141" t="s">
         <v>727</v>
       </c>
@@ -15255,7 +15255,7 @@
       <c r="Z141" t="s">
         <v>735</v>
       </c>
-      <c r="AA141" s="10"/>
+      <c r="AA141" s="11"/>
     </row>
     <row r="142" spans="1:28" ht="86.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
@@ -15279,7 +15279,7 @@
       <c r="G142" t="s">
         <v>738</v>
       </c>
-      <c r="H142" s="11" t="s">
+      <c r="H142" s="12" t="s">
         <v>140</v>
       </c>
       <c r="I142" t="s">
@@ -15324,7 +15324,7 @@
       <c r="Z142" t="s">
         <v>752</v>
       </c>
-      <c r="AA142" s="10" t="s">
+      <c r="AA142" s="11" t="s">
         <v>141</v>
       </c>
     </row>
@@ -15350,7 +15350,7 @@
       <c r="G143" t="s">
         <v>738</v>
       </c>
-      <c r="H143" s="11"/>
+      <c r="H143" s="12"/>
       <c r="I143" t="s">
         <v>743</v>
       </c>
@@ -15393,7 +15393,7 @@
       <c r="Z143" t="s">
         <v>752</v>
       </c>
-      <c r="AA143" s="10"/>
+      <c r="AA143" s="11"/>
     </row>
     <row r="144" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
@@ -15417,7 +15417,7 @@
       <c r="G144" t="s">
         <v>738</v>
       </c>
-      <c r="H144" s="11"/>
+      <c r="H144" s="12"/>
       <c r="I144" t="s">
         <v>743</v>
       </c>
@@ -15460,7 +15460,7 @@
       <c r="Z144" t="s">
         <v>752</v>
       </c>
-      <c r="AA144" s="10"/>
+      <c r="AA144" s="11"/>
     </row>
     <row r="145" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
@@ -15484,7 +15484,7 @@
       <c r="G145" t="s">
         <v>738</v>
       </c>
-      <c r="H145" s="11"/>
+      <c r="H145" s="12"/>
       <c r="I145" t="s">
         <v>743</v>
       </c>
@@ -15527,7 +15527,7 @@
       <c r="Z145" t="s">
         <v>752</v>
       </c>
-      <c r="AA145" s="10"/>
+      <c r="AA145" s="11"/>
     </row>
     <row r="146" spans="1:28" ht="115.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
@@ -15551,7 +15551,7 @@
       <c r="G146" t="s">
         <v>763</v>
       </c>
-      <c r="H146" s="11" t="s">
+      <c r="H146" s="12" t="s">
         <v>764</v>
       </c>
       <c r="I146" t="s">
@@ -15596,10 +15596,10 @@
       <c r="Z146" t="s">
         <v>773</v>
       </c>
-      <c r="AA146" s="10" t="s">
+      <c r="AA146" s="11" t="s">
         <v>765</v>
       </c>
-      <c r="AB146" s="10" t="s">
+      <c r="AB146" s="11" t="s">
         <v>753</v>
       </c>
     </row>
@@ -15625,7 +15625,7 @@
       <c r="G147" t="s">
         <v>763</v>
       </c>
-      <c r="H147" s="11"/>
+      <c r="H147" s="12"/>
       <c r="I147" t="s">
         <v>761</v>
       </c>
@@ -15668,8 +15668,8 @@
       <c r="Z147" t="s">
         <v>773</v>
       </c>
-      <c r="AA147" s="10"/>
-      <c r="AB147" s="10"/>
+      <c r="AA147" s="11"/>
+      <c r="AB147" s="11"/>
     </row>
     <row r="148" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
@@ -15693,7 +15693,7 @@
       <c r="G148" t="s">
         <v>763</v>
       </c>
-      <c r="H148" s="11"/>
+      <c r="H148" s="12"/>
       <c r="I148" t="s">
         <v>761</v>
       </c>
@@ -15736,8 +15736,8 @@
       <c r="Z148" t="s">
         <v>773</v>
       </c>
-      <c r="AA148" s="10"/>
-      <c r="AB148" s="10"/>
+      <c r="AA148" s="11"/>
+      <c r="AB148" s="11"/>
     </row>
     <row r="149" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
@@ -15761,7 +15761,7 @@
       <c r="G149" t="s">
         <v>763</v>
       </c>
-      <c r="H149" s="11"/>
+      <c r="H149" s="12"/>
       <c r="I149" t="s">
         <v>761</v>
       </c>
@@ -15804,8 +15804,8 @@
       <c r="Z149" t="s">
         <v>773</v>
       </c>
-      <c r="AA149" s="10"/>
-      <c r="AB149" s="10"/>
+      <c r="AA149" s="11"/>
+      <c r="AB149" s="11"/>
     </row>
     <row r="150" spans="1:28" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
@@ -15829,7 +15829,7 @@
       <c r="G150" t="s">
         <v>776</v>
       </c>
-      <c r="H150" s="11" t="s">
+      <c r="H150" s="12" t="s">
         <v>89</v>
       </c>
       <c r="I150" t="s">
@@ -15886,7 +15886,7 @@
       <c r="Z150" t="s">
         <v>794</v>
       </c>
-      <c r="AA150" s="10" t="s">
+      <c r="AA150" s="11" t="s">
         <v>786</v>
       </c>
     </row>
@@ -15912,7 +15912,7 @@
       <c r="G151" t="s">
         <v>776</v>
       </c>
-      <c r="H151" s="11"/>
+      <c r="H151" s="12"/>
       <c r="I151" t="s">
         <v>781</v>
       </c>
@@ -15967,7 +15967,7 @@
       <c r="Z151" t="s">
         <v>794</v>
       </c>
-      <c r="AA151" s="10"/>
+      <c r="AA151" s="11"/>
     </row>
     <row r="152" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
@@ -15991,7 +15991,7 @@
       <c r="G152" t="s">
         <v>776</v>
       </c>
-      <c r="H152" s="11"/>
+      <c r="H152" s="12"/>
       <c r="I152" t="s">
         <v>781</v>
       </c>
@@ -16046,7 +16046,7 @@
       <c r="Z152" t="s">
         <v>794</v>
       </c>
-      <c r="AA152" s="10"/>
+      <c r="AA152" s="11"/>
     </row>
     <row r="153" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
@@ -16070,7 +16070,7 @@
       <c r="G153" t="s">
         <v>776</v>
       </c>
-      <c r="H153" s="11"/>
+      <c r="H153" s="12"/>
       <c r="I153" t="s">
         <v>781</v>
       </c>
@@ -16125,7 +16125,7 @@
       <c r="Z153" t="s">
         <v>794</v>
       </c>
-      <c r="AA153" s="10"/>
+      <c r="AA153" s="11"/>
     </row>
     <row r="154" spans="1:28" ht="187.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
@@ -16149,7 +16149,7 @@
       <c r="G154" t="s">
         <v>803</v>
       </c>
-      <c r="H154" s="11" t="s">
+      <c r="H154" s="12" t="s">
         <v>804</v>
       </c>
       <c r="I154" t="s">
@@ -16206,7 +16206,7 @@
       <c r="Z154" t="s">
         <v>813</v>
       </c>
-      <c r="AA154" s="10" t="s">
+      <c r="AA154" s="11" t="s">
         <v>814</v>
       </c>
     </row>
@@ -16232,7 +16232,7 @@
       <c r="G155" t="s">
         <v>803</v>
       </c>
-      <c r="H155" s="11"/>
+      <c r="H155" s="12"/>
       <c r="I155" t="s">
         <v>805</v>
       </c>
@@ -16287,7 +16287,7 @@
       <c r="Z155" t="s">
         <v>813</v>
       </c>
-      <c r="AA155" s="10"/>
+      <c r="AA155" s="11"/>
     </row>
     <row r="156" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
@@ -16311,7 +16311,7 @@
       <c r="G156" t="s">
         <v>803</v>
       </c>
-      <c r="H156" s="11"/>
+      <c r="H156" s="12"/>
       <c r="I156" t="s">
         <v>805</v>
       </c>
@@ -16366,7 +16366,7 @@
       <c r="Z156" t="s">
         <v>813</v>
       </c>
-      <c r="AA156" s="10"/>
+      <c r="AA156" s="11"/>
     </row>
     <row r="157" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
@@ -16390,7 +16390,7 @@
       <c r="G157" t="s">
         <v>803</v>
       </c>
-      <c r="H157" s="11"/>
+      <c r="H157" s="12"/>
       <c r="I157" t="s">
         <v>805</v>
       </c>
@@ -16445,7 +16445,7 @@
       <c r="Z157" t="s">
         <v>813</v>
       </c>
-      <c r="AA157" s="10"/>
+      <c r="AA157" s="11"/>
     </row>
     <row r="158" spans="1:28" ht="187.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
@@ -16469,7 +16469,7 @@
       <c r="G158" t="s">
         <v>818</v>
       </c>
-      <c r="H158" s="11" t="s">
+      <c r="H158" s="12" t="s">
         <v>825</v>
       </c>
       <c r="I158" t="s">
@@ -16526,7 +16526,7 @@
       <c r="Z158" t="s">
         <v>813</v>
       </c>
-      <c r="AA158" s="10" t="s">
+      <c r="AA158" s="11" t="s">
         <v>832</v>
       </c>
     </row>
@@ -16552,7 +16552,7 @@
       <c r="G159" t="s">
         <v>818</v>
       </c>
-      <c r="H159" s="11"/>
+      <c r="H159" s="12"/>
       <c r="I159" t="s">
         <v>824</v>
       </c>
@@ -16607,7 +16607,7 @@
       <c r="Z159" t="s">
         <v>813</v>
       </c>
-      <c r="AA159" s="10"/>
+      <c r="AA159" s="11"/>
     </row>
     <row r="160" spans="1:28" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
@@ -16631,7 +16631,7 @@
       <c r="G160" t="s">
         <v>818</v>
       </c>
-      <c r="H160" s="11"/>
+      <c r="H160" s="12"/>
       <c r="I160" t="s">
         <v>824</v>
       </c>
@@ -16686,7 +16686,7 @@
       <c r="Z160" t="s">
         <v>813</v>
       </c>
-      <c r="AA160" s="10"/>
+      <c r="AA160" s="11"/>
     </row>
     <row r="161" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
@@ -16710,7 +16710,7 @@
       <c r="G161" t="s">
         <v>818</v>
       </c>
-      <c r="H161" s="11"/>
+      <c r="H161" s="12"/>
       <c r="I161" t="s">
         <v>824</v>
       </c>
@@ -16765,10 +16765,86 @@
       <c r="Z161" t="s">
         <v>813</v>
       </c>
-      <c r="AA161" s="10"/>
+      <c r="AA161" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="92">
+    <mergeCell ref="AB6:AB9"/>
+    <mergeCell ref="AB10:AB13"/>
+    <mergeCell ref="H126:H129"/>
+    <mergeCell ref="AA126:AA129"/>
+    <mergeCell ref="AB126:AB129"/>
+    <mergeCell ref="H86:H89"/>
+    <mergeCell ref="AA86:AA89"/>
+    <mergeCell ref="H102:H105"/>
+    <mergeCell ref="AA102:AA105"/>
+    <mergeCell ref="H122:H125"/>
+    <mergeCell ref="AA122:AA125"/>
+    <mergeCell ref="AA98:AA101"/>
+    <mergeCell ref="H62:H65"/>
+    <mergeCell ref="AA62:AA65"/>
+    <mergeCell ref="H66:H69"/>
+    <mergeCell ref="AA66:AA69"/>
+    <mergeCell ref="H82:H85"/>
+    <mergeCell ref="AA82:AA85"/>
+    <mergeCell ref="H70:H73"/>
+    <mergeCell ref="AA70:AA73"/>
+    <mergeCell ref="H74:H77"/>
+    <mergeCell ref="AA74:AA77"/>
+    <mergeCell ref="H78:H81"/>
+    <mergeCell ref="AA78:AA81"/>
+    <mergeCell ref="H50:H53"/>
+    <mergeCell ref="AA50:AA53"/>
+    <mergeCell ref="H54:H57"/>
+    <mergeCell ref="AA54:AA57"/>
+    <mergeCell ref="H58:H61"/>
+    <mergeCell ref="AA58:AA61"/>
+    <mergeCell ref="H2:H5"/>
+    <mergeCell ref="AA2:AA5"/>
+    <mergeCell ref="H6:H9"/>
+    <mergeCell ref="AA6:AA9"/>
+    <mergeCell ref="H10:H13"/>
+    <mergeCell ref="AA10:AA13"/>
+    <mergeCell ref="AA94:AA97"/>
+    <mergeCell ref="H98:H101"/>
+    <mergeCell ref="H14:H17"/>
+    <mergeCell ref="L14:L17"/>
+    <mergeCell ref="AA14:AA17"/>
+    <mergeCell ref="H18:H21"/>
+    <mergeCell ref="AA18:AA21"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="AA30:AA33"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="AA34:AA37"/>
+    <mergeCell ref="H38:H41"/>
+    <mergeCell ref="AA38:AA41"/>
+    <mergeCell ref="H42:H45"/>
+    <mergeCell ref="AA42:AA45"/>
+    <mergeCell ref="H46:H49"/>
+    <mergeCell ref="H138:H141"/>
+    <mergeCell ref="AA138:AA141"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="AA22:AA25"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="H118:H121"/>
+    <mergeCell ref="AA118:AA121"/>
+    <mergeCell ref="H90:H93"/>
+    <mergeCell ref="AA90:AA93"/>
+    <mergeCell ref="H106:H109"/>
+    <mergeCell ref="AA106:AA109"/>
+    <mergeCell ref="H110:H113"/>
+    <mergeCell ref="AA110:AA113"/>
+    <mergeCell ref="H114:H117"/>
+    <mergeCell ref="AA114:AA117"/>
+    <mergeCell ref="H94:H97"/>
+    <mergeCell ref="L90:L93"/>
+    <mergeCell ref="AB18:AB21"/>
+    <mergeCell ref="AB26:AB29"/>
+    <mergeCell ref="AB30:AB33"/>
+    <mergeCell ref="AB54:AB57"/>
+    <mergeCell ref="AB62:AB65"/>
+    <mergeCell ref="AA26:AA29"/>
+    <mergeCell ref="AA46:AA49"/>
     <mergeCell ref="AB130:AB133"/>
     <mergeCell ref="AB146:AB149"/>
     <mergeCell ref="H154:H157"/>
@@ -16785,82 +16861,6 @@
     <mergeCell ref="AA130:AA133"/>
     <mergeCell ref="H134:H137"/>
     <mergeCell ref="AA134:AA137"/>
-    <mergeCell ref="L90:L93"/>
-    <mergeCell ref="AB18:AB21"/>
-    <mergeCell ref="AB26:AB29"/>
-    <mergeCell ref="AB30:AB33"/>
-    <mergeCell ref="AB54:AB57"/>
-    <mergeCell ref="AB62:AB65"/>
-    <mergeCell ref="AA26:AA29"/>
-    <mergeCell ref="AA46:AA49"/>
-    <mergeCell ref="H138:H141"/>
-    <mergeCell ref="AA138:AA141"/>
-    <mergeCell ref="H22:H25"/>
-    <mergeCell ref="AA22:AA25"/>
-    <mergeCell ref="H26:H29"/>
-    <mergeCell ref="H118:H121"/>
-    <mergeCell ref="AA118:AA121"/>
-    <mergeCell ref="H90:H93"/>
-    <mergeCell ref="AA90:AA93"/>
-    <mergeCell ref="H106:H109"/>
-    <mergeCell ref="AA106:AA109"/>
-    <mergeCell ref="H110:H113"/>
-    <mergeCell ref="AA110:AA113"/>
-    <mergeCell ref="H114:H117"/>
-    <mergeCell ref="AA114:AA117"/>
-    <mergeCell ref="H94:H97"/>
-    <mergeCell ref="AA94:AA97"/>
-    <mergeCell ref="H98:H101"/>
-    <mergeCell ref="H14:H17"/>
-    <mergeCell ref="L14:L17"/>
-    <mergeCell ref="AA14:AA17"/>
-    <mergeCell ref="H18:H21"/>
-    <mergeCell ref="AA18:AA21"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="AA30:AA33"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="AA34:AA37"/>
-    <mergeCell ref="H38:H41"/>
-    <mergeCell ref="AA38:AA41"/>
-    <mergeCell ref="H42:H45"/>
-    <mergeCell ref="AA42:AA45"/>
-    <mergeCell ref="H46:H49"/>
-    <mergeCell ref="H2:H5"/>
-    <mergeCell ref="AA2:AA5"/>
-    <mergeCell ref="H6:H9"/>
-    <mergeCell ref="AA6:AA9"/>
-    <mergeCell ref="H10:H13"/>
-    <mergeCell ref="AA10:AA13"/>
-    <mergeCell ref="H50:H53"/>
-    <mergeCell ref="AA50:AA53"/>
-    <mergeCell ref="H54:H57"/>
-    <mergeCell ref="AA54:AA57"/>
-    <mergeCell ref="H58:H61"/>
-    <mergeCell ref="AA58:AA61"/>
-    <mergeCell ref="H82:H85"/>
-    <mergeCell ref="AA82:AA85"/>
-    <mergeCell ref="H70:H73"/>
-    <mergeCell ref="AA70:AA73"/>
-    <mergeCell ref="H74:H77"/>
-    <mergeCell ref="AA74:AA77"/>
-    <mergeCell ref="H78:H81"/>
-    <mergeCell ref="AA78:AA81"/>
-    <mergeCell ref="AB6:AB9"/>
-    <mergeCell ref="AB10:AB13"/>
-    <mergeCell ref="H126:H129"/>
-    <mergeCell ref="AA126:AA129"/>
-    <mergeCell ref="AB126:AB129"/>
-    <mergeCell ref="H86:H89"/>
-    <mergeCell ref="AA86:AA89"/>
-    <mergeCell ref="H102:H105"/>
-    <mergeCell ref="AA102:AA105"/>
-    <mergeCell ref="H122:H125"/>
-    <mergeCell ref="AA122:AA125"/>
-    <mergeCell ref="AA98:AA101"/>
-    <mergeCell ref="H62:H65"/>
-    <mergeCell ref="AA62:AA65"/>
-    <mergeCell ref="H66:H69"/>
-    <mergeCell ref="AA66:AA69"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>